<commit_message>
Update dashboard through September 7
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2406,7 +2406,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Full-text screening ready to start</t>
+          <t>Full-text project opened; reviewer interaction issue under review</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Abstract screening complete; combined 144-record project ready</t>
+          <t>Abstract screening complete; combined 144-record full-text project opened</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2491,7 +2491,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Translated PDF uploaded; AI workflow tested and issue resolved</t>
+          <t>Kate cannot interact with the new project; Amin asked her to verify whether the issue has been resolved</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Begin both full-text screening arms and record time</t>
+          <t>Resolve Kate’s project-interaction issue and confirm both screening arms can begin</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2542,7 +2542,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Setup validated; screening not yet confirmed started</t>
+          <t>Screening start remains unconfirmed pending Kate’s access check</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Needs Action</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3060,12 +3060,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Needs Action</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Combined project ready; translated PDF uploaded and AI workflow issue resolved</t>
+          <t>Combined project opened; Kate’s ability to interact with it remains unconfirmed</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -4790,14 +4790,14 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Complete / Under Review</t>
         </is>
       </c>
       <c r="J78" s="18" t="n"/>
       <c r="K78" s="18" t="n"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>Combined 144-record project configured and ready</t>
+          <t>Combined project configured; reviewer permissions/interactivity under review</t>
         </is>
       </c>
       <c r="M78" s="18" t="inlineStr">
@@ -4847,14 +4847,14 @@
       </c>
       <c r="I79" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J79" s="18" t="n"/>
       <c r="K79" s="18" t="n"/>
       <c r="L79" s="18" t="inlineStr">
         <is>
-          <t>AI decision workflow tested successfully</t>
+          <t>Decision workflow tested; reviewer interaction still requires confirmation</t>
         </is>
       </c>
       <c r="M79" s="18" t="inlineStr">
@@ -4961,14 +4961,14 @@
       </c>
       <c r="I81" s="18" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="J81" s="18" t="n"/>
       <c r="K81" s="18" t="n"/>
       <c r="L81" s="18" t="inlineStr">
         <is>
-          <t>Laser AI team cleared to begin full-text screening</t>
+          <t>Laser AI screening blocked until Kate confirms that she can interact with the project</t>
         </is>
       </c>
       <c r="M81" s="18" t="inlineStr">
@@ -6654,7 +6654,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Needs Action</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -6674,7 +6674,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Confirm logins and reviewer access before setup.</t>
+          <t>Kate can open the new project but cannot interact with it; Meghan to check the configuration</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -6684,7 +6684,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -23234,15 +23234,56 @@
       </c>
     </row>
     <row r="35" ht="24" customHeight="1" s="29">
-      <c r="A35" s="17" t="n"/>
-      <c r="B35" s="17" t="n"/>
-      <c r="C35" s="17" t="n"/>
-      <c r="D35" s="17" t="n"/>
-      <c r="E35" s="17" t="n"/>
-      <c r="F35" s="17" t="n"/>
-      <c r="G35" s="17" t="n"/>
-      <c r="H35" s="17" t="n"/>
-      <c r="I35" s="17" t="n"/>
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>new-24</t>
+        </is>
+      </c>
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>Álvaro Limones — Cochrane review update CD002283</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="inlineStr">
+        <is>
+          <t>Under Shortlisting</t>
+        </is>
+      </c>
+      <c r="D35" s="17" t="inlineStr">
+        <is>
+          <t>Interest received; review update is about to start and timeline/readiness details were requested</t>
+        </is>
+      </c>
+      <c r="E35" s="17" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F35" s="17" t="inlineStr">
+        <is>
+          <t>Álvaro Limones</t>
+        </is>
+      </c>
+      <c r="G35" s="17" t="inlineStr">
+        <is>
+          <t>Awaiting review stage, search date, reference count and screening/extraction timeline</t>
+        </is>
+      </c>
+      <c r="H35" s="17" t="inlineStr">
+        <is>
+          <t>Inclusion depends on alignment with the study timeline and parallel-workflow readiness</t>
+        </is>
+      </c>
+      <c r="I35" s="17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="24" customHeight="1" s="29">
       <c r="A36" s="17" t="n"/>
@@ -32405,7 +32446,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abstract screening underway; expected completion this week; full-text screening planned next week</t>
+          <t>Abstract-screening completion not yet confirmed; full-text setup pending</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -32473,7 +32514,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Murali and Michelle are screening abstracts; completion expected this week</t>
+          <t>Murali and Michelle began screening; completion confirmation is now overdue</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -32507,7 +32548,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete abstract screening, notify the project team, circulate the survey and set up full-text screening</t>
+          <t>Follow up with Murali; after confirmation, circulate the survey and prepare full-text screening</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -32524,7 +32565,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-09-06 (expected)</t>
+          <t>Immediate follow-up</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -32541,7 +32582,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Abstract screening underway; full-text setup planned next</t>
+          <t>Completion confirmation pending; full-text setup cannot proceed yet</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -32597,7 +32638,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -33024,7 +33065,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Murali and Michelle are screening; completion expected this week</t>
+          <t>Abstract-screening completion has not yet been confirmed</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -33046,7 +33087,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Full-text screening planned for next week after the survey and project setup</t>
+          <t>Full-text setup pending abstract-screening confirmation and survey circulation</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -36743,7 +36784,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Needs Action</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -36753,7 +36794,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -36763,7 +36804,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Screening underway; circulate the survey and prepare full-text setup after completion</t>
+          <t>Follow up for completion confirmation, then circulate the survey and prepare full-text setup</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -37046,17 +37087,17 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Needs Action</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Screening underway; notify Krishna after completion so the survey and full-text setup can proceed</t>
+          <t>Completion confirmation is overdue; follow up before circulating the survey and starting full-text setup</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -42133,7 +42174,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Adjudication dataset ready; panel meeting scheduled</t>
+          <t>Adjudication Pilot 2 underway; extension inputs shared</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -42153,17 +42194,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Reference standard confirmed; randomized adjudication dataset prepared; panel invitation sent</t>
+          <t>Pilot 2 underway; 19-record BP mapping and PDF folder shared with Paweł</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Hold the scheduled panel meeting and begin adjudication; resolve CESAR extension PDF/mapping gap</t>
+          <t>Complete Pilot 2, verify Bi 2025 supporting-file coverage and obtain Paweł’s access confirmation</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
         <is>
-          <t>Scheduled — see calendar invitation</t>
+          <t>Pilot 2 underway; completion TBD</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -42205,7 +42246,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Corrective full-text cross-screening setup underway</t>
+          <t>Corrective NK citations uploaded; full-text files received; validation pending</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -42225,12 +42266,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>The 139-record RIS/PDF package was sent to the conventional team; the existing NK project was selected for the 25 AI records</t>
+          <t>Twenty-five citations—24 unique—were uploaded to the existing NK project; corresponding full texts were received</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Add 25 records to the existing NK project, complete both corrective screening arms and rerun the comparison</t>
+          <t>Upload and validate the corrective PDFs, complete both screening arms and rerun the comparison</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -42277,7 +42318,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Full-text screening cleared to begin</t>
+          <t>Full-text project opened; reviewer interaction issue under review</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -42297,12 +42338,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Combined 144-record project ready; translated PDF uploaded and AI workflow issue resolved</t>
+          <t>Combined project opened, but Kate cannot currently interact with it</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Begin both full-text screening arms and record time</t>
+          <t>Resolve Kate’s project-interaction issue and confirm that both screening arms can begin</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -42312,7 +42353,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Needs Action</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -42632,7 +42673,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Abstract screening underway; expected completion this week; full-text screening planned next week</t>
+          <t>Abstract-screening completion not yet confirmed; full-text setup pending</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -42652,17 +42693,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Murali and Michelle have started abstract screening; completion expected this week</t>
+          <t>No completion update received by the 6 September target</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Complete abstract screening, circulate the short survey and set up full-text screening</t>
+          <t>Follow up with Murali; after confirmation, circulate the survey and set up full-text screening</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-09-06 (expected)</t>
+          <t>Immediate follow-up</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -46363,7 +46404,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>All five groups consented; model/data-governance work continues; the BP automated run awaits the complete PDF package, mapping and supplementary-material decision</t>
+          <t>All five extension groups consented; BP mapping and PDF folder shared; adjudication Pilot 2 underway; Bi 2025 supporting-file check pending</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -46417,7 +46458,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Final report/project closeout</t>
+          <t>Final results, communications and project closeout</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -46628,7 +46669,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Laser AI operational; Fruit &amp; Veg full-text workflow validated and ready to screen</t>
+          <t>Laser AI operational; Fruit &amp; Veg full-text project opened, but reviewer interaction remains under review</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -56440,7 +56481,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Adjudication dataset ready; panel meeting scheduled</t>
+          <t>Adjudication Pilot 2 underway; extension inputs shared</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -56508,7 +56549,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Reference standard confirmed; randomized adjudication dataset prepared; panel invitation sent</t>
+          <t>Pilot 2 underway; all 19 BP records mapped and shared with Paweł</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56525,7 +56566,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Panel invitation sent; no advance pilot is required</t>
+          <t>Mapping covers all 19 records: 17 PDFs and two ClinicalTrials.gov registry records</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56542,7 +56583,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Hold the panel meeting and begin adjudication; complete the CESAR extension PDF/mapping package</t>
+          <t>Complete Pilot 2, confirm Bi 2025 supporting-file coverage and obtain Paweł’s access confirmation</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56559,7 +56600,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Scheduled — see calendar invitation</t>
+          <t>Pilot 2 underway; completion TBD</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -56576,7 +56617,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Panel meeting scheduled; CESAR extension input gap remains</t>
+          <t>Pilot 2 underway; Bi 2025 supplementary-file coverage requires confirmation</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -56632,7 +56673,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56879,7 +56920,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Only 4 of 19 full-text PDFs are visible to the extension team; complete mapping and supplementary-material scope are pending</t>
+          <t>Mapping shared for all 19 records; 17 PDFs are available and two registry-only records link to ClinicalTrials.gov</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -57133,12 +57174,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Extraction complete; adjudication ready; CESAR extension inputs incomplete</t>
+          <t>Extraction complete; Pilot 2 underway; Bi 2025 source-file check pending</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Adjudication meeting scheduled; extension screening awaits the complete PDF/mapping package</t>
+          <t>Pilot 2 started; extension mapping shared; Bi 2025 supporting-file verification pending</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -60194,14 +60235,14 @@
       </c>
       <c r="I104" s="18" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J104" s="18" t="n"/>
       <c r="K104" s="18" t="n"/>
       <c r="L104" s="18" t="inlineStr">
         <is>
-          <t>Meeting invitation sent; no advance pilot required</t>
+          <t>Pilot 2 launched; panel received the adjudication files and protocol</t>
         </is>
       </c>
       <c r="M104" s="18" t="inlineStr">
@@ -60304,14 +60345,14 @@
       </c>
       <c r="I106" s="18" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Waiting on Others</t>
         </is>
       </c>
       <c r="J106" s="18" t="n"/>
       <c r="K106" s="18" t="n"/>
       <c r="L106" s="18" t="inlineStr">
         <is>
-          <t>Automated run blocked pending all 19 PDFs, record-to-PDF mapping and a supplementary-material decision</t>
+          <t>Nineteen-record mapping and PDF folder sent to Paweł; awaiting access and run confirmation</t>
         </is>
       </c>
       <c r="M106" s="18" t="inlineStr">
@@ -60414,12 +60455,16 @@
       </c>
       <c r="I108" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J108" s="18" t="n"/>
       <c r="K108" s="18" t="n"/>
-      <c r="L108" s="18" t="n"/>
+      <c r="L108" s="18" t="inlineStr">
+        <is>
+          <t>Adjudication Pilot 2 underway</t>
+        </is>
+      </c>
       <c r="M108" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -61870,7 +61915,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Corrective full-text cross-screening setup underway</t>
+          <t>Corrective NK citations uploaded; PDFs received; validation pending</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -61938,7 +61983,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Corrective screening preparation underway; the conventional package was sent and the existing NK project selected</t>
+          <t>Existing NK project populated with 24 unique corrective citations; full texts received</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -61955,7 +62000,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>The 139-record RIS/PDF package was sent; addition of 25 records to the existing NK project is pending</t>
+          <t>Meghan uploaded 25 citations—24 unique—and Sivem supplied the corresponding full texts</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -61972,7 +62017,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Add 25 records to the existing NK project and complete both corrective screening arms</t>
+          <t>Upload and validate the corrective PDFs, then complete both screening arms</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -62006,7 +62051,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Analysis paused pending corrective cross-screening</t>
+          <t>Analysis paused pending PDF validation and corrective cross-screening</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -62062,7 +62107,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -62309,7 +62354,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Corrective-screening PDFs for 139 records are available in the shared folder; ten extracted-study PDFs were shared with Sean</t>
+          <t>Conventional corrective PDFs are available; Sivem supplied files for the NK corrective set and identified #10631/#10608 as duplicates</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -62547,7 +62592,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>The 139-record package was sent to the conventional team; the 25-record NK setup remains pending</t>
+          <t>The conventional package was sent; 24 unique citations are in NK and their full texts have been received</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -64260,7 +64305,7 @@
       <c r="K78" s="18" t="n"/>
       <c r="L78" s="18" t="inlineStr">
         <is>
-          <t>Sean selected the existing NK project; Meghan to add the 25 records</t>
+          <t>Twenty-five citations uploaded to the existing project—24 unique after deduplication</t>
         </is>
       </c>
       <c r="M78" s="18" t="inlineStr">
@@ -64317,7 +64362,7 @@
       <c r="K79" s="18" t="n"/>
       <c r="L79" s="18" t="inlineStr">
         <is>
-          <t>Validate the existing project after the 25 records are added</t>
+          <t>Upload the supplied PDFs and validate the 24-unique-record setup</t>
         </is>
       </c>
       <c r="M79" s="18" t="inlineStr">
@@ -64431,7 +64476,7 @@
       <c r="K81" s="18" t="n"/>
       <c r="L81" s="18" t="inlineStr">
         <is>
-          <t>Add 25 records to the existing NK project and complete AI-assisted screening</t>
+          <t>Complete AI-assisted screening of the 24 unique records after PDF upload and validation</t>
         </is>
       </c>
       <c r="M81" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Update dashboard through September 10
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2406,7 +2406,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Full-text project opened; reviewer interaction issue under review</t>
+          <t>Full-text pool reopened to 138 records; reviewer confirmation pending</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2491,7 +2491,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Kate cannot interact with the new project; Amin asked her to verify whether the issue has been resolved</t>
+          <t>Amin returned 138 records to the open pool; Kate can now attempt self-distribution</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Resolve Kate’s project-interaction issue and confirm both screening arms can begin</t>
+          <t>Confirm Kate can claim records and that both screening arms have started</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2542,7 +2542,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Screening start remains unconfirmed pending Kate’s access check</t>
+          <t>Pool reopened; screening start remains unconfirmed pending Kate’s response</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Needs Action</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3060,12 +3060,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Needs Action</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Combined project opened; Kate’s ability to interact with it remains unconfirmed</t>
+          <t>Amin reopened 138 records in the pool; Kate’s self-distribution confirmation is pending</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -4350,12 +4350,16 @@
       </c>
       <c r="I70" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J70" s="18" t="n"/>
       <c r="K70" s="18" t="n"/>
-      <c r="L70" s="18" t="n"/>
+      <c r="L70" s="18" t="inlineStr">
+        <is>
+          <t>One abstract-screening survey response received and confirmed</t>
+        </is>
+      </c>
       <c r="M70" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4403,12 +4407,16 @@
       </c>
       <c r="I71" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J71" s="18" t="n"/>
       <c r="K71" s="18" t="n"/>
-      <c r="L71" s="18" t="n"/>
+      <c r="L71" s="18" t="inlineStr">
+        <is>
+          <t>One abstract-screening survey response received and confirmed</t>
+        </is>
+      </c>
       <c r="M71" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4790,14 +4798,14 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Complete / Under Review</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J78" s="18" t="n"/>
       <c r="K78" s="18" t="n"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>Combined project configured; reviewer permissions/interactivity under review</t>
+          <t>Amin opened 138 records in the reviewer pool</t>
         </is>
       </c>
       <c r="M78" s="18" t="inlineStr">
@@ -4854,7 +4862,7 @@
       <c r="K79" s="18" t="n"/>
       <c r="L79" s="18" t="inlineStr">
         <is>
-          <t>Decision workflow tested; reviewer interaction still requires confirmation</t>
+          <t>Pool reopened; awaiting Kate’s claim/distribution confirmation</t>
         </is>
       </c>
       <c r="M79" s="18" t="inlineStr">
@@ -4961,14 +4969,14 @@
       </c>
       <c r="I81" s="18" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="J81" s="18" t="n"/>
       <c r="K81" s="18" t="n"/>
       <c r="L81" s="18" t="inlineStr">
         <is>
-          <t>Laser AI screening blocked until Kate confirms that she can interact with the project</t>
+          <t>The 138 records are open for Kate to claim; screening commencement remains unconfirmed</t>
         </is>
       </c>
       <c r="M81" s="18" t="inlineStr">
@@ -6654,7 +6662,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Needs Action</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -6674,7 +6682,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Kate can open the new project but cannot interact with it; Meghan to check the configuration</t>
+          <t>Amin reopened 138 records; Kate to confirm that she can claim and screen them</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -6684,7 +6692,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -22887,7 +22895,7 @@
       </c>
       <c r="D28" s="17" t="inlineStr">
         <is>
-          <t>Converted to phase1-06; conventional screening complete, Nested Knowledge screening underway and full text deliberately paused</t>
+          <t>Converted to phase1-06; both abstract-screening workflows complete and full-text screening reported underway</t>
         </is>
       </c>
       <c r="E28" s="17" t="inlineStr">
@@ -22902,12 +22910,12 @@
       </c>
       <c r="G28" s="17" t="inlineStr">
         <is>
-          <t>Full text paused until Nested Knowledge abstract screening complete</t>
+          <t>Full-text completion expected within 1–2 weeks</t>
         </is>
       </c>
       <c r="H28" s="17" t="inlineStr">
         <is>
-          <t>Converted to phase1-06 Probiotics; Nested Knowledge allocated</t>
+          <t>Both abstract arms complete; full-text screening underway; setup/consolidation confirmation pending</t>
         </is>
       </c>
       <c r="I28" s="17" t="inlineStr">
@@ -27689,7 +27697,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Conventional screening complete; NK screening underway</t>
+          <t>Both abstract-screening workflows complete; full-text screening reported underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -27757,7 +27765,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Calibration and conventional screening complete; NK screening continuing</t>
+          <t>Covidence and NK abstract screening complete; both teams progressing through full-text screening</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -27774,7 +27782,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Calibration and conventional screening complete; NK screening continuing</t>
+          <t>Covidence and NK abstract screening complete; both teams progressing through full-text screening</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -27791,7 +27799,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete NK screening/time capture, then begin full text</t>
+          <t>Confirm full-text setup and consolidation; complete screening and record time</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -27808,7 +27816,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Next 1–2 weeks</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -27825,7 +27833,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Conventional workflow ahead; full text awaits both workflows</t>
+          <t>Full-text screening reported underway; study-side confirmation pending</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -27881,7 +27889,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -27980,7 +27988,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Conventional complete; NK in progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -27997,7 +28005,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>On hold until Nested Knowledge abstract screening is complete</t>
+          <t>In Progress; setup confirmation pending</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -28301,9 +28309,17 @@
           <t>100</t>
         </is>
       </c>
+      <c r="C43" t="n">
+        <v>100</v>
+      </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Conventional complete; NK in progress</t>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Both title/abstract screening workflows complete</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -28320,12 +28336,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Not Started—sequencing dependency</t>
+          <t>In Progress / Under Review</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Team confirmed that Covidence full-text screening will remain paused</t>
+          <t>Jeremy reported both teams progressing through full text; confirmation requested from Sean and Meghan</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -29213,12 +29229,16 @@
       </c>
       <c r="I63" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J63" s="18" t="n"/>
       <c r="K63" s="18" t="n"/>
-      <c r="L63" s="18" t="n"/>
+      <c r="L63" s="18" t="inlineStr">
+        <is>
+          <t>NK abstract-screening setup and validation completed</t>
+        </is>
+      </c>
       <c r="M63" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -29266,12 +29286,16 @@
       </c>
       <c r="I64" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J64" s="18" t="n"/>
       <c r="K64" s="18" t="n"/>
-      <c r="L64" s="18" t="n"/>
+      <c r="L64" s="18" t="inlineStr">
+        <is>
+          <t>NK abstract-screening setup and validation completed</t>
+        </is>
+      </c>
       <c r="M64" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -29372,12 +29396,16 @@
       </c>
       <c r="I66" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J66" s="18" t="n"/>
       <c r="K66" s="18" t="n"/>
-      <c r="L66" s="18" t="n"/>
+      <c r="L66" s="18" t="inlineStr">
+        <is>
+          <t>Nested Knowledge title/abstract screening complete</t>
+        </is>
+      </c>
       <c r="M66" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -29425,12 +29453,16 @@
       </c>
       <c r="I67" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J67" s="18" t="n"/>
       <c r="K67" s="18" t="n"/>
-      <c r="L67" s="18" t="n"/>
+      <c r="L67" s="18" t="inlineStr">
+        <is>
+          <t>Confirm/export the final NK output and share it with Sean</t>
+        </is>
+      </c>
       <c r="M67" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -29478,12 +29510,16 @@
       </c>
       <c r="I68" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J68" s="18" t="n"/>
       <c r="K68" s="18" t="n"/>
-      <c r="L68" s="18" t="n"/>
+      <c r="L68" s="18" t="inlineStr">
+        <is>
+          <t>Confirm/export the final NK output and share it with Sean</t>
+        </is>
+      </c>
       <c r="M68" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -29531,12 +29567,16 @@
       </c>
       <c r="I69" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J69" s="18" t="n"/>
       <c r="K69" s="18" t="n"/>
-      <c r="L69" s="18" t="n"/>
+      <c r="L69" s="18" t="inlineStr">
+        <is>
+          <t>NK abstract-screening usability survey sent on 9 September</t>
+        </is>
+      </c>
       <c r="M69" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -29796,12 +29836,16 @@
       </c>
       <c r="I74" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J74" s="18" t="n"/>
       <c r="K74" s="18" t="n"/>
-      <c r="L74" s="18" t="n"/>
+      <c r="L74" s="18" t="inlineStr">
+        <is>
+          <t>Team reports full-text screening underway; confirm the retrieval and upload package</t>
+        </is>
+      </c>
       <c r="M74" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -29955,12 +29999,16 @@
       </c>
       <c r="I77" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J77" s="18" t="n"/>
       <c r="K77" s="18" t="n"/>
-      <c r="L77" s="18" t="n"/>
+      <c r="L77" s="18" t="inlineStr">
+        <is>
+          <t>Confirm criteria, tool setup and consolidation with Sean and Meghan</t>
+        </is>
+      </c>
       <c r="M77" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -30008,12 +30056,16 @@
       </c>
       <c r="I78" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J78" s="18" t="n"/>
       <c r="K78" s="18" t="n"/>
-      <c r="L78" s="18" t="n"/>
+      <c r="L78" s="18" t="inlineStr">
+        <is>
+          <t>Confirm criteria, tool setup and consolidation with Sean and Meghan</t>
+        </is>
+      </c>
       <c r="M78" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -30061,12 +30113,16 @@
       </c>
       <c r="I79" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J79" s="18" t="n"/>
       <c r="K79" s="18" t="n"/>
-      <c r="L79" s="18" t="n"/>
+      <c r="L79" s="18" t="inlineStr">
+        <is>
+          <t>Confirm criteria, tool setup and consolidation with Sean and Meghan</t>
+        </is>
+      </c>
       <c r="M79" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -30114,12 +30170,16 @@
       </c>
       <c r="I80" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J80" s="18" t="n"/>
       <c r="K80" s="18" t="n"/>
-      <c r="L80" s="18" t="n"/>
+      <c r="L80" s="18" t="inlineStr">
+        <is>
+          <t>Review team reports both Covidence and NK full-text screening underway</t>
+        </is>
+      </c>
       <c r="M80" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -30167,12 +30227,16 @@
       </c>
       <c r="I81" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J81" s="18" t="n"/>
       <c r="K81" s="18" t="n"/>
-      <c r="L81" s="18" t="n"/>
+      <c r="L81" s="18" t="inlineStr">
+        <is>
+          <t>Review team reports both Covidence and NK full-text screening underway</t>
+        </is>
+      </c>
       <c r="M81" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -31856,7 +31920,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -31866,7 +31930,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -31876,7 +31940,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Continue NK abstract screening before full-text work resumes.</t>
+          <t>Both abstract-screening workflows completed</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -31886,7 +31950,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -31970,7 +32034,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -31980,7 +32044,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>After NK screening</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -31990,7 +32054,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Export output once NK screening is complete.</t>
+          <t>Confirm and export the final NK abstract-screening output</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -32000,7 +32064,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -32027,7 +32091,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -32037,7 +32101,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>After abstract-screening closeout</t>
+          <t>Next 1–2 weeks</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -32047,7 +32111,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>Resume full-text workflow only after abstract-screening outputs are ready.</t>
+          <t>Full-text screening reported underway; setup and consolidation confirmation pending</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -32057,7 +32121,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -32153,12 +32217,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Probiotics full text paused</t>
+          <t>Probiotics abstract screening complete; full-text screening underway</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -32168,32 +32232,32 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Review Team</t>
+          <t>Sean / Meghan / Review Team</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>After NK abstract screening</t>
+          <t>Immediate confirmation</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Team confirmed Covidence full-text screening will remain paused until Nested Knowledge abstract screening is complete.</t>
+          <t>Jeremy confirmed both abstract arms complete and reported full-text screening underway; study-side confirmation requested</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>task-phase1-06-001</t>
+          <t>task-phase1-06-004</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>Complete Nested Knowledge abstract screening</t>
+          <t>Confirm full-text setup and consolidation</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -32258,7 +32322,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Full-text screening deliberately paused</t>
+          <t>Full-text setup/consolidation confirmation pending</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -32268,22 +32332,22 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Review Team</t>
+          <t>Sean / Meghan / Review Team</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>After NK abstract screening</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Sequencing dependency is intentional and should be monitored.</t>
+          <t>Both teams report full-text screening underway; confirm that study requirements are satisfied</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -42174,7 +42238,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Adjudication Pilot 2 underway; extension inputs shared</t>
+          <t>Adjudication Pilot 2 underway; Bi 2025 supplementary-file omission confirmed</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -42194,12 +42258,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Pilot 2 underway; 19-record BP mapping and PDF folder shared with Paweł</t>
+          <t>Pilot 2 underway; mapping shared; only the Bi 2025 main paper was included in Laser AI</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Complete Pilot 2, verify Bi 2025 supporting-file coverage and obtain Paweł’s access confirmation</t>
+          <t>Complete Pilot 2, document the Bi 2025 supplementary-file omission and obtain Paweł’s access/run confirmation</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
@@ -42246,7 +42310,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Corrective NK citations uploaded; full-text files received; validation pending</t>
+          <t>Conventional corrective screening complete; NK corrective set ready</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -42266,12 +42330,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Twenty-five citations—24 unique—were uploaded to the existing NK project; corresponding full texts were received</t>
+          <t>Updated decisions received for all 139 conventional records; 25 full texts are ready in NK</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Upload and validate the corrective PDFs, complete both screening arms and rerun the comparison</t>
+          <t>Complete the 25-record NK corrective screening and rerun the comparison</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -42318,7 +42382,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Full-text project opened; reviewer interaction issue under review</t>
+          <t>Full-text pool reopened to 138 records; reviewer confirmation pending</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -42338,12 +42402,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Combined project opened, but Kate cannot currently interact with it</t>
+          <t>Amin returned 138 records to the open pool for reviewer self-distribution</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Resolve Kate’s project-interaction issue and confirm that both screening arms can begin</t>
+          <t>Confirm Kate can claim records and that both full-text screening arms have started</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -42353,7 +42417,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Needs Action</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -42601,7 +42665,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Conventional abstract screening complete; NK screening underway</t>
+          <t>Both abstract-screening workflows complete; full-text screening reported underway</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -42621,17 +42685,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Calibration complete; conventional screening complete; NK screening continuing</t>
+          <t>Covidence and NK abstract screening complete; both teams have moved to full text</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Complete NK screening, record time and then start full text</t>
+          <t>Confirm full-text setup/consolidation, complete screening and record time</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Next 1–2 weeks</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -46404,7 +46468,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>All five extension groups consented; BP mapping and PDF folder shared; adjudication Pilot 2 underway; Bi 2025 supporting-file check pending</t>
+          <t>All five extension groups consented; Pilot 2 underway; Bi 2025 supplements confirmed absent from Laser AI; available survey counts approved for interim analysis</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -46669,7 +46733,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Laser AI operational; Fruit &amp; Veg full-text project opened, but reviewer interaction remains under review</t>
+          <t>Laser AI operational; 138 Fruit &amp; Veg records reopened in the pool; Kate’s confirmation remains pending</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -56481,7 +56545,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Adjudication Pilot 2 underway; extension inputs shared</t>
+          <t>Adjudication Pilot 2 underway; Bi 2025 supplementary-file omission confirmed</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -56549,7 +56613,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Pilot 2 underway; all 19 BP records mapped and shared with Paweł</t>
+          <t>Pilot 2 underway; all 19 records mapped; Bi 2025 source-file gap confirmed</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56566,7 +56630,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Mapping covers all 19 records: 17 PDFs and two ClinicalTrials.gov registry records</t>
+          <t>All 19 records mapped; Laser AI contains only the Bi 2025 main paper and no supplementary files</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56583,7 +56647,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete Pilot 2, confirm Bi 2025 supporting-file coverage and obtain Paweł’s access confirmation</t>
+          <t>Complete Pilot 2, document the Bi 2025 omission and obtain Paweł’s access/run confirmation</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56617,7 +56681,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Pilot 2 underway; Bi 2025 supplementary-file coverage requires confirmation</t>
+          <t>Pilot 2 underway; Bi 2025 supplements were not included in the Laser AI extraction</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -56673,7 +56737,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56920,7 +56984,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Mapping shared for all 19 records; 17 PDFs are available and two registry-only records link to ClinicalTrials.gov</t>
+          <t>Mapping shared for all 19 records; Bi 2025 supplements were absent from Laser AI</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -57174,12 +57238,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Extraction complete; Pilot 2 underway; Bi 2025 source-file check pending</t>
+          <t>Extraction complete; Pilot 2 underway; Bi 2025 supplement omission confirmed</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Pilot 2 started; extension mapping shared; Bi 2025 supporting-file verification pending</t>
+          <t>Pilot 2 underway; Meghan confirmed that only the Bi 2025 main paper was uploaded</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -58425,12 +58489,16 @@
       </c>
       <c r="I70" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J70" s="18" t="n"/>
       <c r="K70" s="18" t="n"/>
-      <c r="L70" s="18" t="n"/>
+      <c r="L70" s="18" t="inlineStr">
+        <is>
+          <t>Two abstract-screening responses received and confirmed</t>
+        </is>
+      </c>
       <c r="M70" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -58478,12 +58546,16 @@
       </c>
       <c r="I71" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J71" s="18" t="n"/>
       <c r="K71" s="18" t="n"/>
-      <c r="L71" s="18" t="n"/>
+      <c r="L71" s="18" t="inlineStr">
+        <is>
+          <t>Two abstract-screening responses received and confirmed</t>
+        </is>
+      </c>
       <c r="M71" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -59167,12 +59239,16 @@
       </c>
       <c r="I84" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J84" s="18" t="n"/>
       <c r="K84" s="18" t="n"/>
-      <c r="L84" s="18" t="n"/>
+      <c r="L84" s="18" t="inlineStr">
+        <is>
+          <t>Survey sent; three full-text-screening responses received and confirmed</t>
+        </is>
+      </c>
       <c r="M84" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -59220,12 +59296,16 @@
       </c>
       <c r="I85" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J85" s="18" t="n"/>
       <c r="K85" s="18" t="n"/>
-      <c r="L85" s="18" t="n"/>
+      <c r="L85" s="18" t="inlineStr">
+        <is>
+          <t>Survey sent; three full-text-screening responses received and confirmed</t>
+        </is>
+      </c>
       <c r="M85" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -59273,12 +59353,16 @@
       </c>
       <c r="I86" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J86" s="18" t="n"/>
       <c r="K86" s="18" t="n"/>
-      <c r="L86" s="18" t="n"/>
+      <c r="L86" s="18" t="inlineStr">
+        <is>
+          <t>Survey sent; three full-text-screening responses received and confirmed</t>
+        </is>
+      </c>
       <c r="M86" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -59962,12 +60046,16 @@
       </c>
       <c r="I99" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J99" s="18" t="n"/>
       <c r="K99" s="18" t="n"/>
-      <c r="L99" s="18" t="n"/>
+      <c r="L99" s="18" t="inlineStr">
+        <is>
+          <t>Survey sent; three data-extraction responses received and confirmed</t>
+        </is>
+      </c>
       <c r="M99" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -60015,12 +60103,16 @@
       </c>
       <c r="I100" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J100" s="18" t="n"/>
       <c r="K100" s="18" t="n"/>
-      <c r="L100" s="18" t="n"/>
+      <c r="L100" s="18" t="inlineStr">
+        <is>
+          <t>Survey sent; three data-extraction responses received and confirmed</t>
+        </is>
+      </c>
       <c r="M100" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -60068,12 +60160,16 @@
       </c>
       <c r="I101" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J101" s="18" t="n"/>
       <c r="K101" s="18" t="n"/>
-      <c r="L101" s="18" t="n"/>
+      <c r="L101" s="18" t="inlineStr">
+        <is>
+          <t>Survey sent; three data-extraction responses received and confirmed</t>
+        </is>
+      </c>
       <c r="M101" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -60998,7 +61094,7 @@
       </c>
       <c r="D120" s="23" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E120" s="23" t="inlineStr">
@@ -61016,7 +61112,7 @@
       </c>
       <c r="H120" s="23" t="inlineStr">
         <is>
-          <t>Survey shared with review team</t>
+          <t>Two abstract-screening responses received; counts confirmed for interim analysis</t>
         </is>
       </c>
       <c r="I120" s="23" t="inlineStr">
@@ -61445,12 +61541,12 @@
       </c>
       <c r="G133" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="H133" s="23" t="inlineStr">
         <is>
-          <t>Abstract screening survey shared after AI-assisted screening completion</t>
+          <t>Susan confirmed two BP abstract-screening responses</t>
         </is>
       </c>
       <c r="I133" s="23" t="inlineStr">
@@ -61915,7 +62011,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Corrective NK citations uploaded; PDFs received; validation pending</t>
+          <t>Conventional corrective screening complete; NK corrective screening ready</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -61983,7 +62079,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Existing NK project populated with 24 unique corrective citations; full texts received</t>
+          <t>The 139-record conventional corrective screening is complete; 25 NK full texts are ready</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -62000,7 +62096,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Meghan uploaded 25 citations—24 unique—and Sivem supplied the corresponding full texts</t>
+          <t>Sivem supplied updated decisions for 139 records; Meghan confirmed 25 full texts ready in NK</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -62017,7 +62113,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Upload and validate the corrective PDFs, then complete both screening arms</t>
+          <t>Complete the 25-record NK corrective screening and rerun the comparison</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -62051,7 +62147,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Analysis paused pending PDF validation and corrective cross-screening</t>
+          <t>Analysis paused pending completion of the NK corrective screening</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -62107,7 +62203,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -62354,7 +62450,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Conventional corrective PDFs are available; Sivem supplied files for the NK corrective set and identified #10631/#10608 as duplicates</t>
+          <t>Updated decisions received for 139 conventional records; 25 NK full texts are ready; #10631/#10608 identified as duplicates</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -62592,7 +62688,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>The conventional package was sent; 24 unique citations are in NK and their full texts have been received</t>
+          <t>Conventional corrective screening complete; the 25-record NK set is ready for screening</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -63919,12 +64015,16 @@
       </c>
       <c r="I71" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J71" s="18" t="n"/>
       <c r="K71" s="18" t="n"/>
-      <c r="L71" s="18" t="n"/>
+      <c r="L71" s="18" t="inlineStr">
+        <is>
+          <t>Susan confirmed two abstract-screening responses</t>
+        </is>
+      </c>
       <c r="M71" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -64085,7 +64185,7 @@
       <c r="K74" s="18" t="n"/>
       <c r="L74" s="18" t="inlineStr">
         <is>
-          <t>Ten selected-study PDFs shared with Sean</t>
+          <t>Conventional decisions received and 25 corrective full texts ready in NK</t>
         </is>
       </c>
       <c r="M74" s="18" t="inlineStr">
@@ -64135,12 +64235,16 @@
       </c>
       <c r="I75" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J75" s="18" t="n"/>
       <c r="K75" s="18" t="n"/>
-      <c r="L75" s="18" t="n"/>
+      <c r="L75" s="18" t="inlineStr">
+        <is>
+          <t>Duplicate records #10631 and #10608 identified</t>
+        </is>
+      </c>
       <c r="M75" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -64298,14 +64402,14 @@
       </c>
       <c r="I78" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J78" s="18" t="n"/>
       <c r="K78" s="18" t="n"/>
       <c r="L78" s="18" t="inlineStr">
         <is>
-          <t>Twenty-five citations uploaded to the existing project—24 unique after deduplication</t>
+          <t>Meghan confirmed that the 25 full texts are ready for screening</t>
         </is>
       </c>
       <c r="M78" s="18" t="inlineStr">
@@ -64355,14 +64459,14 @@
       </c>
       <c r="I79" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J79" s="18" t="n"/>
       <c r="K79" s="18" t="n"/>
       <c r="L79" s="18" t="inlineStr">
         <is>
-          <t>Upload the supplied PDFs and validate the 24-unique-record setup</t>
+          <t>Meghan confirmed that the 25 full texts are ready for screening</t>
         </is>
       </c>
       <c r="M79" s="18" t="inlineStr">
@@ -64412,14 +64516,14 @@
       </c>
       <c r="I80" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J80" s="18" t="n"/>
       <c r="K80" s="18" t="n"/>
       <c r="L80" s="18" t="inlineStr">
         <is>
-          <t>The 139-record RIS and PDF location were sent; screening completion pending</t>
+          <t>Updated conventional-screening decisions received for all 139 records</t>
         </is>
       </c>
       <c r="M80" s="18" t="inlineStr">
@@ -64469,14 +64573,14 @@
       </c>
       <c r="I81" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="J81" s="18" t="n"/>
       <c r="K81" s="18" t="n"/>
       <c r="L81" s="18" t="inlineStr">
         <is>
-          <t>Complete AI-assisted screening of the 24 unique records after PDF upload and validation</t>
+          <t>Twenty-five corrective full texts are ready for NK screening</t>
         </is>
       </c>
       <c r="M81" s="18" t="inlineStr">
@@ -64632,12 +64736,16 @@
       </c>
       <c r="I84" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J84" s="18" t="n"/>
       <c r="K84" s="18" t="n"/>
-      <c r="L84" s="18" t="n"/>
+      <c r="L84" s="18" t="inlineStr">
+        <is>
+          <t>Survey sent; two full-text-screening responses received and confirmed</t>
+        </is>
+      </c>
       <c r="M84" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -64685,12 +64793,16 @@
       </c>
       <c r="I85" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J85" s="18" t="n"/>
       <c r="K85" s="18" t="n"/>
-      <c r="L85" s="18" t="n"/>
+      <c r="L85" s="18" t="inlineStr">
+        <is>
+          <t>Survey sent; two full-text-screening responses received and confirmed</t>
+        </is>
+      </c>
       <c r="M85" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -64738,12 +64850,16 @@
       </c>
       <c r="I86" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J86" s="18" t="n"/>
       <c r="K86" s="18" t="n"/>
-      <c r="L86" s="18" t="n"/>
+      <c r="L86" s="18" t="inlineStr">
+        <is>
+          <t>Survey sent; two full-text-screening responses received and confirmed</t>
+        </is>
+      </c>
       <c r="M86" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -65435,12 +65551,16 @@
       </c>
       <c r="I99" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J99" s="18" t="n"/>
       <c r="K99" s="18" t="n"/>
-      <c r="L99" s="18" t="n"/>
+      <c r="L99" s="18" t="inlineStr">
+        <is>
+          <t>Survey sent; one data-extraction response received and confirmed</t>
+        </is>
+      </c>
       <c r="M99" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -65488,12 +65608,16 @@
       </c>
       <c r="I100" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J100" s="18" t="n"/>
       <c r="K100" s="18" t="n"/>
-      <c r="L100" s="18" t="n"/>
+      <c r="L100" s="18" t="inlineStr">
+        <is>
+          <t>Survey sent; one data-extraction response received and confirmed</t>
+        </is>
+      </c>
       <c r="M100" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -65541,12 +65665,16 @@
       </c>
       <c r="I101" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J101" s="18" t="n"/>
       <c r="K101" s="18" t="n"/>
-      <c r="L101" s="18" t="n"/>
+      <c r="L101" s="18" t="inlineStr">
+        <is>
+          <t>Survey sent; one data-extraction response received and confirmed</t>
+        </is>
+      </c>
       <c r="M101" s="18" t="inlineStr">
         <is>
           <t>Yes</t>

</xml_diff>

<commit_message>
Sync dashboard through September 21
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -25,7 +25,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upcoming_Meetings" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-06 Probiotics" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-07 Human Milk" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-08 Oral Galactagogues" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-08 LNS" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AI-assisted abstract screening restarting</t>
+          <t>Full-text screening underway; six oversized-PDF exceptions identified</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Laser AI work has restarted. AI-assisted abstract screening is expected to recommence; confirmation of actual commencement is pending.</t>
+          <t>Full-text project active; Kate distributed all 138 available records</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Laser AI work has restarted. AI-assisted abstract screening is expected to recommence; confirmation of actual commencement is pending.</t>
+          <t>Distribution succeeded; six PDFs cannot receive AI suggestions because they exceed 60 pages</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Confirm commencement of AI-assisted abstract screening and continue tracking time separately for both workflows.</t>
+          <t>Document handling of the six exceptions and complete full-text screening</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2537,7 +2537,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Restart approved; actual commencement and current screening progress still require confirmation.</t>
+          <t>Access resolved; six-record comparability issue remains</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2830,7 +2830,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Shared folder provided; PDFs being collected/uploaded for full-text screening.</t>
+          <t>Full-text package available; six PDFs exceed the Laser AI model limit</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3060,7 +3060,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Awaiting conventional export/DOIs, decision on 128 prior records, PDF-sharing method and final decision flow.</t>
+          <t>Kate distributed all 138 records; six oversized files require documented handling</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -4838,12 +4838,16 @@
       </c>
       <c r="I79" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J79" s="18" t="n"/>
       <c r="K79" s="18" t="n"/>
-      <c r="L79" s="18" t="n"/>
+      <c r="L79" s="18" t="inlineStr">
+        <is>
+          <t>Kate confirmed successful distribution of all 138 records</t>
+        </is>
+      </c>
       <c r="M79" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4891,12 +4895,16 @@
       </c>
       <c r="I80" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J80" s="18" t="n"/>
       <c r="K80" s="18" t="n"/>
-      <c r="L80" s="18" t="n"/>
+      <c r="L80" s="18" t="inlineStr">
+        <is>
+          <t>Conventional full-text screening underway</t>
+        </is>
+      </c>
       <c r="M80" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4944,12 +4952,16 @@
       </c>
       <c r="I81" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J81" s="18" t="n"/>
       <c r="K81" s="18" t="n"/>
-      <c r="L81" s="18" t="n"/>
+      <c r="L81" s="18" t="inlineStr">
+        <is>
+          <t>AI-assisted screening underway; six PDFs receive no model suggestions because they exceed 60 pages</t>
+        </is>
+      </c>
       <c r="M81" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -6633,7 +6645,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -6653,7 +6665,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Confirm logins and reviewer access before setup.</t>
+          <t>Kate confirmed that the 138 records were distributed without access issues</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -12677,7 +12689,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Current shared folder in the AI Methods Group location; use this version going forward.</t>
+          <t>Repository for finalized exports and protocols; working RIS and PDF sets remain in the relevant platform until consolidation.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -12725,7 +12737,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Current source of truth. Sean updated shortcuts; the old folder should be deleted or clearly archived to avoid confusion.</t>
+          <t>Use each NK/Laser AI project as the working source; save finalized consolidated exports in this folder.</t>
         </is>
       </c>
     </row>
@@ -22309,7 +22321,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Converted to phase1-07; setup inputs complete and Nested Knowledge configuration underway</t>
+          <t>Converted to phase1-07; both abstract-screening arms complete</t>
         </is>
       </c>
       <c r="E12" s="17" t="inlineStr">
@@ -22324,12 +22336,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Configuration and setup validation underway</t>
+          <t>Full-text consolidation underway</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Converted to phase1-07 Human Milk; RIS, criteria, protocol information and 35 data items received</t>
+          <t>Conventional list revised to 58; AI arm completed 2,024 records; common full-text set pending</t>
         </is>
       </c>
       <c r="I12" s="17" t="inlineStr">
@@ -22408,12 +22420,12 @@
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>Under Shortlisting</t>
+          <t>Converted to full sheet</t>
         </is>
       </c>
       <c r="D14" s="17" t="inlineStr">
         <is>
-          <t>Search by July 2026</t>
+          <t>Converted to phase1-08; expected count confirmed and accessible searches received</t>
         </is>
       </c>
       <c r="E14" s="17" t="inlineStr">
@@ -22422,16 +22434,24 @@
         </is>
       </c>
       <c r="F14" s="17" t="n"/>
-      <c r="G14" s="17" t="n"/>
-      <c r="H14" s="17" t="n"/>
+      <c r="G14" s="17" t="inlineStr">
+        <is>
+          <t>Final upload and deduplication pending</t>
+        </is>
+      </c>
+      <c r="H14" s="17" t="inlineStr">
+        <is>
+          <t>The 14,743 count matches Covidence; seven databases were inaccessible</t>
+        </is>
+      </c>
       <c r="I14" s="17" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -22823,7 +22843,7 @@
       </c>
       <c r="D28" s="17" t="inlineStr">
         <is>
-          <t>Onboarding and tool training completed; awaiting final template revisions</t>
+          <t>Converted to phase1-06; screening lists reconciled and full-text screening underway</t>
         </is>
       </c>
       <c r="E28" s="17" t="inlineStr">
@@ -22838,12 +22858,12 @@
       </c>
       <c r="G28" s="17" t="inlineStr">
         <is>
-          <t>Awaiting final template revisions</t>
+          <t>Missing-PDF retrieval and full-text screening underway</t>
         </is>
       </c>
       <c r="H28" s="17" t="inlineStr">
         <is>
-          <t>Converted to phase1-06 Probiotics; Nested Knowledge allocated</t>
+          <t>Fourteen AI-only and 16 Covidence-only records identified; NK updated</t>
         </is>
       </c>
       <c r="I28" s="17" t="inlineStr">
@@ -22957,7 +22977,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -23129,15 +23149,56 @@
       <c r="I34" s="17" t="n"/>
     </row>
     <row r="35" ht="24" customHeight="1" s="29">
-      <c r="A35" s="17" t="n"/>
-      <c r="B35" s="17" t="n"/>
-      <c r="C35" s="17" t="n"/>
-      <c r="D35" s="17" t="n"/>
-      <c r="E35" s="17" t="n"/>
-      <c r="F35" s="17" t="n"/>
-      <c r="G35" s="17" t="n"/>
-      <c r="H35" s="17" t="n"/>
-      <c r="I35" s="17" t="n"/>
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>new-23</t>
+        </is>
+      </c>
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>Álvaro Limones — Retention procedures for stabilising tooth position after orthodontic treatment</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="inlineStr">
+        <is>
+          <t>Shortlisted</t>
+        </is>
+      </c>
+      <c r="D35" s="17" t="inlineStr">
+        <is>
+          <t>Preliminarily eligible; onboarding started</t>
+        </is>
+      </c>
+      <c r="E35" s="17" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="F35" s="17" t="inlineStr">
+        <is>
+          <t>Álvaro Limones</t>
+        </is>
+      </c>
+      <c r="G35" s="17" t="inlineStr">
+        <is>
+          <t>Searches November 2026; 300–500 references; screening and extraction December 2026</t>
+        </is>
+      </c>
+      <c r="H35" s="17" t="inlineStr">
+        <is>
+          <t>Scope and protocol shared; schedule onboarding with the PI and review team</t>
+        </is>
+      </c>
+      <c r="I35" s="17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="24" customHeight="1" s="29">
       <c r="A36" s="17" t="n"/>
@@ -27540,7 +27601,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abstract screening underway</t>
+          <t>Abstract sets reconciled; full-text screening underway; missing PDFs remain</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -27608,7 +27669,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Setup phase underway; template revisions and project configuration remain before screening begins</t>
+          <t>Fourteen AI-only and 16 Covidence-only records identified; common full-text pool prepared</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -27625,7 +27686,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Setup phase underway; template revisions and project configuration remain before screening begins</t>
+          <t>NK updated with the Covidence-only citations; some PDFs still need retrieval</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -27642,7 +27703,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Continue conventional and AI-assisted abstract screening; monitor progress and time logs; then prepare the full-text screening stage.</t>
+          <t>Retrieve missing PDFs, complete both arms and record Bradley’s Covidence time</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -27676,7 +27737,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Project configuration and screening depend on final data extraction template revisions</t>
+          <t>Reconciliation complete; missing-PDF retrieval remains</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -27732,7 +27793,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -27846,6 +27907,11 @@
           <t>fullText</t>
         </is>
       </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -27964,7 +28030,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Citations aligned; missing PDFs remain</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -28164,6 +28230,11 @@
           <t>Not Started</t>
         </is>
       </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Full-text lists reconciled; NK updated; missing PDFs require retrieval</t>
+        </is>
+      </c>
       <c r="H44" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -29261,12 +29332,16 @@
       </c>
       <c r="I67" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J67" s="18" t="n"/>
       <c r="K67" s="18" t="n"/>
-      <c r="L67" s="18" t="n"/>
+      <c r="L67" s="18" t="inlineStr">
+        <is>
+          <t>NK title/abstract output obtained and compared with Covidence</t>
+        </is>
+      </c>
       <c r="M67" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -29314,12 +29389,16 @@
       </c>
       <c r="I68" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J68" s="18" t="n"/>
       <c r="K68" s="18" t="n"/>
-      <c r="L68" s="18" t="n"/>
+      <c r="L68" s="18" t="inlineStr">
+        <is>
+          <t>Both screening lists shared and reconciled</t>
+        </is>
+      </c>
       <c r="M68" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -29632,12 +29711,16 @@
       </c>
       <c r="I74" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J74" s="18" t="n"/>
       <c r="K74" s="18" t="n"/>
-      <c r="L74" s="18" t="n"/>
+      <c r="L74" s="18" t="inlineStr">
+        <is>
+          <t>Common full-text pool prepared; missing PDFs still need retrieval</t>
+        </is>
+      </c>
       <c r="M74" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -29685,12 +29768,16 @@
       </c>
       <c r="I75" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J75" s="18" t="n"/>
       <c r="K75" s="18" t="n"/>
-      <c r="L75" s="18" t="n"/>
+      <c r="L75" s="18" t="inlineStr">
+        <is>
+          <t>Missing full-text PDFs are being identified and retrieved</t>
+        </is>
+      </c>
       <c r="M75" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -29791,12 +29878,16 @@
       </c>
       <c r="I77" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J77" s="18" t="n"/>
       <c r="K77" s="18" t="n"/>
-      <c r="L77" s="18" t="n"/>
+      <c r="L77" s="18" t="inlineStr">
+        <is>
+          <t>Full-text comparison completed: 14 AI-only and 16 Covidence-only records</t>
+        </is>
+      </c>
       <c r="M77" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -29844,12 +29935,16 @@
       </c>
       <c r="I78" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J78" s="18" t="n"/>
       <c r="K78" s="18" t="n"/>
-      <c r="L78" s="18" t="n"/>
+      <c r="L78" s="18" t="inlineStr">
+        <is>
+          <t>NK updated with the 16 Covidence-only citations</t>
+        </is>
+      </c>
       <c r="M78" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -29897,12 +29992,16 @@
       </c>
       <c r="I79" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J79" s="18" t="n"/>
       <c r="K79" s="18" t="n"/>
-      <c r="L79" s="18" t="n"/>
+      <c r="L79" s="18" t="inlineStr">
+        <is>
+          <t>Reconciled citations are ready for full-text screening</t>
+        </is>
+      </c>
       <c r="M79" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -29955,7 +30054,11 @@
       </c>
       <c r="J80" s="18" t="n"/>
       <c r="K80" s="18" t="n"/>
-      <c r="L80" s="18" t="n"/>
+      <c r="L80" s="18" t="inlineStr">
+        <is>
+          <t>Covidence screening underway; Bradley may assist if his time is recorded</t>
+        </is>
+      </c>
       <c r="M80" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -30008,7 +30111,11 @@
       </c>
       <c r="J81" s="18" t="n"/>
       <c r="K81" s="18" t="n"/>
-      <c r="L81" s="18" t="n"/>
+      <c r="L81" s="18" t="inlineStr">
+        <is>
+          <t>NK screening underway; missing PDFs remain</t>
+        </is>
+      </c>
       <c r="M81" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -31794,9 +31901,14 @@
           <t>task-phase1-05-003</t>
         </is>
       </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Assign one tool only after a review is selected.</t>
+          <t>NK and Covidence outputs received and reconciled</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -31821,9 +31933,14 @@
           <t>task-phase1-05-004</t>
         </is>
       </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>Start onboarding only after candidate and tool are confirmed.</t>
+          <t>Reconciliation complete; retrieve missing PDFs and finish both screening arms</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -32123,7 +32240,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Setup in progress</t>
+          <t>Both abstract-screening arms complete; full-text consolidation underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -32191,7 +32308,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Onboarding/training are complete. The team has supplied a deduplicated RIS file with 2,053 records, 35 selected data items, and Study Protocol Info containing inclusion/exclusion/PICOS details. Nested Knowledge configuration can proceed.</t>
+          <t>Conventional and AI-assisted abstract screening complete</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -32208,7 +32325,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Onboarding/training are complete. The team has supplied a deduplicated RIS file with 2,053 records, 35 selected data items, and Study Protocol Info containing inclusion/exclusion/PICOS details. Nested Knowledge configuration can proceed.</t>
+          <t>Conventional list revised to 58 references; AI arm completed 2,024 records</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -32225,7 +32342,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Configure the Nested Knowledge project, confirm screening instructions/calibration, and begin abstract screening once setup is complete.</t>
+          <t>Correct the final NK decision, consolidate both arms and begin full-text screening</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -32242,7 +32359,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TBD - after setup validation</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -32259,7 +32376,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Key setup inputs are now received; Nested Knowledge configuration is the next step. Full-text PDFs can be assembled later for the full-text stage.</t>
+          <t>One NK decision needs correction; final common full-text set is pending</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -32276,7 +32393,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Full-text setup</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -32315,7 +32432,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -32412,6 +32529,11 @@
           <t>abstract</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -32422,6 +32544,11 @@
       <c r="A27" t="inlineStr">
         <is>
           <t>fullText</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -32542,7 +32669,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Study materials collection underway</t>
+          <t>Revised 58-reference conventional list received; AI-only additions pending consolidation</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -32727,7 +32854,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Both abstract-screening arms completed</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -32744,7 +32876,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Consolidate both arms’ selections and prepare the shared full-text set</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -33766,12 +33903,16 @@
       </c>
       <c r="I65" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J65" s="18" t="n"/>
       <c r="K65" s="18" t="n"/>
-      <c r="L65" s="18" t="n"/>
+      <c r="L65" s="18" t="inlineStr">
+        <is>
+          <t>Murali and Michelle completed conventional abstract screening</t>
+        </is>
+      </c>
       <c r="M65" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -33819,12 +33960,16 @@
       </c>
       <c r="I66" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J66" s="18" t="n"/>
       <c r="K66" s="18" t="n"/>
-      <c r="L66" s="18" t="n"/>
+      <c r="L66" s="18" t="inlineStr">
+        <is>
+          <t>Mohan completed screening of 2,024 records</t>
+        </is>
+      </c>
       <c r="M66" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -33872,12 +34017,16 @@
       </c>
       <c r="I67" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Needs Action</t>
         </is>
       </c>
       <c r="J67" s="18" t="n"/>
       <c r="K67" s="18" t="n"/>
-      <c r="L67" s="18" t="n"/>
+      <c r="L67" s="18" t="inlineStr">
+        <is>
+          <t>Correct the final accidentally deleted record and export the AI decisions</t>
+        </is>
+      </c>
       <c r="M67" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -33925,12 +34074,16 @@
       </c>
       <c r="I68" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J68" s="18" t="n"/>
       <c r="K68" s="18" t="n"/>
-      <c r="L68" s="18" t="n"/>
+      <c r="L68" s="18" t="inlineStr">
+        <is>
+          <t>Combine the AI and conventional full-text selections</t>
+        </is>
+      </c>
       <c r="M68" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -33978,12 +34131,16 @@
       </c>
       <c r="I69" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J69" s="18" t="n"/>
       <c r="K69" s="18" t="n"/>
-      <c r="L69" s="18" t="n"/>
+      <c r="L69" s="18" t="inlineStr">
+        <is>
+          <t>Send the NK usability survey to the AI/NK reviewers, not the conventional reviewers</t>
+        </is>
+      </c>
       <c r="M69" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -34243,12 +34400,16 @@
       </c>
       <c r="I74" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J74" s="18" t="n"/>
       <c r="K74" s="18" t="n"/>
-      <c r="L74" s="18" t="n"/>
+      <c r="L74" s="18" t="inlineStr">
+        <is>
+          <t>Revised conventional list contains 58 references; final union set pending</t>
+        </is>
+      </c>
       <c r="M74" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -34455,12 +34616,16 @@
       </c>
       <c r="I78" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J78" s="18" t="n"/>
       <c r="K78" s="18" t="n"/>
-      <c r="L78" s="18" t="n"/>
+      <c r="L78" s="18" t="inlineStr">
+        <is>
+          <t>Consolidate selections from both screening arms</t>
+        </is>
+      </c>
       <c r="M78" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -34508,12 +34673,16 @@
       </c>
       <c r="I79" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J79" s="18" t="n"/>
       <c r="K79" s="18" t="n"/>
-      <c r="L79" s="18" t="n"/>
+      <c r="L79" s="18" t="inlineStr">
+        <is>
+          <t>Validate the common full-text set after correcting the final NK decision</t>
+        </is>
+      </c>
       <c r="M79" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -34561,12 +34730,16 @@
       </c>
       <c r="I80" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="J80" s="18" t="n"/>
       <c r="K80" s="18" t="n"/>
-      <c r="L80" s="18" t="n"/>
+      <c r="L80" s="18" t="inlineStr">
+        <is>
+          <t>Conventional reviewers may begin their 58 selections but must also screen later AI-only additions</t>
+        </is>
+      </c>
       <c r="M80" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -34614,12 +34787,16 @@
       </c>
       <c r="I81" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J81" s="18" t="n"/>
       <c r="K81" s="18" t="n"/>
-      <c r="L81" s="18" t="n"/>
+      <c r="L81" s="18" t="inlineStr">
+        <is>
+          <t>Start after the combined full-text set is finalized</t>
+        </is>
+      </c>
       <c r="M81" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -36405,9 +36582,24 @@
           <t>task-phase1-05-003</t>
         </is>
       </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Consolidate full-text selections and start screening</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Final-decision correction and full-text-set consolidation</t>
+        </is>
+      </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Assign one tool only after a review is selected.</t>
+          <t>Both arms completed; revised 58-reference list received; one NK decision requires correction</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -36417,7 +36609,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -36518,9 +36710,24 @@
           <t>comm-phase1-05-001</t>
         </is>
       </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Human Milk abstract screening complete; full-text consolidation underway</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Under Review</t>
+        </is>
+      </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>One additional eligible review still needs to be identified or confirmed for Phase 1.</t>
+          <t>Both arms completed; conventional list revised to 58; correct the final NK decision and prepare the union set</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -36795,7 +37002,7 @@
     <row r="1" ht="18" customHeight="1" s="29">
       <c r="A1" s="28" t="inlineStr">
         <is>
-          <t>phase1-08 Oral Galactagogues | Dashboard Content Sheet</t>
+          <t>phase1-08 LNS | Dashboard Content Sheet</t>
         </is>
       </c>
       <c r="K1" s="18" t="n"/>
@@ -36865,7 +37072,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Oral Galactagogues</t>
+          <t>LNS</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -36882,7 +37089,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Oral galactagogues (natural therapies or drugs) for increasing breast milk production in mothers of non-hospitalised term infants</t>
+          <t>Preventive lipid-based nutrient supplements given with complementary foods to infants and young children 6 to 23 months of age for health, nutrition, and developmental outcomes</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -36916,7 +37123,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
+          <t>Expected reference count confirmed; available searches received</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -36950,7 +37157,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Laser AI</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -36967,7 +37174,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Siew Cheng Foong</t>
+          <t>Jai Das</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -36984,7 +37191,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Team declined participation because all relevant studies had already undergone screening, INSPECT-SR, data extraction and ROB 2; blinding was not feasible.</t>
+          <t>The 14,743-reference count matches Covidence; accessible searches have been supplied</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -37001,7 +37208,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Team declined participation because all relevant studies had already undergone screening, INSPECT-SR, data extraction and ROB 2; blinding was not feasible.</t>
+          <t>Seven databases were inaccessible; all other search results were provided</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -37018,7 +37225,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Retain as withdrawn/historical record; no active onboarding or tool setup required.</t>
+          <t>Upload and deduplicate the available results; document the seven inaccessible databases</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -37035,7 +37242,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>Awaiting final upload and deduplication</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -37052,7 +37259,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Rerun search produced 377 records, but all relevant studies had already been processed. Team formally declined on 2026-08-11.</t>
+          <t>Count confirmed; final reference set pending incorporation of received searches</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -37069,7 +37276,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -37108,7 +37315,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -37173,7 +37380,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -37188,6 +37395,11 @@
           <t>setup</t>
         </is>
       </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -37200,11 +37412,6 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Withdrawn - not participating</t>
-        </is>
-      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -37215,11 +37422,6 @@
       <c r="A27" t="inlineStr">
         <is>
           <t>fullText</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Rerun search produced 377 records, but all relevant studies had already been processed. Team formally declined on 2026-08-11.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -37313,12 +37515,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Expected count confirmed; available search results received; seven databases inaccessible</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -37509,12 +37711,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Onboarding confirmed; tool allocation and setup to follow.</t>
+          <t>Count confirmed; available searches awaiting upload and deduplication</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -38452,11 +38654,16 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J63" s="18" t="inlineStr"/>
       <c r="K63" s="18" t="inlineStr"/>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Available search files received; seven database searches were unavailable</t>
+        </is>
+      </c>
       <c r="M63" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -38504,12 +38711,16 @@
       </c>
       <c r="I64" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J64" s="18" t="inlineStr"/>
       <c r="K64" s="18" t="inlineStr"/>
-      <c r="L64" s="18" t="inlineStr"/>
+      <c r="L64" s="18" t="inlineStr">
+        <is>
+          <t>Expected 14,743 count confirmed; validate final count after upload and deduplication</t>
+        </is>
+      </c>
       <c r="M64" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -41084,7 +41295,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Complete onboarding and confirm tool-training/setup plan</t>
+          <t>Incorporate the available LNS search results</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -41104,7 +41315,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>After upload and deduplication</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -41114,7 +41325,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Onboarding confirmed; tool training and setup to follow.</t>
+          <t>Count confirmed; all accessible results received; document seven inaccessible databases</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -41124,7 +41335,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -41224,37 +41435,37 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>LNS count confirmed; available searches received</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Siew Cheng Foong / review team / Cochrane elective students / project team</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>Oral galactagogues onboarding confirmed</t>
-        </is>
-      </c>
-      <c r="D122" t="inlineStr">
-        <is>
-          <t>Siew Cheng Foong / review team / Cochrane elective students / project team</t>
-        </is>
-      </c>
-      <c r="E122" t="inlineStr">
-        <is>
-          <t>Krishna</t>
-        </is>
-      </c>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Initial onboarding will cover the study and parallel workflow; tool training and setup will be scheduled afterward.</t>
+          <t>The count matches Covidence; available files need incorporation and deduplication</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -41614,7 +41825,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Data extraction underway</t>
+          <t>Full Blood Pressure adjudication underway; first review folder opened</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -41634,17 +41845,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Data extraction is underway in both workflows. Completion was expected during the week of 2026-08-03, but final completion has not yet been confirmed.</t>
+          <t>First adjudication folder shared; Bartosz completed his assessment; weekly panel meetings scheduled</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Confirm whether both workflows have completed data extraction; collect outputs, time logs and usability-survey responses.</t>
+          <t>Complete remaining adjudications, consolidate decisions and collect specific questions for senior reviewers</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
         <is>
-          <t>Completion confirmation overdue</t>
+          <t>Weekly through 2026-10-29</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -41686,7 +41897,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Data extraction underway</t>
+          <t>Corrective screening in progress; consolidated full-text package available</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -41706,12 +41917,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Abstract and full-text screening are complete in the AI-assisted and conventional workflows. Ten studies are selected for data extraction. Conventional screening time-on-task is now complete; Robin's full-text time was corrected to 4h12. Repeated Laser AI run-validation issues remain provisional.</t>
+          <t>Conventional corrections received; 25-record NK corrective set ready; platform PDF package available</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Finalise the Nested Knowledge data-extraction workflow; correct Run 10 and resolve the 44 unevaluated citations in Runs 3-5; complete the interim comparison.</t>
+          <t>Complete the 25-record NK screening, rerun the comparison and save the finalized export</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -41758,7 +41969,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>AI-assisted abstract screening restarting</t>
+          <t>Full-text screening underway; six-record model-limit exception open</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -41778,12 +41989,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Laser AI work has restarted. AI-assisted abstract screening is expected to recommence; confirmation of actual commencement is pending.</t>
+          <t>Kate distributed all 138 records; six PDFs exceed Laser AI’s 60-page limit</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Confirm commencement of AI-assisted abstract screening and continue tracking conventional and AI-assisted screening time separately.</t>
+          <t>Resolve comparator handling for six oversized PDFs and complete both screening arms</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -41969,7 +42180,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Broad Phase 2 deferred; one additional review onboarding separately</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -41989,17 +42200,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Future batch planning</t>
+          <t>CD002283 is onboarding as the eighth current-study topic</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Keep placeholders until Phase 1 stabilizes.</t>
+          <t>Track CD002283 in New_Reviews until full setup begins</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Searches expected November 2026</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -42041,7 +42252,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Abstract screening underway</t>
+          <t>Abstract sets reconciled; full-text screening underway; missing PDFs remain</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -42061,12 +42272,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Setup phase underway; template revisions and project configuration remain before screening begins</t>
+          <t>Fourteen AI-only and 16 Covidence-only records identified; NK updated with Covidence additions</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Continue conventional and AI-assisted abstract screening; monitor progress and time logs; then prepare the full-text screening stage.</t>
+          <t>Retrieve missing PDFs, complete both full-text arms and record Bradley’s time</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -42113,7 +42324,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Setup in progress</t>
+          <t>Both abstract-screening arms complete; full-text consolidation underway</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -42133,17 +42344,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Onboarding/training are complete. The team has supplied a deduplicated RIS file with 2,053 records, 35 selected data items, and Study Protocol Info containing inclusion/exclusion/PICOS details. Nested Knowledge configuration can proceed.</t>
+          <t>Conventional arm selected 58 references; AI arm completed 2,024 records with one erroneous final decision</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Configure the Nested Knowledge project, confirm screening instructions/calibration, and begin abstract screening once setup is complete.</t>
+          <t>Correct the final NK decision, consolidate both arms’ full-text selections and send the survey to the NK reviewers</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>TBD - after setup validation</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -42170,12 +42381,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Oral Galactagogues</t>
+          <t>LNS</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Oral galactagogues (natural therapies or drugs) for increasing breast milk production in mothers of non-hospitalised term infants</t>
+          <t>Preventive lipid-based nutrient supplements given with complementary foods to infants and young children 6 to 23 months of age for health, nutrition, and developmental outcomes</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -42185,7 +42396,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
+          <t>Expected 14,743-reference count confirmed; available searches received</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -42195,32 +42406,32 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Laser AI</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Siew Cheng Foong</t>
+          <t>Jai Das</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Team declined participation because all relevant studies had already undergone screening, INSPECT-SR, data extraction and ROB 2; blinding was not feasible.</t>
+          <t>Count matches Covidence; all accessible searches supplied; seven databases were inaccessible</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Retain as withdrawn/historical record; no active onboarding or tool setup required.</t>
+          <t>Load and deduplicate the received searches, document inaccessible databases and finalize the screening set</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>Awaiting final upload and deduplication</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -42230,7 +42441,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>phase1-08 Oral Galactagogues</t>
+          <t>phase1-08 LNS</t>
         </is>
       </c>
     </row>
@@ -45844,7 +46055,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Decision Gate</t>
+          <t>All five extension groups consented; full adjudication underway; first BP review opened and one assessment completed</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -45871,7 +46082,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Broad Phase 2 deferred; CD002283 is onboarding as the eighth current-study topic</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -45996,7 +46207,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>AI Methods Group folder is the current source of truth; old folder should be archived or deleted.</t>
+          <t>Use NK/Laser AI as the working source for RIS and PDF sets; save finalized consolidated exports in this folder.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -46109,7 +46320,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Laser AI work restarted; Fruit &amp; Veg screening restart pending confirmation.</t>
+          <t>Kate distributed 138 records; six PDFs exceed the 60-page model limit and require documented comparator handling</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -55921,7 +56132,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Data extraction underway</t>
+          <t>Full Blood Pressure adjudication underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -55989,7 +56200,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Data extraction is underway in both workflows; final completion has not yet been confirmed.</t>
+          <t>First adjudication review opened; weekly panel process underway</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56006,7 +56217,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Completion was expected during the week of 2026-08-03; confirmation remains pending.</t>
+          <t>First-review folder and spreadsheet shared; Bartosz completed his assessment</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56023,7 +56234,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Confirm completion of both extraction workflows and collect outputs, time logs and usability-survey responses.</t>
+          <t>Complete remaining assessments, consolidate decisions and collect focused senior-reviewer questions</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56040,7 +56251,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Completion confirmation overdue</t>
+          <t>Weekly through 2026-10-29</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -56057,7 +56268,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Data extraction is underway; completion is now expected during the week of 2026-08-10.</t>
+          <t>Full adjudication underway; shared senior-reviewer question document pending</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -56113,7 +56324,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56355,7 +56566,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>All 19 records mapped; Bi 2025 supplements documented as absent from the Laser AI extraction</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -56593,7 +56804,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Extraction complete; full adjudication underway</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>First BP adjudication review opened; one adjudicator completed; weekly meetings scheduled</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -59642,7 +59858,11 @@
       </c>
       <c r="J104" s="18" t="n"/>
       <c r="K104" s="18" t="n"/>
-      <c r="L104" s="18" t="n"/>
+      <c r="L104" s="18" t="inlineStr">
+        <is>
+          <t>Full adjudication opened; first-review materials shared and one assessment completed</t>
+        </is>
+      </c>
       <c r="M104" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -59854,7 +60074,11 @@
       </c>
       <c r="J108" s="18" t="n"/>
       <c r="K108" s="18" t="n"/>
-      <c r="L108" s="18" t="n"/>
+      <c r="L108" s="18" t="inlineStr">
+        <is>
+          <t>Weekly adjudication meetings scheduled through 29 October</t>
+        </is>
+      </c>
       <c r="M108" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -61305,7 +61529,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Data extraction underway</t>
+          <t>Corrective screening in progress; consolidated platform package available</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -61373,7 +61597,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Abstract and full-text screening are complete in the AI-assisted and conventional workflows. Ten studies are selected for data extraction. Conventional screening time-on-task is now complete; Robin's full-text time was corrected to 4h12. Repeated Laser AI run-validation issues remain provisional.</t>
+          <t>Full-text setup and consolidation complete; 25-record NK corrective screening remains</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -61390,7 +61614,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Abstract and full-text screening are complete in the AI-assisted and conventional workflows. Ten studies are selected for data extraction. Conventional screening time-on-task is now complete; Robin's full-text time was corrected to 4h12. Repeated Laser AI run-validation issues remain provisional.</t>
+          <t>Psoriasis is currently the complete PDF package available to the extension team</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -61407,7 +61631,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Finalise the Nested Knowledge data-extraction workflow; correct Run 10 and resolve the 44 unevaluated citations in Runs 3-5; complete the interim comparison.</t>
+          <t>Complete the NK corrective screening, rerun the comparison and save the finalized export</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -61441,7 +61665,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Repeated Laser AI outputs still require validation before final reporting; conventional screening timing has now been received and updated.</t>
+          <t>Extension files are available; final validation still awaits the NK corrective decisions</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -61497,7 +61721,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -61739,7 +61963,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Consolidated full-text package available directly from NK; duplicate records remain documented</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -61969,7 +62193,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Conventional and AI-assisted full-text screening complete; 10 studies selected.</t>
+          <t>Full-text package consolidated for export; the 25-record NK corrective screening remains pending</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">

</xml_diff>

<commit_message>
Fix executive stage tracker milestones
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2287,6 +2287,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -2469,7 +2470,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Full-text project active; Kate distributed all 138 available records</t>
+          <t>Full-text screening underway</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2602,6 +2603,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -2692,7 +2694,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Restarting - commencement to be confirmed</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2724,6 +2726,7 @@
           <t>extraction</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2736,12 +2739,14 @@
           <t>analysis</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -2927,6 +2932,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -3092,6 +3098,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -6554,6 +6561,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -7870,6 +7878,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -8180,6 +8189,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -8305,6 +8315,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -8490,6 +8501,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -8640,6 +8652,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -12054,6 +12067,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -12355,6 +12369,7 @@
         </is>
       </c>
     </row>
+    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -12500,6 +12515,7 @@
         </is>
       </c>
     </row>
+    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -12609,6 +12625,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -12894,6 +12911,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -13076,7 +13094,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Protocol and 35 selected extraction items are received. Screening has not started. Sean is awaiting clarification on wildcard operators before executing available database searches; LILACS/IBECS access remains unresolved.</t>
+          <t>Abstract screening ready to begin</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -13209,6 +13227,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -13282,7 +13301,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>3,486 references uploaded; decision flow approved</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -13297,6 +13321,11 @@
           <t>abstract</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13309,6 +13338,7 @@
           <t>fullText</t>
         </is>
       </c>
+      <c r="B27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13321,6 +13351,7 @@
           <t>extraction</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13333,12 +13364,14 @@
           <t>analysis</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -13524,6 +13557,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -13679,6 +13713,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -17113,6 +17148,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -17414,6 +17450,7 @@
         </is>
       </c>
     </row>
+    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -17559,6 +17596,7 @@
         </is>
       </c>
     </row>
+    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -17684,6 +17722,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -17999,6 +18038,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -18119,6 +18159,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -18304,6 +18345,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -18454,6 +18496,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -21868,6 +21911,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -21998,6 +22042,7 @@
         </is>
       </c>
     </row>
+    <row r="116"/>
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
         <is>
@@ -22088,6 +22133,7 @@
         </is>
       </c>
     </row>
+    <row r="120"/>
     <row r="121">
       <c r="A121" s="5" t="inlineStr">
         <is>
@@ -22200,6 +22246,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -22251,6 +22298,8 @@
         <v/>
       </c>
     </row>
+    <row r="9"/>
+    <row r="10"/>
     <row r="11" ht="16" customHeight="1" s="29">
       <c r="A11" s="16" t="inlineStr">
         <is>
@@ -23376,6 +23425,8 @@
       <c r="H51" s="17" t="n"/>
       <c r="I51" s="17" t="n"/>
     </row>
+    <row r="52"/>
+    <row r="53"/>
     <row r="54">
       <c r="A54" s="31" t="inlineStr">
         <is>
@@ -27487,6 +27538,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -27669,7 +27721,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Fourteen AI-only and 16 Covidence-only records identified; common full-text pool prepared</t>
+          <t>Full-text screening underway</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -27802,6 +27854,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -27892,7 +27945,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -27909,7 +27962,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -27924,6 +27977,7 @@
           <t>extraction</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -27936,12 +27990,14 @@
           <t>analysis</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -28127,6 +28183,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -28258,6 +28315,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -31708,6 +31766,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -31959,6 +32018,7 @@
         </is>
       </c>
     </row>
+    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -32050,6 +32110,7 @@
         </is>
       </c>
     </row>
+    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -32126,6 +32187,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -32308,7 +32370,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Conventional and AI-assisted abstract screening complete</t>
+          <t>Full-text setup and reconciliation underway</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -32441,6 +32503,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -32514,7 +32577,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -32563,6 +32626,7 @@
           <t>extraction</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -32575,12 +32639,14 @@
           <t>analysis</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -32766,6 +32832,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -32907,6 +32974,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -36389,6 +36457,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -36645,6 +36714,7 @@
         </is>
       </c>
     </row>
+    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -36751,6 +36821,7 @@
         </is>
       </c>
     </row>
+    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -36900,6 +36971,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
@@ -36960,6 +37032,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="28" customHeight="1" s="29">
       <c r="A16" s="19" t="inlineStr">
         <is>
@@ -37009,6 +37082,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -37191,7 +37265,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>The 14,743-reference count matches Covidence; accessible searches have been supplied</t>
+          <t>Setup: final search upload and deduplication underway</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -37324,6 +37398,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -37412,6 +37487,7 @@
           <t>abstract</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -37424,6 +37500,7 @@
           <t>fullText</t>
         </is>
       </c>
+      <c r="B27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -37436,6 +37513,7 @@
           <t>extraction</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -37448,12 +37526,14 @@
           <t>analysis</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -37639,6 +37719,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -37794,6 +37875,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -41214,6 +41296,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -41344,6 +41427,10 @@
         </is>
       </c>
     </row>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -41489,6 +41576,7 @@
         </is>
       </c>
     </row>
+    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -41830,7 +41918,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -41845,7 +41933,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>First adjudication folder shared; Bartosz completed his assessment; weekly panel meetings scheduled</t>
+          <t>Analysis: full adjudication underway</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -41902,7 +41990,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -41917,7 +42005,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Conventional corrections received; 25-record NK corrective set ready; platform PDF package available</t>
+          <t>Analysis: corrective validation in progress</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -41989,7 +42077,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Kate distributed all 138 records; six PDFs exceed Laser AI’s 60-page limit</t>
+          <t>Full-text screening underway</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -42128,7 +42216,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Protocol and 35 selected extraction items are received. Screening has not started. Sean is awaiting clarification on wildcard operators before executing available database searches; LILACS/IBECS access remains unresolved.</t>
+          <t>Abstract screening ready to begin</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -42272,7 +42360,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Fourteen AI-only and 16 Covidence-only records identified; NK updated with Covidence additions</t>
+          <t>Full-text screening underway</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -42344,7 +42432,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Conventional arm selected 58 references; AI arm completed 2,024 records with one erroneous final decision</t>
+          <t>Full-text setup and reconciliation underway</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -42416,7 +42504,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Count matches Covidence; all accessible searches supplied; seven databases were inaccessible</t>
+          <t>Setup: final search upload and deduplication underway</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -45942,6 +46030,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -46118,6 +46207,8 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
@@ -46329,6 +46420,8 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
@@ -46612,6 +46705,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -46922,6 +47016,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -47042,6 +47137,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -47227,6 +47323,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -47377,6 +47474,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -50791,6 +50889,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -51040,6 +51139,7 @@
         </is>
       </c>
     </row>
+    <row r="118"/>
     <row r="119">
       <c r="A119" s="5" t="inlineStr">
         <is>
@@ -51247,6 +51347,7 @@
         </is>
       </c>
     </row>
+    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -51377,6 +51478,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -51687,6 +51789,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -51807,6 +51910,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -51992,6 +52096,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -52142,6 +52247,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -55556,6 +55662,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -55743,6 +55850,7 @@
         </is>
       </c>
     </row>
+    <row r="117"/>
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
         <is>
@@ -55888,6 +55996,7 @@
         </is>
       </c>
     </row>
+    <row r="121"/>
     <row r="122">
       <c r="A122" s="5" t="inlineStr">
         <is>
@@ -56018,6 +56127,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -56149,7 +56259,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -56200,7 +56310,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>First adjudication review opened; weekly panel process underway</t>
+          <t>Analysis: full adjudication underway</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56333,6 +56443,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -56457,7 +56568,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -56472,12 +56583,18 @@
           <t>analysis</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -56663,6 +56780,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -56818,6 +56936,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -60240,6 +60359,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -60761,6 +60881,7 @@
     <row r="124" s="29"/>
     <row r="125" s="29"/>
     <row r="126" s="29"/>
+    <row r="127"/>
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
         <is>
@@ -61216,6 +61337,7 @@
     <row r="138" s="29"/>
     <row r="139" s="29"/>
     <row r="140" s="29"/>
+    <row r="141"/>
     <row r="142">
       <c r="A142" s="5" t="inlineStr">
         <is>
@@ -61415,6 +61537,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -61546,7 +61669,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -61597,7 +61720,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Full-text setup and consolidation complete; 25-record NK corrective screening remains</t>
+          <t>Analysis: corrective validation in progress</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -61730,6 +61853,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -61837,7 +61961,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Complete / corrective follow-up</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -61854,7 +61978,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -61869,12 +61993,18 @@
           <t>analysis</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Risk — corrective validation pending</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -62060,6 +62190,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -62230,6 +62361,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -65644,6 +65776,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -66215,6 +66348,7 @@
     <row r="124" s="29"/>
     <row r="125" s="29"/>
     <row r="126" s="29"/>
+    <row r="127"/>
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
         <is>
@@ -66783,6 +66917,7 @@
     </row>
     <row r="138" s="29"/>
     <row r="139" s="29"/>
+    <row r="140"/>
     <row r="141">
       <c r="A141" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Sync executive stage tracker milestones
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2287,6 +2287,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -2469,7 +2470,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Full-text project active; Kate distributed all 138 available records</t>
+          <t>Full-text screening underway</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2602,6 +2603,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -2692,7 +2694,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Restarting - commencement to be confirmed</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2724,6 +2726,7 @@
           <t>extraction</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2736,12 +2739,14 @@
           <t>analysis</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -2927,6 +2932,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -3092,6 +3098,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -6554,6 +6561,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -7870,6 +7878,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -8180,6 +8189,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -8305,6 +8315,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -8490,6 +8501,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -8640,6 +8652,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -12054,6 +12067,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -12355,6 +12369,7 @@
         </is>
       </c>
     </row>
+    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -12500,6 +12515,7 @@
         </is>
       </c>
     </row>
+    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -12609,6 +12625,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -12894,6 +12911,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -13076,7 +13094,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Protocol and 35 selected extraction items are received. Screening has not started. Sean is awaiting clarification on wildcard operators before executing available database searches; LILACS/IBECS access remains unresolved.</t>
+          <t>Abstract screening ready to begin</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -13209,6 +13227,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -13282,7 +13301,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>3,486 references uploaded; decision flow approved</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -13297,6 +13321,11 @@
           <t>abstract</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13309,6 +13338,7 @@
           <t>fullText</t>
         </is>
       </c>
+      <c r="B27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13321,6 +13351,7 @@
           <t>extraction</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13333,12 +13364,14 @@
           <t>analysis</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -13524,6 +13557,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -13679,6 +13713,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -17113,6 +17148,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -17414,6 +17450,7 @@
         </is>
       </c>
     </row>
+    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -17559,6 +17596,7 @@
         </is>
       </c>
     </row>
+    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -17684,6 +17722,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -17999,6 +18038,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -18119,6 +18159,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -18304,6 +18345,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -18454,6 +18496,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -21868,6 +21911,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -21998,6 +22042,7 @@
         </is>
       </c>
     </row>
+    <row r="116"/>
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
         <is>
@@ -22088,6 +22133,7 @@
         </is>
       </c>
     </row>
+    <row r="120"/>
     <row r="121">
       <c r="A121" s="5" t="inlineStr">
         <is>
@@ -22200,6 +22246,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -22251,6 +22298,8 @@
         <v/>
       </c>
     </row>
+    <row r="9"/>
+    <row r="10"/>
     <row r="11" ht="16" customHeight="1" s="29">
       <c r="A11" s="16" t="inlineStr">
         <is>
@@ -23376,6 +23425,8 @@
       <c r="H51" s="17" t="n"/>
       <c r="I51" s="17" t="n"/>
     </row>
+    <row r="52"/>
+    <row r="53"/>
     <row r="54">
       <c r="A54" s="31" t="inlineStr">
         <is>
@@ -27487,6 +27538,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -27669,7 +27721,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Fourteen AI-only and 16 Covidence-only records identified; common full-text pool prepared</t>
+          <t>Full-text screening underway</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -27802,6 +27854,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -27892,7 +27945,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -27909,7 +27962,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -27924,6 +27977,7 @@
           <t>extraction</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -27936,12 +27990,14 @@
           <t>analysis</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -28127,6 +28183,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -28258,6 +28315,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -31708,6 +31766,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -31959,6 +32018,7 @@
         </is>
       </c>
     </row>
+    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -32050,6 +32110,7 @@
         </is>
       </c>
     </row>
+    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -32126,6 +32187,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -32308,7 +32370,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Conventional and AI-assisted abstract screening complete</t>
+          <t>Full-text setup and reconciliation underway</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -32441,6 +32503,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -32514,7 +32577,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -32563,6 +32626,7 @@
           <t>extraction</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -32575,12 +32639,14 @@
           <t>analysis</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -32766,6 +32832,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -32907,6 +32974,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -36389,6 +36457,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -36645,6 +36714,7 @@
         </is>
       </c>
     </row>
+    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -36751,6 +36821,7 @@
         </is>
       </c>
     </row>
+    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -36900,6 +36971,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
@@ -36960,6 +37032,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="28" customHeight="1" s="29">
       <c r="A16" s="19" t="inlineStr">
         <is>
@@ -37009,6 +37082,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -37191,7 +37265,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>The 14,743-reference count matches Covidence; accessible searches have been supplied</t>
+          <t>Setup: final search upload and deduplication underway</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -37324,6 +37398,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -37412,6 +37487,7 @@
           <t>abstract</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -37424,6 +37500,7 @@
           <t>fullText</t>
         </is>
       </c>
+      <c r="B27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -37436,6 +37513,7 @@
           <t>extraction</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -37448,12 +37526,14 @@
           <t>analysis</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -37639,6 +37719,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -37794,6 +37875,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -41214,6 +41296,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -41344,6 +41427,10 @@
         </is>
       </c>
     </row>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -41489,6 +41576,7 @@
         </is>
       </c>
     </row>
+    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -41830,7 +41918,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -41845,7 +41933,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>First adjudication folder shared; Bartosz completed his assessment; weekly panel meetings scheduled</t>
+          <t>Analysis: full adjudication underway</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -41902,7 +41990,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -41917,7 +42005,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Conventional corrections received; 25-record NK corrective set ready; platform PDF package available</t>
+          <t>Analysis: corrective validation in progress</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -41989,7 +42077,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Kate distributed all 138 records; six PDFs exceed Laser AI’s 60-page limit</t>
+          <t>Full-text screening underway</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -42128,7 +42216,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Protocol and 35 selected extraction items are received. Screening has not started. Sean is awaiting clarification on wildcard operators before executing available database searches; LILACS/IBECS access remains unresolved.</t>
+          <t>Abstract screening ready to begin</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -42272,7 +42360,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Fourteen AI-only and 16 Covidence-only records identified; NK updated with Covidence additions</t>
+          <t>Full-text screening underway</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -42344,7 +42432,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Conventional arm selected 58 references; AI arm completed 2,024 records with one erroneous final decision</t>
+          <t>Full-text setup and reconciliation underway</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -42416,7 +42504,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Count matches Covidence; all accessible searches supplied; seven databases were inaccessible</t>
+          <t>Setup: final search upload and deduplication underway</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -45942,6 +46030,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -46118,6 +46207,8 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
@@ -46329,6 +46420,8 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
@@ -46612,6 +46705,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -46922,6 +47016,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -47042,6 +47137,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -47227,6 +47323,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -47377,6 +47474,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -50791,6 +50889,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -51040,6 +51139,7 @@
         </is>
       </c>
     </row>
+    <row r="118"/>
     <row r="119">
       <c r="A119" s="5" t="inlineStr">
         <is>
@@ -51247,6 +51347,7 @@
         </is>
       </c>
     </row>
+    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -51377,6 +51478,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -51687,6 +51789,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -51807,6 +51910,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -51992,6 +52096,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -52142,6 +52247,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -55556,6 +55662,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -55743,6 +55850,7 @@
         </is>
       </c>
     </row>
+    <row r="117"/>
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
         <is>
@@ -55888,6 +55996,7 @@
         </is>
       </c>
     </row>
+    <row r="121"/>
     <row r="122">
       <c r="A122" s="5" t="inlineStr">
         <is>
@@ -56018,6 +56127,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -56149,7 +56259,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -56200,7 +56310,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>First adjudication review opened; weekly panel process underway</t>
+          <t>Analysis: full adjudication underway</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56333,6 +56443,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -56457,7 +56568,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -56472,12 +56583,18 @@
           <t>analysis</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -56663,6 +56780,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -56818,6 +56936,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -60240,6 +60359,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -60761,6 +60881,7 @@
     <row r="124" s="29"/>
     <row r="125" s="29"/>
     <row r="126" s="29"/>
+    <row r="127"/>
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
         <is>
@@ -61216,6 +61337,7 @@
     <row r="138" s="29"/>
     <row r="139" s="29"/>
     <row r="140" s="29"/>
+    <row r="141"/>
     <row r="142">
       <c r="A142" s="5" t="inlineStr">
         <is>
@@ -61415,6 +61537,7 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -61546,7 +61669,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -61597,7 +61720,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Full-text setup and consolidation complete; 25-record NK corrective screening remains</t>
+          <t>Analysis: corrective validation in progress</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -61730,6 +61853,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -61837,7 +61961,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Complete / corrective follow-up</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -61854,7 +61978,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -61869,12 +61993,18 @@
           <t>analysis</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Risk — corrective validation pending</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -62060,6 +62190,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -62230,6 +62361,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -65644,6 +65776,7 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -66215,6 +66348,7 @@
     <row r="124" s="29"/>
     <row r="125" s="29"/>
     <row r="126" s="29"/>
+    <row r="127"/>
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
         <is>
@@ -66783,6 +66917,7 @@
     </row>
     <row r="138" s="29"/>
     <row r="139" s="29"/>
+    <row r="140"/>
     <row r="141">
       <c r="A141" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update dashboard through September 24
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2287,7 +2287,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -2487,7 +2486,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Distribution succeeded; six PDFs cannot receive AI suggestions because they exceed 60 pages</t>
+          <t>Kate successfully distributed all 138 records; six oversized PDFs cannot receive model suggestions</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2504,7 +2503,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Document handling of the six exceptions and complete full-text screening</t>
+          <t>Complete both full-text arms and document the six exceptions in the comparison</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2538,7 +2537,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Access resolved; six-record comparability issue remains</t>
+          <t>Screening underway; six records will be evaluated without AI model suggestions</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2594,7 +2593,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2603,7 +2602,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -2726,7 +2724,6 @@
           <t>extraction</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2739,14 +2736,12 @@
           <t>analysis</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -2835,7 +2830,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Full-text package available; six PDFs exceed the Laser AI model limit</t>
+          <t>Full-text set contains 144 records; six oversized PDFs were distributed without model suggestions</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2932,7 +2927,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -3066,7 +3060,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Kate distributed all 138 records; six oversized files require documented handling</t>
+          <t>Kate distributed the 138 records; both full-text workflows are underway</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -3098,7 +3092,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -4852,7 +4845,7 @@
       <c r="K79" s="18" t="n"/>
       <c r="L79" s="18" t="inlineStr">
         <is>
-          <t>Kate confirmed successful distribution of all 138 records</t>
+          <t>Kate successfully claimed and distributed the records</t>
         </is>
       </c>
       <c r="M79" s="18" t="inlineStr">
@@ -4909,7 +4902,7 @@
       <c r="K80" s="18" t="n"/>
       <c r="L80" s="18" t="inlineStr">
         <is>
-          <t>Conventional full-text screening underway</t>
+          <t>Conventional full-text screening underway; the six oversized records were already screened conventionally</t>
         </is>
       </c>
       <c r="M80" s="18" t="inlineStr">
@@ -4966,7 +4959,7 @@
       <c r="K81" s="18" t="n"/>
       <c r="L81" s="18" t="inlineStr">
         <is>
-          <t>AI-assisted screening underway; six PDFs receive no model suggestions because they exceed 60 pages</t>
+          <t>Laser AI screening underway; six PDFs will be screened without model suggestions</t>
         </is>
       </c>
       <c r="M81" s="18" t="inlineStr">
@@ -6561,7 +6554,6 @@
         </is>
       </c>
     </row>
-    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -6673,7 +6665,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Kate confirmed that the 138 records were distributed without access issues</t>
+          <t>Kate confirmed successful distribution of all 138 records</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -6683,7 +6675,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7878,7 +7870,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -8189,7 +8180,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -8315,7 +8305,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -8501,7 +8490,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -8652,7 +8640,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -12067,7 +12054,6 @@
         </is>
       </c>
     </row>
-    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -12369,7 +12355,6 @@
         </is>
       </c>
     </row>
-    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -12515,7 +12500,6 @@
         </is>
       </c>
     </row>
-    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -12625,7 +12609,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -12911,7 +12894,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -13227,7 +13209,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -13338,7 +13319,6 @@
           <t>fullText</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13351,7 +13331,6 @@
           <t>extraction</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13364,14 +13343,12 @@
           <t>analysis</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -13557,7 +13534,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -13713,7 +13689,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -17148,7 +17123,6 @@
         </is>
       </c>
     </row>
-    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -17450,7 +17424,6 @@
         </is>
       </c>
     </row>
-    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -17596,7 +17569,6 @@
         </is>
       </c>
     </row>
-    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -17722,7 +17694,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -18038,7 +18009,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -18159,7 +18129,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -18345,7 +18314,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -18496,7 +18464,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -21911,7 +21878,6 @@
         </is>
       </c>
     </row>
-    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -22042,7 +22008,6 @@
         </is>
       </c>
     </row>
-    <row r="116"/>
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
         <is>
@@ -22133,7 +22098,6 @@
         </is>
       </c>
     </row>
-    <row r="120"/>
     <row r="121">
       <c r="A121" s="5" t="inlineStr">
         <is>
@@ -22246,7 +22210,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -22298,8 +22261,6 @@
         <v/>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10"/>
     <row r="11" ht="16" customHeight="1" s="29">
       <c r="A11" s="16" t="inlineStr">
         <is>
@@ -22370,7 +22331,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Converted to phase1-07; both abstract-screening arms complete</t>
+          <t>Converted to phase1-07; both abstract arms complete and full-text reconciliation underway</t>
         </is>
       </c>
       <c r="E12" s="17" t="inlineStr">
@@ -22385,12 +22346,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Full-text consolidation underway</t>
+          <t>Full-text reconciliation underway</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Conventional list revised to 58; AI arm completed 2,024 records; common full-text set pending</t>
+          <t>Seventy-four full-text studies identified; five record-level issues require reconciliation</t>
         </is>
       </c>
       <c r="I12" s="17" t="inlineStr">
@@ -22474,7 +22435,7 @@
       </c>
       <c r="D14" s="17" t="inlineStr">
         <is>
-          <t>Converted to phase1-08; expected count confirmed and accessible searches received</t>
+          <t>Converted to phase1-08; latest uploads produced 16,891 deduplicated citations</t>
         </is>
       </c>
       <c r="E14" s="17" t="inlineStr">
@@ -22485,12 +22446,12 @@
       <c r="F14" s="17" t="n"/>
       <c r="G14" s="17" t="inlineStr">
         <is>
-          <t>Final upload and deduplication pending</t>
+          <t>Awaiting decision-flow approval and Laser AI access</t>
         </is>
       </c>
       <c r="H14" s="17" t="inlineStr">
         <is>
-          <t>The 14,743 count matches Covidence; seven databases were inaccessible</t>
+          <t>Baseline count confirmed; all accessible searches uploaded; seven databases inaccessible</t>
         </is>
       </c>
       <c r="I14" s="17" t="inlineStr">
@@ -22892,7 +22853,7 @@
       </c>
       <c r="D28" s="17" t="inlineStr">
         <is>
-          <t>Converted to phase1-06; screening lists reconciled and full-text screening underway</t>
+          <t>Converted to phase1-06; both full-text arms aligned and cleared to proceed</t>
         </is>
       </c>
       <c r="E28" s="17" t="inlineStr">
@@ -22907,12 +22868,12 @@
       </c>
       <c r="G28" s="17" t="inlineStr">
         <is>
-          <t>Missing-PDF retrieval and full-text screening underway</t>
+          <t>Full-text screening underway; missing PDFs still required</t>
         </is>
       </c>
       <c r="H28" s="17" t="inlineStr">
         <is>
-          <t>Fourteen AI-only and 16 Covidence-only records identified; NK updated</t>
+          <t>Meghan confirmed alignment of both arms; missing PDFs remain</t>
         </is>
       </c>
       <c r="I28" s="17" t="inlineStr">
@@ -23210,12 +23171,12 @@
       </c>
       <c r="C35" s="17" t="inlineStr">
         <is>
-          <t>Shortlisted</t>
+          <t>Shortlisted / Onboarding</t>
         </is>
       </c>
       <c r="D35" s="17" t="inlineStr">
         <is>
-          <t>Preliminarily eligible; onboarding started</t>
+          <t>Preliminary eligibility confirmed; scope and onboarding materials shared</t>
         </is>
       </c>
       <c r="E35" s="17" t="inlineStr">
@@ -23230,12 +23191,12 @@
       </c>
       <c r="G35" s="17" t="inlineStr">
         <is>
-          <t>Searches November 2026; 300–500 references; screening and extraction December 2026</t>
+          <t>Initial onboarding proposed for 28 September–2 October; searches expected in November</t>
         </is>
       </c>
       <c r="H35" s="17" t="inlineStr">
         <is>
-          <t>Scope and protocol shared; schedule onboarding with the PI and review team</t>
+          <t>Gerald approved onboarding; approximately 300–500 references expected; final eighth review under the current project</t>
         </is>
       </c>
       <c r="I35" s="17" t="inlineStr">
@@ -23425,8 +23386,6 @@
       <c r="H51" s="17" t="n"/>
       <c r="I51" s="17" t="n"/>
     </row>
-    <row r="52"/>
-    <row r="53"/>
     <row r="54">
       <c r="A54" s="31" t="inlineStr">
         <is>
@@ -26941,7 +26900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="14" customWidth="1" style="29" min="1" max="2"/>
@@ -27482,6 +27441,100 @@
         </is>
       </c>
       <c r="M9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>mtg-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>CESAR – Time-on-Task Analysis</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Review preliminary time-on-task analysis and agree next steps</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Amin Sharifan / Afroditi Kanellopoulou / Krishna</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Scheduled; Teams link needs adding</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>mtg-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Cochrane AI Platform Study – Adjudication Panel</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Weekly adjudication meetings through 29 October</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Adjudication Panel / Sean / Krishna</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Analysis / Adjudication</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -27538,7 +27591,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -27653,7 +27705,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abstract sets reconciled; full-text screening underway; missing PDFs remain</t>
+          <t>Abstract outputs reconciled; both full-text arms cleared to proceed; missing PDFs remain</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -27738,7 +27790,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>NK updated with the Covidence-only citations; some PDFs still need retrieval</t>
+          <t>NK updated with 16 Covidence-only citations; 14 AI-only citations were identified; both arms are aligned</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -27755,7 +27807,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Retrieve missing PDFs, complete both arms and record Bradley’s Covidence time</t>
+          <t>Retrieve missing PDFs, complete both full-text arms and record time</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -27789,7 +27841,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Reconciliation complete; missing-PDF retrieval remains</t>
+          <t>Meghan confirmed both arms are aligned and cleared to proceed; missing PDFs remain</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -27845,7 +27897,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -27854,7 +27906,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -27962,7 +28013,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -27977,7 +28028,6 @@
           <t>extraction</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -27990,14 +28040,12 @@
           <t>analysis</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -28081,12 +28129,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Citations aligned; missing PDFs remain</t>
+          <t>Citations consolidated; the review team still needs to retrieve missing PDFs</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -28183,7 +28231,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -28284,12 +28331,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Full-text lists reconciled; NK updated; missing PDFs require retrieval</t>
+          <t>Meghan confirmed both arms are aligned and cleared to proceed; missing PDFs remain</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -28315,7 +28362,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -29397,7 +29443,7 @@
       <c r="K67" s="18" t="n"/>
       <c r="L67" s="18" t="inlineStr">
         <is>
-          <t>NK title/abstract output obtained and compared with Covidence</t>
+          <t>NK and Covidence selections compared: 14 AI-only and 16 Covidence-only citations identified</t>
         </is>
       </c>
       <c r="M67" s="18" t="inlineStr">
@@ -29454,7 +29500,7 @@
       <c r="K68" s="18" t="n"/>
       <c r="L68" s="18" t="inlineStr">
         <is>
-          <t>Both screening lists shared and reconciled</t>
+          <t>Reconciled citation information shared with the project team</t>
         </is>
       </c>
       <c r="M68" s="18" t="inlineStr">
@@ -29776,7 +29822,7 @@
       <c r="K74" s="18" t="n"/>
       <c r="L74" s="18" t="inlineStr">
         <is>
-          <t>Common full-text pool prepared; missing PDFs still need retrieval</t>
+          <t>Both arms cleared; missing full-text PDFs still require retrieval</t>
         </is>
       </c>
       <c r="M74" s="18" t="inlineStr">
@@ -29833,7 +29879,7 @@
       <c r="K75" s="18" t="n"/>
       <c r="L75" s="18" t="inlineStr">
         <is>
-          <t>Missing full-text PDFs are being identified and retrieved</t>
+          <t>Missing PDFs are being identified and retrieved by the review team</t>
         </is>
       </c>
       <c r="M75" s="18" t="inlineStr">
@@ -29943,7 +29989,7 @@
       <c r="K77" s="18" t="n"/>
       <c r="L77" s="18" t="inlineStr">
         <is>
-          <t>Full-text comparison completed: 14 AI-only and 16 Covidence-only records</t>
+          <t>Meghan confirmed alignment and readiness of both full-text arms</t>
         </is>
       </c>
       <c r="M77" s="18" t="inlineStr">
@@ -30000,7 +30046,7 @@
       <c r="K78" s="18" t="n"/>
       <c r="L78" s="18" t="inlineStr">
         <is>
-          <t>NK updated with the 16 Covidence-only citations</t>
+          <t>Meghan confirmed alignment and readiness of both full-text arms</t>
         </is>
       </c>
       <c r="M78" s="18" t="inlineStr">
@@ -30057,7 +30103,7 @@
       <c r="K79" s="18" t="n"/>
       <c r="L79" s="18" t="inlineStr">
         <is>
-          <t>Reconciled citations are ready for full-text screening</t>
+          <t>Meghan confirmed alignment and readiness of both full-text arms</t>
         </is>
       </c>
       <c r="M79" s="18" t="inlineStr">
@@ -31766,7 +31812,6 @@
         </is>
       </c>
     </row>
-    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -31967,7 +32012,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>NK and Covidence outputs received and reconciled</t>
+          <t>NK and Covidence abstract outputs reconciled</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -31977,7 +32022,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -31999,7 +32044,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>Reconciliation complete; retrieve missing PDFs and finish both screening arms</t>
+          <t>Both arms cleared and screening underway; missing PDFs remain</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -32009,7 +32054,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -32018,7 +32063,6 @@
         </is>
       </c>
     </row>
-    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -32084,9 +32128,24 @@
           <t>comm-phase1-05-001</t>
         </is>
       </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Probiotics full-text screening cleared in both arms</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>One additional eligible review still needs to be identified or confirmed for Phase 1.</t>
+          <t>Meghan confirmed alignment of both arms; missing PDFs remain</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -32096,7 +32155,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>Identify additional eligible review</t>
+          <t>Retrieve missing PDFs and complete full-text screening</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -32110,7 +32169,6 @@
         </is>
       </c>
     </row>
-    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -32143,7 +32201,27 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Open Phase 1 review slot</t>
+          <t>Missing Probiotics full-text PDFs</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Next 1–2 weeks</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Citation sets are aligned and both arms are cleared, but missing PDFs remain</t>
         </is>
       </c>
     </row>
@@ -32187,7 +32265,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -32302,7 +32379,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Both abstract-screening arms complete; full-text consolidation underway</t>
+          <t>Both abstract arms complete; 74-study full-text set identified; reconciliation underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -32370,7 +32447,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Full-text setup and reconciliation underway</t>
+          <t>Mohan completed 2,024 AI-arm abstracts; AI selected 42 and the conventional arm selected 59</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -32387,7 +32464,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Conventional list revised to 58 references; AI arm completed 2,024 records</t>
+          <t>A 74-study combined set was identified; four conventional-only citations are absent from NK and one AI decision needs correction</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -32404,7 +32481,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Correct the final NK decision, consolidate both arms and begin full-text screening</t>
+          <t>Reconcile the full-text set, circulate the survey and begin both full-text arms</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -32438,7 +32515,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>One NK decision needs correction; final common full-text set is pending</t>
+          <t>Abstract screening complete; full-text reconciliation underway</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -32494,7 +32571,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -32503,7 +32580,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -32611,7 +32687,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -32626,7 +32702,6 @@
           <t>extraction</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -32639,14 +32714,12 @@
           <t>analysis</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -32730,12 +32803,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Revised 58-reference conventional list received; AI-only additions pending consolidation</t>
+          <t>Seventy-four studies identified; four conventional-only citations are absent from NK and one AI decision needs correction</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -32832,7 +32905,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -32926,7 +32998,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Both abstract-screening arms completed</t>
+          <t>Both abstract arms complete; Mohan screened all 2,024 NK records</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -32948,7 +33020,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Consolidate both arms’ selections and prepare the shared full-text set</t>
+          <t>Full-text set reconciliation underway; RIS and Excel files sent to the conventional team</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -32974,7 +33046,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -33417,12 +33488,16 @@
       </c>
       <c r="I55" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J55" s="18" t="n"/>
       <c r="K55" s="18" t="n"/>
-      <c r="L55" s="18" t="n"/>
+      <c r="L55" s="18" t="inlineStr">
+        <is>
+          <t>Mohan completed the AI-arm screening; conventional-team participation is confirmed</t>
+        </is>
+      </c>
       <c r="M55" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -33978,7 +34053,7 @@
       <c r="K65" s="18" t="n"/>
       <c r="L65" s="18" t="inlineStr">
         <is>
-          <t>Murali and Michelle completed conventional abstract screening</t>
+          <t>Conventional abstract screening complete; 59 records advanced</t>
         </is>
       </c>
       <c r="M65" s="18" t="inlineStr">
@@ -34035,7 +34110,7 @@
       <c r="K66" s="18" t="n"/>
       <c r="L66" s="18" t="inlineStr">
         <is>
-          <t>Mohan completed screening of 2,024 records</t>
+          <t>AI-assisted abstract screening complete; 42 records advanced</t>
         </is>
       </c>
       <c r="M66" s="18" t="inlineStr">
@@ -34085,14 +34160,14 @@
       </c>
       <c r="I67" s="18" t="inlineStr">
         <is>
-          <t>Needs Action</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J67" s="18" t="n"/>
       <c r="K67" s="18" t="n"/>
       <c r="L67" s="18" t="inlineStr">
         <is>
-          <t>Correct the final accidentally deleted record and export the AI decisions</t>
+          <t>AI-arm output exported; 16 records were unique to the AI arm</t>
         </is>
       </c>
       <c r="M67" s="18" t="inlineStr">
@@ -34142,14 +34217,14 @@
       </c>
       <c r="I68" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J68" s="18" t="n"/>
       <c r="K68" s="18" t="n"/>
       <c r="L68" s="18" t="inlineStr">
         <is>
-          <t>Combine the AI and conventional full-text selections</t>
+          <t>RIS and Excel files sent to Michelle and copied to the project team</t>
         </is>
       </c>
       <c r="M68" s="18" t="inlineStr">
@@ -34206,7 +34281,7 @@
       <c r="K69" s="18" t="n"/>
       <c r="L69" s="18" t="inlineStr">
         <is>
-          <t>Send the NK usability survey to the AI/NK reviewers, not the conventional reviewers</t>
+          <t>Abstract screening is complete; send the survey to Mohan</t>
         </is>
       </c>
       <c r="M69" s="18" t="inlineStr">
@@ -34468,14 +34543,14 @@
       </c>
       <c r="I74" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J74" s="18" t="n"/>
       <c r="K74" s="18" t="n"/>
       <c r="L74" s="18" t="inlineStr">
         <is>
-          <t>Revised conventional list contains 58 references; final union set pending</t>
+          <t>Combined 74-study full-text set being reconciled</t>
         </is>
       </c>
       <c r="M74" s="18" t="inlineStr">
@@ -34684,14 +34759,14 @@
       </c>
       <c r="I78" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J78" s="18" t="n"/>
       <c r="K78" s="18" t="n"/>
       <c r="L78" s="18" t="inlineStr">
         <is>
-          <t>Consolidate selections from both screening arms</t>
+          <t>Full-text project configuration underway</t>
         </is>
       </c>
       <c r="M78" s="18" t="inlineStr">
@@ -34741,14 +34816,14 @@
       </c>
       <c r="I79" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J79" s="18" t="n"/>
       <c r="K79" s="18" t="n"/>
       <c r="L79" s="18" t="inlineStr">
         <is>
-          <t>Validate the common full-text set after correcting the final NK decision</t>
+          <t>Validate the reconciled 74-study set before screening</t>
         </is>
       </c>
       <c r="M79" s="18" t="inlineStr">
@@ -34798,14 +34873,14 @@
       </c>
       <c r="I80" s="18" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J80" s="18" t="n"/>
       <c r="K80" s="18" t="n"/>
       <c r="L80" s="18" t="inlineStr">
         <is>
-          <t>Conventional reviewers may begin their 58 selections but must also screen later AI-only additions</t>
+          <t>Conventional records can be advanced after final reconciliation</t>
         </is>
       </c>
       <c r="M80" s="18" t="inlineStr">
@@ -34855,14 +34930,14 @@
       </c>
       <c r="I81" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J81" s="18" t="n"/>
       <c r="K81" s="18" t="n"/>
       <c r="L81" s="18" t="inlineStr">
         <is>
-          <t>Start after the combined full-text set is finalized</t>
+          <t>Add the four missing citations and correct the deleted AI decision</t>
         </is>
       </c>
       <c r="M81" s="18" t="inlineStr">
@@ -36457,7 +36532,6 @@
         </is>
       </c>
     </row>
-    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -36653,7 +36727,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Consolidate full-text selections and start screening</t>
+          <t>Reconcile the full-text set and begin full-text screening</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -36663,12 +36737,12 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>Final-decision correction and full-text-set consolidation</t>
+          <t>Full-text reconciliation</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Both arms completed; revised 58-reference list received; one NK decision requires correction</t>
+          <t>Abstract screening complete; reconcile the 74 studies, circulate the survey and begin full-text screening</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -36678,7 +36752,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -36714,7 +36788,6 @@
         </is>
       </c>
     </row>
-    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -36782,12 +36855,22 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Human Milk abstract screening complete; full-text consolidation underway</t>
+          <t>Human Milk abstract screening complete; full-text reconciliation underway</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Meghan / Michelle / Mohan / Krishna</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -36797,7 +36880,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Both arms completed; conventional list revised to 58; correct the final NK decision and prepare the union set</t>
+          <t>Both abstract arms complete; 74 studies identified; four citations and one screening decision need reconciliation</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -36807,7 +36890,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>Identify additional eligible review</t>
+          <t>Reconcile records, circulate the survey and begin full-text screening</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -36821,7 +36904,6 @@
         </is>
       </c>
     </row>
-    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -36854,7 +36936,22 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Open Phase 1 review slot</t>
+          <t>Reconcile the 74-study full-text set</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Meghan / Review Team / Krishna</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Resolve four missing NK citations and one deleted AI decision before finalizing the full-text set</t>
         </is>
       </c>
     </row>
@@ -36971,7 +37068,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
@@ -37032,7 +37128,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="28" customHeight="1" s="29">
       <c r="A16" s="19" t="inlineStr">
         <is>
@@ -37082,7 +37177,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -37197,7 +37291,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Expected reference count confirmed; available searches received</t>
+          <t>Latest searches uploaded; 16,891 citations deduplicated; decision-flow approval pending</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -37265,7 +37359,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Setup: final search upload and deduplication underway</t>
+          <t>The 14,743 baseline was confirmed; latest accessible searches increased the set to 16,891</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -37282,7 +37376,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Seven databases were inaccessible; all other search results were provided</t>
+          <t>All available searches supplied; seven databases were inaccessible; decision-flow syntax sent for approval</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -37299,7 +37393,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Upload and deduplicate the available results; document the seven inaccessible databases</t>
+          <t>Approve the decision flow, provide Laser AI access and document the inaccessible databases</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -37316,7 +37410,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Awaiting final upload and deduplication</t>
+          <t>Awaiting decision-flow approval</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -37333,7 +37427,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Count confirmed; final reference set pending incorporation of received searches</t>
+          <t>Final accessible reference set loaded; screening access pending approval</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -37350,7 +37444,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -37389,7 +37483,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -37398,7 +37492,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -37487,7 +37580,6 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -37500,7 +37592,6 @@
           <t>fullText</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -37513,7 +37604,6 @@
           <t>extraction</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -37526,14 +37616,12 @@
           <t>analysis</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -37595,12 +37683,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Expected count confirmed; available search results received; seven databases inaccessible</t>
+          <t>Latest accessible searches uploaded and deduplicated to 16,891; seven databases inaccessible</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -37639,12 +37727,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Decision-flow syntax sent on 22 September for review and approval</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -37719,7 +37807,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -37792,12 +37879,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Count confirmed; available searches awaiting upload and deduplication</t>
+          <t>Latest reference set contains 16,891 deduplicated citations; decision-flow approval and access remain pending</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -37875,7 +37962,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -38476,11 +38562,16 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J58" s="18" t="inlineStr"/>
       <c r="K58" s="18" t="inlineStr"/>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>All available search results received; seven databases were inaccessible</t>
+        </is>
+      </c>
       <c r="M58" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -38528,11 +38619,16 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J59" s="18" t="inlineStr"/>
       <c r="K59" s="18" t="inlineStr"/>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Protocol and criteria received; decision-flow syntax awaiting approval</t>
+        </is>
+      </c>
       <c r="M59" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -38736,14 +38832,14 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J63" s="18" t="inlineStr"/>
       <c r="K63" s="18" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Available search files received; seven database searches were unavailable</t>
+          <t>Latest uploads completed; 16,891 citations after deduplication</t>
         </is>
       </c>
       <c r="M63" s="18" t="inlineStr">
@@ -38800,7 +38896,7 @@
       <c r="K64" s="18" t="inlineStr"/>
       <c r="L64" s="18" t="inlineStr">
         <is>
-          <t>Expected 14,743 count confirmed; validate final count after upload and deduplication</t>
+          <t>Approve the decision flow before distributing citations and providing access</t>
         </is>
       </c>
       <c r="M64" s="18" t="inlineStr">
@@ -41296,7 +41392,6 @@
         </is>
       </c>
     </row>
-    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -41378,7 +41473,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Incorporate the available LNS search results</t>
+          <t>Approve LNS decision flow and provide Laser AI access</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -41398,17 +41493,17 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>After upload and deduplication</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Onboarding meeting</t>
+          <t>Decision-flow approval</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Count confirmed; all accessible results received; document seven inaccessible databases</t>
+          <t>Latest searches uploaded; 16,891 citations deduplicated; approval required before access is provided</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -41418,7 +41513,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -41427,10 +41522,6 @@
         </is>
       </c>
     </row>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -41522,12 +41613,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>LNS count confirmed; available searches received</t>
+          <t>LNS latest searches uploaded; decision-flow approval pending</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -41537,7 +41628,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Krishna</t>
+          <t>Syeda Kanza Naqvi / Jai Das / Meghan</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -41547,12 +41638,12 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>The count matches Covidence; available files need incorporation and deduplication</t>
+          <t>Baseline count confirmed; latest uploads produced 16,891 deduplicated citations; seven databases inaccessible</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -41562,7 +41653,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>Complete onboarding and confirm tool-training/setup plan</t>
+          <t>Approve the decision flow and provide Laser AI access</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -41576,7 +41667,6 @@
         </is>
       </c>
     </row>
-    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -41913,7 +42003,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Full Blood Pressure adjudication underway; first review folder opened</t>
+          <t>Extraction complete; adjudication and analysis underway</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -41933,17 +42023,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Analysis: full adjudication underway</t>
+          <t>Remaining-conflict rationales circulated; Bi 2025 omission documented</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Complete remaining adjudications, consolidate decisions and collect specific questions for senior reviewers</t>
+          <t>Consolidate Pilot 2 decisions, continue analysis and restore Paweł’s access to the shared files</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
         <is>
-          <t>Weekly through 2026-10-29</t>
+          <t>Preliminary results requested by end October</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -41985,7 +42075,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Corrective screening in progress; consolidated full-text package available</t>
+          <t>Analysis underway; corrective validation and final reconciliation in progress</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -42057,7 +42147,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Full-text screening underway; six-record model-limit exception open</t>
+          <t>Full-text screening underway; six oversized-PDF exceptions identified</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -42077,12 +42167,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Full-text screening underway</t>
+          <t>Kate distributed all 138 records; six oversized PDFs will be screened without model suggestions</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Resolve comparator handling for six oversized PDFs and complete both screening arms</t>
+          <t>Complete full-text screening and document the six model-suggestion exceptions</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -42340,7 +42430,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Abstract sets reconciled; full-text screening underway; missing PDFs remain</t>
+          <t>Abstract outputs reconciled; both full-text arms cleared to proceed; missing PDFs remain</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -42360,12 +42450,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Full-text screening underway</t>
+          <t>NK updated with Covidence-only citations; Meghan confirmed both arms are aligned</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Retrieve missing PDFs, complete both full-text arms and record Bradley’s time</t>
+          <t>Retrieve missing PDFs, complete both full-text arms and record time</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -42412,7 +42502,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Both abstract-screening arms complete; full-text consolidation underway</t>
+          <t>Both abstract arms complete; 74-study full-text set identified; reconciliation underway</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -42432,12 +42522,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Full-text setup and reconciliation underway</t>
+          <t>Mohan completed 2,024 NK records; four conventional-only citations are absent from NK and one AI decision needs correction</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Correct the final NK decision, consolidate both arms’ full-text selections and send the survey to the NK reviewers</t>
+          <t>Reconcile the full-text set, circulate the survey and begin both full-text arms</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -42484,7 +42574,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Expected 14,743-reference count confirmed; available searches received</t>
+          <t>Latest accessible searches uploaded; 16,891 citations deduplicated; decision-flow approval pending</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -42504,22 +42594,22 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Setup: final search upload and deduplication underway</t>
+          <t>The 14,743 baseline was confirmed; latest uploads increased the deduplicated set to 16,891</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Load and deduplicate the received searches, document inaccessible databases and finalize the screening set</t>
+          <t>Approve the decision flow, provide Laser AI access and document the seven inaccessible databases</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Awaiting final upload and deduplication</t>
+          <t>Awaiting decision-flow approval</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -46030,7 +46120,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -46117,7 +46206,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Current Focus</t>
+          <t>Focus on completing active reviews while onboarding the final Orthodontic Retention review</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -46144,7 +46233,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>All five extension groups consented; full adjudication underway; first BP review opened and one assessment completed</t>
+          <t>BP adjudication and analysis underway; CESAR analysis meetings scheduled; preliminary results targeted for the end of October</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -46171,7 +46260,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Broad Phase 2 deferred; CD002283 is onboarding as the eighth current-study topic</t>
+          <t>Deferred after Orthodontic Retention onboarding; no additional reviews currently planned</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -46207,8 +46296,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
@@ -46411,7 +46498,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Kate distributed 138 records; six PDFs exceed the 60-page model limit and require documented comparator handling</t>
+          <t>Fruit &amp; Vegetable full-text screening underway; six oversized PDFs will be screened without model suggestions</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -46420,8 +46507,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
@@ -46705,7 +46790,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -47016,7 +47100,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -47137,7 +47220,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -47323,7 +47405,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -47474,7 +47555,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -50889,7 +50969,6 @@
         </is>
       </c>
     </row>
-    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -51139,7 +51218,6 @@
         </is>
       </c>
     </row>
-    <row r="118"/>
     <row r="119">
       <c r="A119" s="5" t="inlineStr">
         <is>
@@ -51347,7 +51425,6 @@
         </is>
       </c>
     </row>
-    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -51478,7 +51555,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -51789,7 +51865,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -51910,7 +51985,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -52096,7 +52170,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -52247,7 +52320,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -55662,7 +55734,6 @@
         </is>
       </c>
     </row>
-    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -55850,7 +55921,6 @@
         </is>
       </c>
     </row>
-    <row r="117"/>
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
         <is>
@@ -55996,7 +56066,6 @@
         </is>
       </c>
     </row>
-    <row r="121"/>
     <row r="122">
       <c r="A122" s="5" t="inlineStr">
         <is>
@@ -56127,7 +56196,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -56242,7 +56310,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Full Blood Pressure adjudication underway</t>
+          <t>Extraction complete; adjudication and analysis underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -56310,7 +56378,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Analysis: full adjudication underway</t>
+          <t>Pilot 2 conflict resolution and analysis underway</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56327,7 +56395,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>First-review folder and spreadsheet shared; Bartosz completed his assessment</t>
+          <t>Andreea circulated rationales for the remaining conflicts; the Bi 2025 paper and supplements were re-shared</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56344,7 +56412,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete remaining assessments, consolidate decisions and collect focused senior-reviewer questions</t>
+          <t>Consolidate panel decisions, restore Paweł’s file access and prepare preliminary analysis</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56361,7 +56429,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Weekly through 2026-10-29</t>
+          <t>Preliminary results requested by end October</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -56378,7 +56446,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Full adjudication underway; shared senior-reviewer question document pending</t>
+          <t>Bi 2025 remains a documented limitation; Paweł reports that the shared links do not work</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -56434,7 +56502,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56443,7 +56511,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -56594,7 +56661,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -56780,7 +56846,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -56936,7 +57001,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -60082,12 +60146,16 @@
       </c>
       <c r="I106" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="J106" s="18" t="n"/>
       <c r="K106" s="18" t="n"/>
-      <c r="L106" s="18" t="n"/>
+      <c r="L106" s="18" t="inlineStr">
+        <is>
+          <t>Paweł reported that the shared links do not work; a fully automated analysis meeting is being arranged</t>
+        </is>
+      </c>
       <c r="M106" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -60195,7 +60263,7 @@
       <c r="K108" s="18" t="n"/>
       <c r="L108" s="18" t="inlineStr">
         <is>
-          <t>Weekly adjudication meetings scheduled through 29 October</t>
+          <t>Remaining-conflict rationales circulated; weekly adjudication continues through 29 October</t>
         </is>
       </c>
       <c r="M108" s="18" t="inlineStr">
@@ -60245,12 +60313,16 @@
       </c>
       <c r="I109" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Scheduled</t>
         </is>
       </c>
       <c r="J109" s="18" t="n"/>
       <c r="K109" s="18" t="n"/>
-      <c r="L109" s="18" t="n"/>
+      <c r="L109" s="18" t="inlineStr">
+        <is>
+          <t>Time-on-task analysis meeting scheduled for 28 September; preliminary results requested by end October</t>
+        </is>
+      </c>
       <c r="M109" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -60298,12 +60370,16 @@
       </c>
       <c r="I110" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Scheduling</t>
         </is>
       </c>
       <c r="J110" s="18" t="n"/>
       <c r="K110" s="18" t="n"/>
-      <c r="L110" s="18" t="n"/>
+      <c r="L110" s="18" t="inlineStr">
+        <is>
+          <t>Availability is being reconciled for the downstream-impact analysis meeting</t>
+        </is>
+      </c>
       <c r="M110" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -60359,7 +60435,6 @@
         </is>
       </c>
     </row>
-    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -60881,7 +60956,6 @@
     <row r="124" s="29"/>
     <row r="125" s="29"/>
     <row r="126" s="29"/>
-    <row r="127"/>
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
         <is>
@@ -61337,7 +61411,6 @@
     <row r="138" s="29"/>
     <row r="139" s="29"/>
     <row r="140" s="29"/>
-    <row r="141"/>
     <row r="142">
       <c r="A142" s="5" t="inlineStr">
         <is>
@@ -61537,7 +61610,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -61652,7 +61724,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Corrective screening in progress; consolidated platform package available</t>
+          <t>Analysis underway; corrective validation and final reconciliation in progress</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -61788,7 +61860,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Extension files are available; final validation still awaits the NK corrective decisions</t>
+          <t>Analysis active, but final outputs remain dependent on corrective NK screening and reconciliation</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -61844,7 +61916,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -61853,7 +61925,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -62004,7 +62075,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
@@ -62190,7 +62260,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -62361,7 +62430,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -65776,7 +65844,6 @@
         </is>
       </c>
     </row>
-    <row r="112"/>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
@@ -66348,7 +66415,6 @@
     <row r="124" s="29"/>
     <row r="125" s="29"/>
     <row r="126" s="29"/>
-    <row r="127"/>
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
         <is>
@@ -66917,7 +66983,6 @@
     </row>
     <row r="138" s="29"/>
     <row r="139" s="29"/>
-    <row r="140"/>
     <row r="141">
       <c r="A141" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update dashboard through September 30
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -17876,7 +17876,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Future batch planning</t>
+          <t>Not active; no Phase 2 under the current project</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -17910,7 +17910,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Keep placeholders until Phase 1 stabilizes.</t>
+          <t>No action; retain only for future standalone consideration</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -17927,7 +17927,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Not applicable</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -17944,7 +17944,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Phase 2 depends on Phase 1 stabilization and lessons learned.</t>
+          <t>Scope closed under the current project after the eighth review was onboarded</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -18000,7 +18000,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -21959,7 +21959,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Keep Phase 2 placeholder until Phase 1 stabilizes</t>
+          <t>Close Phase 2 under the current project</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -21969,27 +21969,27 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>After Phase 1</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Phase 1 lessons learned</t>
+          <t>Project scope decision</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Use Phase 1 lessons before scaling Phase 2.</t>
+          <t>No further AI-tool onboarding is planned; Orthodontic Retention is the final review</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -21999,7 +21999,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -22331,7 +22331,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Converted to phase1-07; both abstract arms complete and full-text reconciliation underway</t>
+          <t>Converted to phase1-07; abstract screening complete and the 77-reference full-text set approved</t>
         </is>
       </c>
       <c r="E12" s="17" t="inlineStr">
@@ -22346,12 +22346,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Full-text reconciliation underway</t>
+          <t>Full-text screening ready; target 31 October</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Seventy-four full-text studies identified; five record-level issues require reconciliation</t>
+          <t>Both arms will use 77 references; at least two conventional reviewers are required following Michelle’s withdrawal</t>
         </is>
       </c>
       <c r="I12" s="17" t="inlineStr">
@@ -22435,7 +22435,7 @@
       </c>
       <c r="D14" s="17" t="inlineStr">
         <is>
-          <t>Converted to phase1-08; latest uploads produced 16,891 deduplicated citations</t>
+          <t>Converted to phase1-08; decision flow approved and abstract screening ready</t>
         </is>
       </c>
       <c r="E14" s="17" t="inlineStr">
@@ -22446,12 +22446,12 @@
       <c r="F14" s="17" t="n"/>
       <c r="G14" s="17" t="inlineStr">
         <is>
-          <t>Awaiting decision-flow approval and Laser AI access</t>
+          <t>Ready for abstract screening</t>
         </is>
       </c>
       <c r="H14" s="17" t="inlineStr">
         <is>
-          <t>Baseline count confirmed; all accessible searches uploaded; seven databases inaccessible</t>
+          <t>16,891 citations loaded; team access and citation distribution enabled; seven inaccessible databases documented</t>
         </is>
       </c>
       <c r="I14" s="17" t="inlineStr">
@@ -23171,12 +23171,12 @@
       </c>
       <c r="C35" s="17" t="inlineStr">
         <is>
-          <t>Shortlisted / Onboarding</t>
+          <t>Onboarding</t>
         </is>
       </c>
       <c r="D35" s="17" t="inlineStr">
         <is>
-          <t>Preliminary eligibility confirmed; scope and onboarding materials shared</t>
+          <t>Initial onboarding completed; reviewer-allocation model awaiting confirmation</t>
         </is>
       </c>
       <c r="E35" s="17" t="inlineStr">
@@ -23186,17 +23186,17 @@
       </c>
       <c r="F35" s="17" t="inlineStr">
         <is>
-          <t>Álvaro Limones</t>
+          <t>Álvaro Limones / Concepción Martín Álvaro</t>
         </is>
       </c>
       <c r="G35" s="17" t="inlineStr">
         <is>
-          <t>Initial onboarding proposed for 28 September–2 October; searches expected in November</t>
+          <t>Initial onboarding completed; searches expected in November</t>
         </is>
       </c>
       <c r="H35" s="17" t="inlineStr">
         <is>
-          <t>Gerald approved onboarding; approximately 300–500 references expected; final eighth review under the current project</t>
+          <t>Crossed reviewer allocation proposed; Gerald’s approval is pending</t>
         </is>
       </c>
       <c r="I35" s="17" t="inlineStr">
@@ -27464,7 +27464,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Review preliminary time-on-task analysis and agree next steps</t>
+          <t>Time-on-task meeting held; BP and Psoriasis data confirmed and follow-up actions agreed</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -27484,7 +27484,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Scheduled; Teams link needs adding</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -27511,7 +27511,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Weekly adjudication meetings through 29 October</t>
+          <t>Recurring Thursday adjudication meetings through December; first review completed</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -32379,7 +32379,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Both abstract arms complete; 74-study full-text set identified; reconciliation underway</t>
+          <t>Abstract screening complete; reconciled 77-reference full-text set approved</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -32396,7 +32396,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -32447,7 +32447,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Mohan completed 2,024 AI-arm abstracts; AI selected 42 and the conventional arm selected 59</t>
+          <t>Both abstract arms complete; reconciled full-text set expanded to 77 references</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -32464,7 +32464,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>A 74-study combined set was identified; four conventional-only citations are absent from NK and one AI decision needs correction</t>
+          <t>Meghan cleared both arms to use the 77-reference set and will update Nested Knowledge</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -32481,7 +32481,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Reconcile the full-text set, circulate the survey and begin both full-text arms</t>
+          <t>Send the abstract survey, confirm at least two conventional reviewers and complete both full-text arms</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -32498,7 +32498,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Immediate</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -32515,7 +32515,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Abstract screening complete; full-text reconciliation underway</t>
+          <t>Full-text set finalized; NK update and conventional-reviewer coverage pending</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -32571,7 +32571,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -32687,7 +32687,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Ready / Under Review</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -32808,7 +32808,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Seventy-four studies identified; four conventional-only citations are absent from NK and one AI decision needs correction</t>
+          <t>Seventy-seven full-text references approved; PDF collection and NK updating remain</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -32891,12 +32891,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Michelle’s time report received; remaining reviewer time logs pending</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -33015,12 +33015,17 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Ready / Under Review</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Full-text set reconciliation underway; RIS and Excel files sent to the conventional team</t>
+          <t>Conventional arm can proceed; NK update pending for the AI arm; at least two conventional reviewers required</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -34543,14 +34548,14 @@
       </c>
       <c r="I74" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J74" s="18" t="n"/>
       <c r="K74" s="18" t="n"/>
       <c r="L74" s="18" t="inlineStr">
         <is>
-          <t>Combined 74-study full-text set being reconciled</t>
+          <t>Reconciled 77-reference full-text set approved</t>
         </is>
       </c>
       <c r="M74" s="18" t="inlineStr">
@@ -34759,14 +34764,14 @@
       </c>
       <c r="I78" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J78" s="18" t="n"/>
       <c r="K78" s="18" t="n"/>
       <c r="L78" s="18" t="inlineStr">
         <is>
-          <t>Full-text project configuration underway</t>
+          <t>Meghan will update Nested Knowledge to the 77-reference set</t>
         </is>
       </c>
       <c r="M78" s="18" t="inlineStr">
@@ -34823,7 +34828,7 @@
       <c r="K79" s="18" t="n"/>
       <c r="L79" s="18" t="inlineStr">
         <is>
-          <t>Validate the reconciled 74-study set before screening</t>
+          <t>Validate the 77-reference set after the NK update</t>
         </is>
       </c>
       <c r="M79" s="18" t="inlineStr">
@@ -34873,14 +34878,14 @@
       </c>
       <c r="I80" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="J80" s="18" t="n"/>
       <c r="K80" s="18" t="n"/>
       <c r="L80" s="18" t="inlineStr">
         <is>
-          <t>Conventional records can be advanced after final reconciliation</t>
+          <t>Conventional screening cleared for 77 references; confirm at least two reviewers</t>
         </is>
       </c>
       <c r="M80" s="18" t="inlineStr">
@@ -34937,7 +34942,7 @@
       <c r="K81" s="18" t="n"/>
       <c r="L81" s="18" t="inlineStr">
         <is>
-          <t>Add the four missing citations and correct the deleted AI decision</t>
+          <t>Update NK to the approved 77-reference set before AI full-text screening</t>
         </is>
       </c>
       <c r="M81" s="18" t="inlineStr">
@@ -36727,7 +36732,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Reconcile the full-text set and begin full-text screening</t>
+          <t>Complete full-text screening using the 77-reference set</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -36735,14 +36740,24 @@
           <t>In Progress</t>
         </is>
       </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>Full-text reconciliation</t>
+          <t>Full-text screening</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Abstract screening complete; reconcile the 74 studies, circulate the survey and begin full-text screening</t>
+          <t>Both arms cleared to use 77 references; send the survey and confirm conventional-reviewer coverage</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -36752,7 +36767,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -36855,22 +36870,22 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Human Milk abstract screening complete; full-text reconciliation underway</t>
+          <t>Human Milk 77-reference full-text set approved</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Meghan / Michelle / Mohan / Krishna</t>
+          <t>Meghan / Murali / Mohan / Krishna</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Immediate</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -36880,7 +36895,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Both abstract arms complete; 74 studies identified; four citations and one screening decision need reconciliation</t>
+          <t>Both arms will use 77 references; Michelle cannot continue screening and conventional-reviewer coverage must be confirmed</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -36890,7 +36905,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>Reconcile records, circulate the survey and begin full-text screening</t>
+          <t>Send the survey, confirm two conventional reviewers and complete full-text screening</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -36936,12 +36951,22 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Reconcile the 74-study full-text set</t>
+          <t>Complete full-text screening on the 77-reference set</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Meghan / Review Team / Krishna</t>
+          <t>Murali / Mohan / Meghan / Krishna</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -36951,7 +36976,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Resolve four missing NK citations and one deleted AI decision before finalizing the full-text set</t>
+          <t>Use the approved 77-reference set; confirm two conventional reviewers and document the source-set discrepancies</t>
         </is>
       </c>
     </row>
@@ -37291,7 +37316,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Latest searches uploaded; 16,891 citations deduplicated; decision-flow approval pending</t>
+          <t>Decision flow approved; Laser AI access provided; abstract screening ready to start</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -37376,7 +37401,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>All available searches supplied; seven databases were inaccessible; decision-flow syntax sent for approval</t>
+          <t>Kanza approved the decision flow; team members were added to Laser AI and citations can be distributed</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -37393,7 +37418,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Approve the decision flow, provide Laser AI access and document the inaccessible databases</t>
+          <t>Begin parallel abstract screening and record time</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -37410,7 +37435,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Awaiting decision-flow approval</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -37427,7 +37452,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Final accessible reference set loaded; screening access pending approval</t>
+          <t>Setup complete; reviewer distribution and screening commencement pending</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -37444,7 +37469,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -37483,7 +37508,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -37565,7 +37590,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -37578,6 +37603,11 @@
       <c r="A26" t="inlineStr">
         <is>
           <t>abstract</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Ready</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -37727,12 +37757,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Decision-flow syntax sent on 22 September for review and approval</t>
+          <t>Decision flow approved on 29 September</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -37879,12 +37909,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Latest reference set contains 16,891 deduplicated citations; decision-flow approval and access remain pending</t>
+          <t>Laser AI project ready with 16,891 citations; team access provided</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -37907,7 +37937,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Decision flow approved; citations ready for reviewer distribution</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -38619,14 +38654,14 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J59" s="18" t="inlineStr"/>
       <c r="K59" s="18" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>Protocol and criteria received; decision-flow syntax awaiting approval</t>
+          <t>Kanza approved the decision flow on 29 September</t>
         </is>
       </c>
       <c r="M59" s="18" t="inlineStr">
@@ -38832,14 +38867,14 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J63" s="18" t="inlineStr"/>
       <c r="K63" s="18" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Latest uploads completed; 16,891 citations after deduplication</t>
+          <t>All accessible searches uploaded; 16,891 citations after deduplication</t>
         </is>
       </c>
       <c r="M63" s="18" t="inlineStr">
@@ -38889,14 +38924,14 @@
       </c>
       <c r="I64" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J64" s="18" t="inlineStr"/>
       <c r="K64" s="18" t="inlineStr"/>
       <c r="L64" s="18" t="inlineStr">
         <is>
-          <t>Approve the decision flow before distributing citations and providing access</t>
+          <t>Decision flow approved; access provided and citations can be distributed</t>
         </is>
       </c>
       <c r="M64" s="18" t="inlineStr">
@@ -41473,7 +41508,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Approve LNS decision flow and provide Laser AI access</t>
+          <t>Begin LNS abstract screening and record time</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -41483,7 +41518,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -41498,12 +41533,12 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Decision-flow approval</t>
+          <t>Citation distribution</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Latest searches uploaded; 16,891 citations deduplicated; approval required before access is provided</t>
+          <t>Decision flow approved and Laser AI access provided; reviewers can claim citations from the open pool</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -41513,7 +41548,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -41613,12 +41648,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>LNS latest searches uploaded; decision-flow approval pending</t>
+          <t>LNS setup complete; abstract screening ready to start</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -41638,12 +41673,12 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Baseline count confirmed; latest uploads produced 16,891 deduplicated citations; seven databases inaccessible</t>
+          <t>Kanza approved the decision flow; team access and citation distribution enabled</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -41653,7 +41688,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>Approve the decision flow and provide Laser AI access</t>
+          <t>Begin parallel abstract screening and record time</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -42003,7 +42038,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Extraction complete; adjudication and analysis underway</t>
+          <t>Extraction and adjudication complete; analysis underway</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -42023,17 +42058,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Remaining-conflict rationales circulated; Bi 2025 omission documented</t>
+          <t>Pilot 2 completed, including conflict resolution; Bi 2025 omission remains documented</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Consolidate Pilot 2 decisions, continue analysis and restore Paweł’s access to the shared files</t>
+          <t>Complete the time-on-task, fully automated and downstream-impact analyses</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
         <is>
-          <t>Preliminary results requested by end October</t>
+          <t>December 2026</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -42095,7 +42130,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Analysis: corrective validation in progress</t>
+          <t>Updated decisions received for all 139 conventional records; 25 full texts are ready in NK; time-on-task data are available</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -42502,12 +42537,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Both abstract arms complete; 74-study full-text set identified; reconciliation underway</t>
+          <t>Abstract screening complete; reconciled 77-reference full-text set approved</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -42522,17 +42557,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Mohan completed 2,024 NK records; four conventional-only citations are absent from NK and one AI decision needs correction</t>
+          <t>Both arms will use the 77-reference set; the NK update and conventional-reviewer coverage remain pending</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Reconcile the full-text set, circulate the survey and begin both full-text arms</t>
+          <t>Send the abstract survey, confirm at least two conventional reviewers and complete full-text screening</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Immediate</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -42574,7 +42609,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Latest accessible searches uploaded; 16,891 citations deduplicated; decision-flow approval pending</t>
+          <t>Decision flow approved; Laser AI access provided; abstract screening ready to start</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -42594,22 +42629,22 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>The 14,743 baseline was confirmed; latest uploads increased the deduplicated set to 16,891</t>
+          <t>Kanza approved the decision flow; team members were added to Laser AI and citations can be distributed</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Approve the decision flow, provide Laser AI access and document the seven inaccessible databases</t>
+          <t>Begin parallel abstract screening and record time</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Awaiting decision-flow approval</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -46223,7 +46258,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Interim Analysis</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -46233,7 +46268,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>BP adjudication and analysis underway; CESAR analysis meetings scheduled; preliminary results targeted for the end of October</t>
+          <t>BP adjudication complete; time-on-task, automated and downstream-impact analyses underway; no interim report or mid-term review is planned</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -46255,12 +46290,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Start July to End September</t>
+          <t>Not planned under current project</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Deferred after Orthodontic Retention onboarding; no additional reviews currently planned</t>
+          <t>No Phase 2 under the current project; Orthodontic Retention is the final onboarded review</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -56310,7 +56345,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Extraction complete; adjudication and analysis underway</t>
+          <t>Extraction and adjudication complete; analysis underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -56378,7 +56413,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Pilot 2 conflict resolution and analysis underway</t>
+          <t>Pilot 2 completed, including conflict resolution; analysis underway</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56395,7 +56430,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Andreea circulated rationales for the remaining conflicts; the Bi 2025 paper and supplements were re-shared</t>
+          <t>Panel completed the first adjudication review, including conflict resolution; Bi 2025 remains documented</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56412,7 +56447,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Consolidate panel decisions, restore Paweł’s file access and prepare preliminary analysis</t>
+          <t>Complete the time-on-task, fully automated and downstream-impact analyses</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56429,7 +56464,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Preliminary results requested by end October</t>
+          <t>December 2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -56446,7 +56481,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Bi 2025 remains a documented limitation; Paweł reports that the shared links do not work</t>
+          <t>Bi 2025 remains documented; a direct invitation and Teams link were sent for the automated-analysis meeting</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -56502,7 +56537,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56837,7 +56872,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Time reports received; time-on-task analysis underway</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -56987,12 +57022,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Extraction complete; full adjudication underway</t>
+          <t>Extraction and adjudication complete; analysis underway</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>First BP adjudication review opened; one adjudicator completed; weekly meetings scheduled</t>
+          <t>BP adjudication completed; Bi 2025 retained as a documented source-file limitation</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -60036,14 +60071,14 @@
       </c>
       <c r="I104" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J104" s="18" t="n"/>
       <c r="K104" s="18" t="n"/>
       <c r="L104" s="18" t="inlineStr">
         <is>
-          <t>Full adjudication opened; first-review materials shared and one assessment completed</t>
+          <t>Panel completed adjudication, including conflict resolution, on 24 September</t>
         </is>
       </c>
       <c r="M104" s="18" t="inlineStr">
@@ -60146,14 +60181,14 @@
       </c>
       <c r="I106" s="18" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Scheduled</t>
         </is>
       </c>
       <c r="J106" s="18" t="n"/>
       <c r="K106" s="18" t="n"/>
       <c r="L106" s="18" t="inlineStr">
         <is>
-          <t>Paweł reported that the shared links do not work; a fully automated analysis meeting is being arranged</t>
+          <t>Fully automated analysis meeting scheduled for 1 October; direct invitation and Teams link sent</t>
         </is>
       </c>
       <c r="M106" s="18" t="inlineStr">
@@ -60256,14 +60291,14 @@
       </c>
       <c r="I108" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J108" s="18" t="n"/>
       <c r="K108" s="18" t="n"/>
       <c r="L108" s="18" t="inlineStr">
         <is>
-          <t>Remaining-conflict rationales circulated; weekly adjudication continues through 29 October</t>
+          <t>BP adjudication completed, including conflict resolution; recurring meetings remain for subsequent reviews</t>
         </is>
       </c>
       <c r="M108" s="18" t="inlineStr">
@@ -60313,14 +60348,14 @@
       </c>
       <c r="I109" s="18" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J109" s="18" t="n"/>
       <c r="K109" s="18" t="n"/>
       <c r="L109" s="18" t="inlineStr">
         <is>
-          <t>Time-on-task analysis meeting scheduled for 28 September; preliminary results requested by end October</t>
+          <t>Time-on-task meeting held on 28 September; BP and Psoriasis data received</t>
         </is>
       </c>
       <c r="M109" s="18" t="inlineStr">
@@ -60370,14 +60405,14 @@
       </c>
       <c r="I110" s="18" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduled</t>
         </is>
       </c>
       <c r="J110" s="18" t="n"/>
       <c r="K110" s="18" t="n"/>
       <c r="L110" s="18" t="inlineStr">
         <is>
-          <t>Availability is being reconciled for the downstream-impact analysis meeting</t>
+          <t>Downstream-impact analysis meeting scheduled for 2 October</t>
         </is>
       </c>
       <c r="M110" s="18" t="inlineStr">
@@ -61916,7 +61951,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -62251,7 +62286,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Conventional timing received: Emilie abstract 3h36m10s, full text 12h; Robin abstract 6h35m, full text 4h12m (corrected from 3h06m).</t>
+          <t>Screening times received: Laurence 5h30 abstract/4h10 full text; Sivem 5h05 abstract/4h40 full text; extraction times also available</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -65730,12 +65765,16 @@
       </c>
       <c r="I109" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J109" s="18" t="n"/>
       <c r="K109" s="18" t="n"/>
-      <c r="L109" s="18" t="n"/>
+      <c r="L109" s="18" t="inlineStr">
+        <is>
+          <t>Psoriasis time-on-task data received; analysis underway</t>
+        </is>
+      </c>
       <c r="M109" s="18" t="inlineStr">
         <is>
           <t>Yes</t>

</xml_diff>

<commit_message>
Add Orthodontic Retention review
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -26,6 +26,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-06 Probiotics" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-07 Human Milk" sheetId="19" state="visible" r:id="rId19"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-08 LNS" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="phase1-09 Orthodontic Retention" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -23171,12 +23172,12 @@
       </c>
       <c r="C35" s="17" t="inlineStr">
         <is>
-          <t>Onboarding</t>
+          <t>Converted to full sheet</t>
         </is>
       </c>
       <c r="D35" s="17" t="inlineStr">
         <is>
-          <t>Initial onboarding completed; reviewer-allocation model awaiting confirmation</t>
+          <t>Converted to phase1-09; initial onboarding completed and reviewer allocation awaiting confirmation</t>
         </is>
       </c>
       <c r="E35" s="17" t="inlineStr">
@@ -23191,22 +23192,22 @@
       </c>
       <c r="G35" s="17" t="inlineStr">
         <is>
-          <t>Initial onboarding completed; searches expected in November</t>
+          <t>Onboarding completed; searches expected in November and screening/data extraction planned for December</t>
         </is>
       </c>
       <c r="H35" s="17" t="inlineStr">
         <is>
-          <t>Crossed reviewer allocation proposed; Gerald’s approval is pending</t>
+          <t>Final eighth review; crossed reviewer allocation proposed and awaiting Gerald's confirmation</t>
         </is>
       </c>
       <c r="I35" s="17" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -41793,13 +41794,4732 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M130"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
+  <cols>
+    <col width="14" customWidth="1" style="29" min="1" max="1"/>
+    <col width="16" customWidth="1" style="29" min="2" max="2"/>
+    <col width="28" customWidth="1" style="29" min="3" max="3"/>
+    <col width="18" customWidth="1" style="29" min="4" max="4"/>
+    <col width="48" customWidth="1" style="29" min="5" max="5"/>
+    <col width="28" customWidth="1" style="29" min="6" max="6"/>
+    <col width="24" customWidth="1" style="29" min="7" max="8"/>
+    <col width="18" customWidth="1" style="29" min="9" max="10"/>
+    <col width="16" customWidth="1" style="29" min="11" max="11"/>
+    <col width="30" customWidth="1" style="29" min="12" max="12"/>
+    <col width="12" customWidth="1" style="29" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18" customHeight="1" s="29">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>phase1-08 LNS | Dashboard Content Sheet</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>phase1-09 Orthodontic Retention | Dashboard Content Sheet</t>
+        </is>
+      </c>
+      <c r="K1" s="18" t="n"/>
+      <c r="L1" s="18" t="n"/>
+      <c r="M1" s="18" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Executive Review Card</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n"/>
+      <c r="C3" s="5" t="n"/>
+      <c r="D3" s="5" t="n"/>
+      <c r="E3" s="5" t="n"/>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n"/>
+      <c r="I3" s="5" t="n"/>
+      <c r="J3" s="5" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Card Field</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ReviewID</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>phase1-09</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ShortName</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Orthodontic Retention</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ReviewTitle</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Retention procedures for stabilising tooth position after treatment with orthodontic braces</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Initial onboarding completed; reviewer-allocation model awaiting confirmation</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Tool</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Álvaro Limones / Concepción Martín Álvaro</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CurrentStage</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Approximately 300–500 references expected; searches planned for November</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CurrentUpdate</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Initial onboarding completed; crossed reviewer-allocation model proposed and awaiting Gerald's confirmation</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>NextAction</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Gerald to confirm the crossed reviewer allocation; then finalize team split, tool assignment and setup</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TargetDate</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>December 2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Variance</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Final eighth review; onboarding completed and setup depends on reviewer-allocation confirmation</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>DisplayInHTML</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Set to No if review should not appear in dashboard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>LastUpdated</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard Milestones</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="5" t="n"/>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="5" t="n"/>
+      <c r="G22" s="5" t="n"/>
+      <c r="H22" s="5" t="n"/>
+      <c r="I22" s="5" t="n"/>
+      <c r="J22" s="5" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="inlineStr">
+        <is>
+          <t>TargetDate</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="F23" s="1" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>onboarding</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>December 2026</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Initial onboarding completed; reviewer allocation awaiting Gerald confirmation</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>setup</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>December 2026</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Tool assignment and setup pending reviewer allocation</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>fullText</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>analysis</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Files Displayed in Review Detail</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n"/>
+      <c r="C31" s="5" t="n"/>
+      <c r="D31" s="5" t="n"/>
+      <c r="E31" s="5" t="n"/>
+      <c r="F31" s="5" t="n"/>
+      <c r="G31" s="5" t="n"/>
+      <c r="H31" s="5" t="n"/>
+      <c r="I31" s="5" t="n"/>
+      <c r="J31" s="5" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>FileType</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="C32" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D32" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E32" s="1" t="inlineStr">
+        <is>
+          <t>DueDate</t>
+        </is>
+      </c>
+      <c r="F32" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="G32" s="1" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>RIS</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Searches planned for November</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Approximately 300-500 references expected</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>PDFs</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Criteria</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Pending reviewer allocation</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Extraction</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Protocol</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Time Log</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Stage Progress: Visual Tracker / Operations</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n"/>
+      <c r="C40" s="5" t="n"/>
+      <c r="D40" s="5" t="n"/>
+      <c r="E40" s="5" t="n"/>
+      <c r="F40" s="5" t="n"/>
+      <c r="G40" s="5" t="n"/>
+      <c r="H40" s="5" t="n"/>
+      <c r="I40" s="5" t="n"/>
+      <c r="J40" s="5" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>StageName</t>
+        </is>
+      </c>
+      <c r="B41" s="1" t="inlineStr">
+        <is>
+          <t>HumanProgress</t>
+        </is>
+      </c>
+      <c r="C41" s="1" t="inlineStr">
+        <is>
+          <t>AIProgress</t>
+        </is>
+      </c>
+      <c r="D41" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E41" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F41" s="1" t="inlineStr">
+        <is>
+          <t>TargetDate</t>
+        </is>
+      </c>
+      <c r="G41" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="H41" s="1" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Setup / Coordination</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>December 2026</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Initial onboarding completed; reviewer allocation awaiting Gerald confirmation</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Abstract Screening</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Searches expected in November</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Full-text Screening</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Data Extraction / Analysis</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Review Workflow Status: Full 63 Actions</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n"/>
+      <c r="C47" s="5" t="n"/>
+      <c r="D47" s="5" t="n"/>
+      <c r="E47" s="5" t="n"/>
+      <c r="F47" s="5" t="n"/>
+      <c r="G47" s="5" t="n"/>
+      <c r="H47" s="5" t="n"/>
+      <c r="I47" s="5" t="n"/>
+      <c r="J47" s="5" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>ActionOrder</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>WorkflowStepID</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>WorkflowGroup</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>ShortName</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>Responsible</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>DependsOn</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>Blocks</t>
+        </is>
+      </c>
+      <c r="I48" s="6" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J48" s="6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="K48" s="10" t="inlineStr">
+        <is>
+          <t>DueDate</t>
+        </is>
+      </c>
+      <c r="L48" s="10" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="M48" s="10" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B49" s="18" t="inlineStr">
+        <is>
+          <t>w01</t>
+        </is>
+      </c>
+      <c r="C49" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D49" s="18" t="inlineStr">
+        <is>
+          <t>Review selected</t>
+        </is>
+      </c>
+      <c r="E49" s="18" t="inlineStr">
+        <is>
+          <t>Selection of review - core team</t>
+        </is>
+      </c>
+      <c r="F49" s="18" t="inlineStr">
+        <is>
+          <t>Core Team</t>
+        </is>
+      </c>
+      <c r="G49" s="18" t="n"/>
+      <c r="H49" s="18" t="inlineStr">
+        <is>
+          <t>w02</t>
+        </is>
+      </c>
+      <c r="I49" s="18" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="J49" s="18" t="n"/>
+      <c r="K49" s="18" t="n"/>
+      <c r="L49" s="18" t="n"/>
+      <c r="M49" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B50" s="18" t="inlineStr">
+        <is>
+          <t>w02</t>
+        </is>
+      </c>
+      <c r="C50" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D50" s="18" t="inlineStr">
+        <is>
+          <t>PM confirmation</t>
+        </is>
+      </c>
+      <c r="E50" s="18" t="inlineStr">
+        <is>
+          <t>Selection of review - project manager confirmation</t>
+        </is>
+      </c>
+      <c r="F50" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G50" s="18" t="inlineStr">
+        <is>
+          <t>w01</t>
+        </is>
+      </c>
+      <c r="H50" s="18" t="inlineStr">
+        <is>
+          <t>w03</t>
+        </is>
+      </c>
+      <c r="I50" s="18" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="J50" s="18" t="n"/>
+      <c r="K50" s="18" t="n"/>
+      <c r="L50" s="18" t="n"/>
+      <c r="M50" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B51" s="18" t="inlineStr">
+        <is>
+          <t>w03</t>
+        </is>
+      </c>
+      <c r="C51" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D51" s="18" t="inlineStr">
+        <is>
+          <t>Final confirmation</t>
+        </is>
+      </c>
+      <c r="E51" s="18" t="inlineStr">
+        <is>
+          <t>Selection of review - final confirmation</t>
+        </is>
+      </c>
+      <c r="F51" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G51" s="18" t="inlineStr">
+        <is>
+          <t>w02</t>
+        </is>
+      </c>
+      <c r="H51" s="18" t="inlineStr">
+        <is>
+          <t>w04</t>
+        </is>
+      </c>
+      <c r="I51" s="18" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="J51" s="18" t="n"/>
+      <c r="K51" s="18" t="n"/>
+      <c r="L51" s="18" t="n"/>
+      <c r="M51" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B52" s="18" t="inlineStr">
+        <is>
+          <t>w04</t>
+        </is>
+      </c>
+      <c r="C52" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D52" s="18" t="inlineStr">
+        <is>
+          <t>Tool allocated</t>
+        </is>
+      </c>
+      <c r="E52" s="18" t="inlineStr">
+        <is>
+          <t>Confirm allocated AI tool for review</t>
+        </is>
+      </c>
+      <c r="F52" s="18" t="inlineStr">
+        <is>
+          <t>Core Team</t>
+        </is>
+      </c>
+      <c r="G52" s="18" t="inlineStr">
+        <is>
+          <t>w03</t>
+        </is>
+      </c>
+      <c r="H52" s="18" t="inlineStr">
+        <is>
+          <t>w05,w07,w15,w30,w45</t>
+        </is>
+      </c>
+      <c r="I52" s="18" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J52" s="18" t="n"/>
+      <c r="K52" s="18" t="n"/>
+      <c r="L52" s="18" t="inlineStr">
+        <is>
+          <t>Tool allocation to be confirmed after onboarding.</t>
+        </is>
+      </c>
+      <c r="M52" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="28" customHeight="1" s="29">
+      <c r="A53" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B53" s="18" t="inlineStr">
+        <is>
+          <t>w05</t>
+        </is>
+      </c>
+      <c r="C53" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D53" s="18" t="inlineStr">
+        <is>
+          <t>Team split</t>
+        </is>
+      </c>
+      <c r="E53" s="18" t="inlineStr">
+        <is>
+          <t>Confirm review team split: Human workflow and AI-assisted workflow</t>
+        </is>
+      </c>
+      <c r="F53" s="18" t="inlineStr">
+        <is>
+          <t>Krishna / Review Team</t>
+        </is>
+      </c>
+      <c r="G53" s="18" t="inlineStr">
+        <is>
+          <t>w04</t>
+        </is>
+      </c>
+      <c r="H53" s="18" t="inlineStr">
+        <is>
+          <t>w08,w09,w17,w32,w47</t>
+        </is>
+      </c>
+      <c r="I53" s="18" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J53" s="18" t="n"/>
+      <c r="K53" s="18" t="n"/>
+      <c r="L53" s="18" t="inlineStr"/>
+      <c r="M53" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="B54" s="18" t="inlineStr">
+        <is>
+          <t>w06</t>
+        </is>
+      </c>
+      <c r="C54" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D54" s="18" t="inlineStr">
+        <is>
+          <t>Folder access</t>
+        </is>
+      </c>
+      <c r="E54" s="18" t="inlineStr">
+        <is>
+          <t>Confirm SharePoint/folder access for review team</t>
+        </is>
+      </c>
+      <c r="F54" s="18" t="inlineStr">
+        <is>
+          <t>Krishna / Review Team</t>
+        </is>
+      </c>
+      <c r="G54" s="18" t="inlineStr">
+        <is>
+          <t>w03</t>
+        </is>
+      </c>
+      <c r="H54" s="18" t="inlineStr">
+        <is>
+          <t>w10,w11,w12</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J54" s="18" t="n"/>
+      <c r="K54" s="18" t="n"/>
+      <c r="M54" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="28" customHeight="1" s="29">
+      <c r="A55" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="B55" s="18" t="inlineStr">
+        <is>
+          <t>w07</t>
+        </is>
+      </c>
+      <c r="C55" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D55" s="18" t="inlineStr">
+        <is>
+          <t>Tool access</t>
+        </is>
+      </c>
+      <c r="E55" s="18" t="inlineStr">
+        <is>
+          <t>Confirm AI tool access for allocated users</t>
+        </is>
+      </c>
+      <c r="F55" s="18" t="inlineStr">
+        <is>
+          <t>Response Team / Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G55" s="18" t="inlineStr">
+        <is>
+          <t>w04</t>
+        </is>
+      </c>
+      <c r="H55" s="18" t="inlineStr">
+        <is>
+          <t>w15,w30,w45</t>
+        </is>
+      </c>
+      <c r="I55" s="18" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J55" s="18" t="n"/>
+      <c r="K55" s="18" t="n"/>
+      <c r="L55" s="18" t="inlineStr"/>
+      <c r="M55" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="B56" s="18" t="inlineStr">
+        <is>
+          <t>w08</t>
+        </is>
+      </c>
+      <c r="C56" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D56" s="18" t="inlineStr">
+        <is>
+          <t>Blinding shared</t>
+        </is>
+      </c>
+      <c r="E56" s="18" t="inlineStr">
+        <is>
+          <t>Confirm blinding instructions shared with review teams</t>
+        </is>
+      </c>
+      <c r="F56" s="18" t="inlineStr">
+        <is>
+          <t>Krishna / Sean</t>
+        </is>
+      </c>
+      <c r="G56" s="18" t="inlineStr">
+        <is>
+          <t>w05</t>
+        </is>
+      </c>
+      <c r="H56" s="18" t="inlineStr">
+        <is>
+          <t>w17,w18,w32,w33,w47,w48</t>
+        </is>
+      </c>
+      <c r="I56" s="18" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J56" s="18" t="n"/>
+      <c r="K56" s="18" t="n"/>
+      <c r="L56" s="18" t="inlineStr"/>
+      <c r="M56" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="B57" s="18" t="inlineStr">
+        <is>
+          <t>w09</t>
+        </is>
+      </c>
+      <c r="C57" s="18" t="inlineStr">
+        <is>
+          <t>Review selection and onboarding</t>
+        </is>
+      </c>
+      <c r="D57" s="18" t="inlineStr">
+        <is>
+          <t>Time tracking</t>
+        </is>
+      </c>
+      <c r="E57" s="18" t="inlineStr">
+        <is>
+          <t>Confirm Clockify or alternate time-tracking setup</t>
+        </is>
+      </c>
+      <c r="F57" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G57" s="18" t="inlineStr">
+        <is>
+          <t>w05</t>
+        </is>
+      </c>
+      <c r="H57" s="18" t="inlineStr">
+        <is>
+          <t>w17,w18,w32,w33,w47,w48</t>
+        </is>
+      </c>
+      <c r="I57" s="18" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J57" s="18" t="n"/>
+      <c r="K57" s="18" t="n"/>
+      <c r="L57" s="18" t="inlineStr"/>
+      <c r="M57" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="28" customHeight="1" s="29">
+      <c r="A58" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="B58" s="18" t="inlineStr">
+        <is>
+          <t>w10</t>
+        </is>
+      </c>
+      <c r="C58" s="18" t="inlineStr">
+        <is>
+          <t>Setup package and data item readiness</t>
+        </is>
+      </c>
+      <c r="D58" s="18" t="inlineStr">
+        <is>
+          <t>RIS files</t>
+        </is>
+      </c>
+      <c r="E58" s="18" t="inlineStr">
+        <is>
+          <t>Review team to share RIS files with setup team</t>
+        </is>
+      </c>
+      <c r="F58" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G58" s="18" t="inlineStr">
+        <is>
+          <t>w06</t>
+        </is>
+      </c>
+      <c r="H58" s="18" t="inlineStr">
+        <is>
+          <t>w15</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J58" s="18" t="n"/>
+      <c r="K58" s="18" t="n"/>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>All available search results received; seven databases were inaccessible</t>
+        </is>
+      </c>
+      <c r="M58" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="28" customHeight="1" s="29">
+      <c r="A59" s="18" t="n">
+        <v>11</v>
+      </c>
+      <c r="B59" s="18" t="inlineStr">
+        <is>
+          <t>w11</t>
+        </is>
+      </c>
+      <c r="C59" s="18" t="inlineStr">
+        <is>
+          <t>Setup package and data item readiness</t>
+        </is>
+      </c>
+      <c r="D59" s="18" t="inlineStr">
+        <is>
+          <t>Protocol &amp; criteria</t>
+        </is>
+      </c>
+      <c r="E59" s="18" t="inlineStr">
+        <is>
+          <t>Review team to share protocol and inclusion/exclusion criteria</t>
+        </is>
+      </c>
+      <c r="F59" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G59" s="18" t="inlineStr">
+        <is>
+          <t>w06</t>
+        </is>
+      </c>
+      <c r="H59" s="18" t="inlineStr">
+        <is>
+          <t>w12,w15,w29</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J59" s="18" t="n"/>
+      <c r="K59" s="18" t="n"/>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Kanza approved the decision flow on 29 September</t>
+        </is>
+      </c>
+      <c r="M59" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="28" customHeight="1" s="29">
+      <c r="A60" s="18" t="n">
+        <v>12</v>
+      </c>
+      <c r="B60" s="18" t="inlineStr">
+        <is>
+          <t>w12</t>
+        </is>
+      </c>
+      <c r="C60" s="18" t="inlineStr">
+        <is>
+          <t>Setup package and data item readiness</t>
+        </is>
+      </c>
+      <c r="D60" s="18" t="inlineStr">
+        <is>
+          <t>Data items</t>
+        </is>
+      </c>
+      <c r="E60" s="18" t="inlineStr">
+        <is>
+          <t>Finalise data items with Sean</t>
+        </is>
+      </c>
+      <c r="F60" s="18" t="inlineStr">
+        <is>
+          <t>Review Team / Sean</t>
+        </is>
+      </c>
+      <c r="G60" s="18" t="inlineStr">
+        <is>
+          <t>w11</t>
+        </is>
+      </c>
+      <c r="H60" s="18" t="inlineStr">
+        <is>
+          <t>w13,w14,w43,w44</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J60" s="18" t="n"/>
+      <c r="K60" s="18" t="n"/>
+      <c r="M60" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="28" customHeight="1" s="29">
+      <c r="A61" s="18" t="n">
+        <v>13</v>
+      </c>
+      <c r="B61" s="18" t="inlineStr">
+        <is>
+          <t>w13</t>
+        </is>
+      </c>
+      <c r="C61" s="18" t="inlineStr">
+        <is>
+          <t>Setup package and data item readiness</t>
+        </is>
+      </c>
+      <c r="D61" s="18" t="inlineStr">
+        <is>
+          <t>Comparable DE</t>
+        </is>
+      </c>
+      <c r="E61" s="18" t="inlineStr">
+        <is>
+          <t>Confirm data extraction structure is comparable between Human and AI workflows</t>
+        </is>
+      </c>
+      <c r="F61" s="18" t="inlineStr">
+        <is>
+          <t>Review Team / Sean</t>
+        </is>
+      </c>
+      <c r="G61" s="18" t="inlineStr">
+        <is>
+          <t>w12</t>
+        </is>
+      </c>
+      <c r="H61" s="18" t="inlineStr">
+        <is>
+          <t>w14,w44</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J61" s="18" t="n"/>
+      <c r="K61" s="18" t="n"/>
+      <c r="M61" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="28" customHeight="1" s="29">
+      <c r="A62" s="18" t="n">
+        <v>14</v>
+      </c>
+      <c r="B62" s="18" t="inlineStr">
+        <is>
+          <t>w14</t>
+        </is>
+      </c>
+      <c r="C62" s="18" t="inlineStr">
+        <is>
+          <t>Setup package and data item readiness</t>
+        </is>
+      </c>
+      <c r="D62" s="18" t="inlineStr">
+        <is>
+          <t>Sean approval</t>
+        </is>
+      </c>
+      <c r="E62" s="18" t="inlineStr">
+        <is>
+          <t>Confirm extraction form/template is approved by Sean</t>
+        </is>
+      </c>
+      <c r="F62" s="18" t="inlineStr">
+        <is>
+          <t>Sean</t>
+        </is>
+      </c>
+      <c r="G62" s="18" t="inlineStr">
+        <is>
+          <t>w13</t>
+        </is>
+      </c>
+      <c r="H62" s="18" t="inlineStr">
+        <is>
+          <t>w43,w44,w45</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J62" s="18" t="n"/>
+      <c r="K62" s="18" t="n"/>
+      <c r="M62" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="28" customHeight="1" s="29">
+      <c r="A63" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="B63" s="18" t="inlineStr">
+        <is>
+          <t>w15</t>
+        </is>
+      </c>
+      <c r="C63" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D63" s="18" t="inlineStr">
+        <is>
+          <t>Tool setup</t>
+        </is>
+      </c>
+      <c r="E63" s="18" t="inlineStr">
+        <is>
+          <t>Tool setup - allocated AI tool for abstract screening</t>
+        </is>
+      </c>
+      <c r="F63" s="18" t="inlineStr">
+        <is>
+          <t>Response Team / Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G63" s="18" t="inlineStr">
+        <is>
+          <t>w04,w07,w10,w11</t>
+        </is>
+      </c>
+      <c r="H63" s="18" t="inlineStr">
+        <is>
+          <t>w16</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J63" s="18" t="n"/>
+      <c r="K63" s="18" t="n"/>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>All accessible searches uploaded; 16,891 citations after deduplication</t>
+        </is>
+      </c>
+      <c r="M63" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="28" customHeight="1" s="29">
+      <c r="A64" s="18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B64" s="18" t="inlineStr">
+        <is>
+          <t>w16</t>
+        </is>
+      </c>
+      <c r="C64" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D64" s="18" t="inlineStr">
+        <is>
+          <t>Setup validated</t>
+        </is>
+      </c>
+      <c r="E64" s="18" t="inlineStr">
+        <is>
+          <t>Review team validates abstract screening setup before starting</t>
+        </is>
+      </c>
+      <c r="F64" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G64" s="18" t="inlineStr">
+        <is>
+          <t>w15</t>
+        </is>
+      </c>
+      <c r="H64" s="18" t="inlineStr">
+        <is>
+          <t>w17,w18</t>
+        </is>
+      </c>
+      <c r="I64" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J64" s="18" t="n"/>
+      <c r="K64" s="18" t="n"/>
+      <c r="L64" s="18" t="inlineStr">
+        <is>
+          <t>Decision flow approved; access provided and citations can be distributed</t>
+        </is>
+      </c>
+      <c r="M64" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B65" s="18" t="inlineStr">
+        <is>
+          <t>w17</t>
+        </is>
+      </c>
+      <c r="C65" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D65" s="18" t="inlineStr">
+        <is>
+          <t>Human screening</t>
+        </is>
+      </c>
+      <c r="E65" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening - Human workflow</t>
+        </is>
+      </c>
+      <c r="F65" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G65" s="18" t="inlineStr">
+        <is>
+          <t>w05,w08,w09,w16</t>
+        </is>
+      </c>
+      <c r="H65" s="18" t="inlineStr">
+        <is>
+          <t>w21,w24,w25</t>
+        </is>
+      </c>
+      <c r="I65" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J65" s="18" t="n"/>
+      <c r="K65" s="18" t="n"/>
+      <c r="L65" s="18" t="inlineStr"/>
+      <c r="M65" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="18" t="n">
+        <v>18</v>
+      </c>
+      <c r="B66" s="18" t="inlineStr">
+        <is>
+          <t>w18</t>
+        </is>
+      </c>
+      <c r="C66" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D66" s="18" t="inlineStr">
+        <is>
+          <t>AI screening</t>
+        </is>
+      </c>
+      <c r="E66" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening - allocated AI tool</t>
+        </is>
+      </c>
+      <c r="F66" s="18" t="inlineStr">
+        <is>
+          <t>Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G66" s="18" t="inlineStr">
+        <is>
+          <t>w07,w08,w09,w16</t>
+        </is>
+      </c>
+      <c r="H66" s="18" t="inlineStr">
+        <is>
+          <t>w19,w21,w24,w25</t>
+        </is>
+      </c>
+      <c r="I66" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J66" s="18" t="n"/>
+      <c r="K66" s="18" t="n"/>
+      <c r="L66" s="18" t="inlineStr"/>
+      <c r="M66" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="18" t="n">
+        <v>19</v>
+      </c>
+      <c r="B67" s="18" t="inlineStr">
+        <is>
+          <t>w19</t>
+        </is>
+      </c>
+      <c r="C67" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D67" s="18" t="inlineStr">
+        <is>
+          <t>Export AI output</t>
+        </is>
+      </c>
+      <c r="E67" s="18" t="inlineStr">
+        <is>
+          <t>Export abstract screening output from allocated AI tool</t>
+        </is>
+      </c>
+      <c r="F67" s="18" t="inlineStr">
+        <is>
+          <t>Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G67" s="18" t="inlineStr">
+        <is>
+          <t>w18</t>
+        </is>
+      </c>
+      <c r="H67" s="18" t="inlineStr">
+        <is>
+          <t>w20</t>
+        </is>
+      </c>
+      <c r="I67" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J67" s="18" t="n"/>
+      <c r="K67" s="18" t="n"/>
+      <c r="L67" s="18" t="inlineStr"/>
+      <c r="M67" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="18" t="n">
+        <v>20</v>
+      </c>
+      <c r="B68" s="18" t="inlineStr">
+        <is>
+          <t>w20</t>
+        </is>
+      </c>
+      <c r="C68" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D68" s="18" t="inlineStr">
+        <is>
+          <t>Share output</t>
+        </is>
+      </c>
+      <c r="E68" s="18" t="inlineStr">
+        <is>
+          <t>Share abstract screening output with Sean / data manager</t>
+        </is>
+      </c>
+      <c r="F68" s="18" t="inlineStr">
+        <is>
+          <t>Krishna / Data Manager</t>
+        </is>
+      </c>
+      <c r="G68" s="18" t="inlineStr">
+        <is>
+          <t>w19</t>
+        </is>
+      </c>
+      <c r="H68" s="18" t="inlineStr">
+        <is>
+          <t>w24,w25</t>
+        </is>
+      </c>
+      <c r="I68" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J68" s="18" t="n"/>
+      <c r="K68" s="18" t="n"/>
+      <c r="L68" s="18" t="inlineStr"/>
+      <c r="M68" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="18" t="n">
+        <v>21</v>
+      </c>
+      <c r="B69" s="18" t="inlineStr">
+        <is>
+          <t>w21</t>
+        </is>
+      </c>
+      <c r="C69" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D69" s="18" t="inlineStr">
+        <is>
+          <t>Survey sent</t>
+        </is>
+      </c>
+      <c r="E69" s="18" t="inlineStr">
+        <is>
+          <t>Share usability survey on abstract screening experience</t>
+        </is>
+      </c>
+      <c r="F69" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G69" s="18" t="inlineStr">
+        <is>
+          <t>w17,w18</t>
+        </is>
+      </c>
+      <c r="H69" s="18" t="inlineStr">
+        <is>
+          <t>w22</t>
+        </is>
+      </c>
+      <c r="I69" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J69" s="18" t="n"/>
+      <c r="K69" s="18" t="n"/>
+      <c r="L69" s="18" t="inlineStr"/>
+      <c r="M69" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="18" t="n">
+        <v>22</v>
+      </c>
+      <c r="B70" s="18" t="inlineStr">
+        <is>
+          <t>w22</t>
+        </is>
+      </c>
+      <c r="C70" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D70" s="18" t="inlineStr">
+        <is>
+          <t>Survey submitted</t>
+        </is>
+      </c>
+      <c r="E70" s="18" t="inlineStr">
+        <is>
+          <t>Submit usability survey on abstract screening experience</t>
+        </is>
+      </c>
+      <c r="F70" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G70" s="18" t="inlineStr">
+        <is>
+          <t>w21</t>
+        </is>
+      </c>
+      <c r="H70" s="18" t="inlineStr">
+        <is>
+          <t>w23</t>
+        </is>
+      </c>
+      <c r="I70" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J70" s="18" t="n"/>
+      <c r="K70" s="18" t="n"/>
+      <c r="L70" s="18" t="inlineStr"/>
+      <c r="M70" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="28" customHeight="1" s="29">
+      <c r="A71" s="18" t="n">
+        <v>23</v>
+      </c>
+      <c r="B71" s="18" t="inlineStr">
+        <is>
+          <t>w23</t>
+        </is>
+      </c>
+      <c r="C71" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D71" s="18" t="inlineStr">
+        <is>
+          <t>Survey received</t>
+        </is>
+      </c>
+      <c r="E71" s="18" t="inlineStr">
+        <is>
+          <t>Confirm usability survey responses received for abstract screening</t>
+        </is>
+      </c>
+      <c r="F71" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G71" s="18" t="inlineStr">
+        <is>
+          <t>w22</t>
+        </is>
+      </c>
+      <c r="H71" s="18" t="inlineStr">
+        <is>
+          <t>w24</t>
+        </is>
+      </c>
+      <c r="I71" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J71" s="18" t="n"/>
+      <c r="K71" s="18" t="n"/>
+      <c r="L71" s="18" t="inlineStr"/>
+      <c r="M71" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="28" customHeight="1" s="29">
+      <c r="A72" s="18" t="n">
+        <v>24</v>
+      </c>
+      <c r="B72" s="18" t="inlineStr">
+        <is>
+          <t>w24</t>
+        </is>
+      </c>
+      <c r="C72" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D72" s="18" t="inlineStr">
+        <is>
+          <t>Quality check</t>
+        </is>
+      </c>
+      <c r="E72" s="18" t="inlineStr">
+        <is>
+          <t>Data completeness and quality check before abstract screening adjudication</t>
+        </is>
+      </c>
+      <c r="F72" s="18" t="inlineStr">
+        <is>
+          <t>Data Manager / Sean</t>
+        </is>
+      </c>
+      <c r="G72" s="18" t="inlineStr">
+        <is>
+          <t>w20,w23</t>
+        </is>
+      </c>
+      <c r="H72" s="18" t="inlineStr">
+        <is>
+          <t>w25</t>
+        </is>
+      </c>
+      <c r="I72" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J72" s="18" t="n"/>
+      <c r="K72" s="18" t="n"/>
+      <c r="L72" s="18" t="inlineStr"/>
+      <c r="M72" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="18" t="n">
+        <v>25</v>
+      </c>
+      <c r="B73" s="18" t="inlineStr">
+        <is>
+          <t>w25</t>
+        </is>
+      </c>
+      <c r="C73" s="18" t="inlineStr">
+        <is>
+          <t>Abstract screening</t>
+        </is>
+      </c>
+      <c r="D73" s="18" t="inlineStr">
+        <is>
+          <t>Abstract adjudication</t>
+        </is>
+      </c>
+      <c r="E73" s="18" t="inlineStr">
+        <is>
+          <t>Adjudication panel after abstract screening</t>
+        </is>
+      </c>
+      <c r="F73" s="18" t="inlineStr">
+        <is>
+          <t>Sean and Adjudication Panel</t>
+        </is>
+      </c>
+      <c r="G73" s="18" t="inlineStr">
+        <is>
+          <t>w24</t>
+        </is>
+      </c>
+      <c r="H73" s="18" t="inlineStr">
+        <is>
+          <t>w26,w28,w30</t>
+        </is>
+      </c>
+      <c r="I73" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J73" s="18" t="n"/>
+      <c r="K73" s="18" t="n"/>
+      <c r="L73" s="18" t="inlineStr"/>
+      <c r="M73" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="18" t="n">
+        <v>26</v>
+      </c>
+      <c r="B74" s="18" t="inlineStr">
+        <is>
+          <t>w26</t>
+        </is>
+      </c>
+      <c r="C74" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D74" s="18" t="inlineStr">
+        <is>
+          <t>PDFs received</t>
+        </is>
+      </c>
+      <c r="E74" s="18" t="inlineStr">
+        <is>
+          <t>Review team to share PDF files with setup team</t>
+        </is>
+      </c>
+      <c r="F74" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G74" s="18" t="inlineStr">
+        <is>
+          <t>w25</t>
+        </is>
+      </c>
+      <c r="H74" s="18" t="inlineStr">
+        <is>
+          <t>w27,w29</t>
+        </is>
+      </c>
+      <c r="I74" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J74" s="18" t="n"/>
+      <c r="K74" s="18" t="n"/>
+      <c r="L74" s="18" t="inlineStr"/>
+      <c r="M74" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="18" t="n">
+        <v>27</v>
+      </c>
+      <c r="B75" s="18" t="inlineStr">
+        <is>
+          <t>w27</t>
+        </is>
+      </c>
+      <c r="C75" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D75" s="18" t="inlineStr">
+        <is>
+          <t>PDF issues logged</t>
+        </is>
+      </c>
+      <c r="E75" s="18" t="inlineStr">
+        <is>
+          <t>Confirm unavailable PDFs or access issues are logged</t>
+        </is>
+      </c>
+      <c r="F75" s="18" t="inlineStr">
+        <is>
+          <t>Review Team / Krishna</t>
+        </is>
+      </c>
+      <c r="G75" s="18" t="inlineStr">
+        <is>
+          <t>w26</t>
+        </is>
+      </c>
+      <c r="H75" s="18" t="inlineStr">
+        <is>
+          <t>w29</t>
+        </is>
+      </c>
+      <c r="I75" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J75" s="18" t="n"/>
+      <c r="K75" s="18" t="n"/>
+      <c r="L75" s="18" t="inlineStr"/>
+      <c r="M75" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="28" customHeight="1" s="29">
+      <c r="A76" s="18" t="n">
+        <v>28</v>
+      </c>
+      <c r="B76" s="18" t="inlineStr">
+        <is>
+          <t>w28</t>
+        </is>
+      </c>
+      <c r="C76" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D76" s="18" t="inlineStr">
+        <is>
+          <t>Check-in meeting</t>
+        </is>
+      </c>
+      <c r="E76" s="18" t="inlineStr">
+        <is>
+          <t>Meeting with Gerald, Amin, Susan, and optional review team members</t>
+        </is>
+      </c>
+      <c r="F76" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G76" s="18" t="inlineStr">
+        <is>
+          <t>w25</t>
+        </is>
+      </c>
+      <c r="H76" s="18" t="inlineStr">
+        <is>
+          <t>w29</t>
+        </is>
+      </c>
+      <c r="I76" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J76" s="18" t="n"/>
+      <c r="K76" s="18" t="n"/>
+      <c r="L76" s="18" t="inlineStr"/>
+      <c r="M76" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="18" t="n">
+        <v>29</v>
+      </c>
+      <c r="B77" s="18" t="inlineStr">
+        <is>
+          <t>w29</t>
+        </is>
+      </c>
+      <c r="C77" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D77" s="18" t="inlineStr">
+        <is>
+          <t>Criteria finalized</t>
+        </is>
+      </c>
+      <c r="E77" s="18" t="inlineStr">
+        <is>
+          <t>Confirm full-text screening criteria are finalized</t>
+        </is>
+      </c>
+      <c r="F77" s="18" t="inlineStr">
+        <is>
+          <t>Review Team / Sean</t>
+        </is>
+      </c>
+      <c r="G77" s="18" t="inlineStr">
+        <is>
+          <t>w11,w26,w27,w28</t>
+        </is>
+      </c>
+      <c r="H77" s="18" t="inlineStr">
+        <is>
+          <t>w30</t>
+        </is>
+      </c>
+      <c r="I77" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J77" s="18" t="n"/>
+      <c r="K77" s="18" t="n"/>
+      <c r="L77" s="18" t="inlineStr"/>
+      <c r="M77" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="28" customHeight="1" s="29">
+      <c r="A78" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="B78" s="18" t="inlineStr">
+        <is>
+          <t>w30</t>
+        </is>
+      </c>
+      <c r="C78" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D78" s="18" t="inlineStr">
+        <is>
+          <t>Tool setup</t>
+        </is>
+      </c>
+      <c r="E78" s="18" t="inlineStr">
+        <is>
+          <t>Tool setup - allocated AI tool for full-text screening</t>
+        </is>
+      </c>
+      <c r="F78" s="18" t="inlineStr">
+        <is>
+          <t>Response Team / Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G78" s="18" t="inlineStr">
+        <is>
+          <t>w04,w07,w29</t>
+        </is>
+      </c>
+      <c r="H78" s="18" t="inlineStr">
+        <is>
+          <t>w31</t>
+        </is>
+      </c>
+      <c r="I78" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J78" s="18" t="n"/>
+      <c r="K78" s="18" t="n"/>
+      <c r="L78" s="18" t="inlineStr"/>
+      <c r="M78" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="28" customHeight="1" s="29">
+      <c r="A79" s="18" t="n">
+        <v>31</v>
+      </c>
+      <c r="B79" s="18" t="inlineStr">
+        <is>
+          <t>w31</t>
+        </is>
+      </c>
+      <c r="C79" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D79" s="18" t="inlineStr">
+        <is>
+          <t>Setup validated</t>
+        </is>
+      </c>
+      <c r="E79" s="18" t="inlineStr">
+        <is>
+          <t>Review team validates full-text screening setup before starting</t>
+        </is>
+      </c>
+      <c r="F79" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G79" s="18" t="inlineStr">
+        <is>
+          <t>w30</t>
+        </is>
+      </c>
+      <c r="H79" s="18" t="inlineStr">
+        <is>
+          <t>w32,w33</t>
+        </is>
+      </c>
+      <c r="I79" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J79" s="18" t="n"/>
+      <c r="K79" s="18" t="n"/>
+      <c r="L79" s="18" t="inlineStr"/>
+      <c r="M79" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="18" t="n">
+        <v>32</v>
+      </c>
+      <c r="B80" s="18" t="inlineStr">
+        <is>
+          <t>w32</t>
+        </is>
+      </c>
+      <c r="C80" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D80" s="18" t="inlineStr">
+        <is>
+          <t>Human full text</t>
+        </is>
+      </c>
+      <c r="E80" s="18" t="inlineStr">
+        <is>
+          <t>Full-text screening - Human workflow</t>
+        </is>
+      </c>
+      <c r="F80" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G80" s="18" t="inlineStr">
+        <is>
+          <t>w05,w08,w09,w31</t>
+        </is>
+      </c>
+      <c r="H80" s="18" t="inlineStr">
+        <is>
+          <t>w36,w39,w40</t>
+        </is>
+      </c>
+      <c r="I80" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J80" s="18" t="n"/>
+      <c r="K80" s="18" t="n"/>
+      <c r="L80" s="18" t="inlineStr"/>
+      <c r="M80" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="18" t="n">
+        <v>33</v>
+      </c>
+      <c r="B81" s="18" t="inlineStr">
+        <is>
+          <t>w33</t>
+        </is>
+      </c>
+      <c r="C81" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D81" s="18" t="inlineStr">
+        <is>
+          <t>AI full text</t>
+        </is>
+      </c>
+      <c r="E81" s="18" t="inlineStr">
+        <is>
+          <t>Full-text screening - allocated AI tool</t>
+        </is>
+      </c>
+      <c r="F81" s="18" t="inlineStr">
+        <is>
+          <t>Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G81" s="18" t="inlineStr">
+        <is>
+          <t>w07,w08,w09,w31</t>
+        </is>
+      </c>
+      <c r="H81" s="18" t="inlineStr">
+        <is>
+          <t>w34,w36,w39,w40</t>
+        </is>
+      </c>
+      <c r="I81" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J81" s="18" t="n"/>
+      <c r="K81" s="18" t="n"/>
+      <c r="L81" s="18" t="inlineStr"/>
+      <c r="M81" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="18" t="n">
+        <v>34</v>
+      </c>
+      <c r="B82" s="18" t="inlineStr">
+        <is>
+          <t>w34</t>
+        </is>
+      </c>
+      <c r="C82" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D82" s="18" t="inlineStr">
+        <is>
+          <t>Export AI output</t>
+        </is>
+      </c>
+      <c r="E82" s="18" t="inlineStr">
+        <is>
+          <t>Export full-text screening output from allocated AI tool</t>
+        </is>
+      </c>
+      <c r="F82" s="18" t="inlineStr">
+        <is>
+          <t>Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G82" s="18" t="inlineStr">
+        <is>
+          <t>w33</t>
+        </is>
+      </c>
+      <c r="H82" s="18" t="inlineStr">
+        <is>
+          <t>w35</t>
+        </is>
+      </c>
+      <c r="I82" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J82" s="18" t="n"/>
+      <c r="K82" s="18" t="n"/>
+      <c r="L82" s="18" t="inlineStr"/>
+      <c r="M82" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="18" t="n">
+        <v>35</v>
+      </c>
+      <c r="B83" s="18" t="inlineStr">
+        <is>
+          <t>w35</t>
+        </is>
+      </c>
+      <c r="C83" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D83" s="18" t="inlineStr">
+        <is>
+          <t>Share output</t>
+        </is>
+      </c>
+      <c r="E83" s="18" t="inlineStr">
+        <is>
+          <t>Share full-text screening output with Sean / data manager</t>
+        </is>
+      </c>
+      <c r="F83" s="18" t="inlineStr">
+        <is>
+          <t>Krishna / Data Manager</t>
+        </is>
+      </c>
+      <c r="G83" s="18" t="inlineStr">
+        <is>
+          <t>w34</t>
+        </is>
+      </c>
+      <c r="H83" s="18" t="inlineStr">
+        <is>
+          <t>w39,w40</t>
+        </is>
+      </c>
+      <c r="I83" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J83" s="18" t="n"/>
+      <c r="K83" s="18" t="n"/>
+      <c r="L83" s="18" t="inlineStr"/>
+      <c r="M83" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="18" t="n">
+        <v>36</v>
+      </c>
+      <c r="B84" s="18" t="inlineStr">
+        <is>
+          <t>w36</t>
+        </is>
+      </c>
+      <c r="C84" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D84" s="18" t="inlineStr">
+        <is>
+          <t>Survey sent</t>
+        </is>
+      </c>
+      <c r="E84" s="18" t="inlineStr">
+        <is>
+          <t>Share usability survey on full-text screening workflow</t>
+        </is>
+      </c>
+      <c r="F84" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G84" s="18" t="inlineStr">
+        <is>
+          <t>w32,w33</t>
+        </is>
+      </c>
+      <c r="H84" s="18" t="inlineStr">
+        <is>
+          <t>w37</t>
+        </is>
+      </c>
+      <c r="I84" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J84" s="18" t="n"/>
+      <c r="K84" s="18" t="n"/>
+      <c r="L84" s="18" t="inlineStr"/>
+      <c r="M84" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="18" t="n">
+        <v>37</v>
+      </c>
+      <c r="B85" s="18" t="inlineStr">
+        <is>
+          <t>w37</t>
+        </is>
+      </c>
+      <c r="C85" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D85" s="18" t="inlineStr">
+        <is>
+          <t>Survey submitted</t>
+        </is>
+      </c>
+      <c r="E85" s="18" t="inlineStr">
+        <is>
+          <t>Submit usability survey on full-text screening workflow</t>
+        </is>
+      </c>
+      <c r="F85" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G85" s="18" t="inlineStr">
+        <is>
+          <t>w36</t>
+        </is>
+      </c>
+      <c r="H85" s="18" t="inlineStr">
+        <is>
+          <t>w38</t>
+        </is>
+      </c>
+      <c r="I85" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J85" s="18" t="n"/>
+      <c r="K85" s="18" t="n"/>
+      <c r="L85" s="18" t="inlineStr"/>
+      <c r="M85" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="28" customHeight="1" s="29">
+      <c r="A86" s="18" t="n">
+        <v>38</v>
+      </c>
+      <c r="B86" s="18" t="inlineStr">
+        <is>
+          <t>w38</t>
+        </is>
+      </c>
+      <c r="C86" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D86" s="18" t="inlineStr">
+        <is>
+          <t>Survey received</t>
+        </is>
+      </c>
+      <c r="E86" s="18" t="inlineStr">
+        <is>
+          <t>Confirm usability survey responses received for full-text screening</t>
+        </is>
+      </c>
+      <c r="F86" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G86" s="18" t="inlineStr">
+        <is>
+          <t>w37</t>
+        </is>
+      </c>
+      <c r="H86" s="18" t="inlineStr">
+        <is>
+          <t>w39</t>
+        </is>
+      </c>
+      <c r="I86" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J86" s="18" t="n"/>
+      <c r="K86" s="18" t="n"/>
+      <c r="L86" s="18" t="inlineStr"/>
+      <c r="M86" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="28" customHeight="1" s="29">
+      <c r="A87" s="18" t="n">
+        <v>39</v>
+      </c>
+      <c r="B87" s="18" t="inlineStr">
+        <is>
+          <t>w39</t>
+        </is>
+      </c>
+      <c r="C87" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D87" s="18" t="inlineStr">
+        <is>
+          <t>Quality check</t>
+        </is>
+      </c>
+      <c r="E87" s="18" t="inlineStr">
+        <is>
+          <t>Data completeness and quality check before full-text adjudication</t>
+        </is>
+      </c>
+      <c r="F87" s="18" t="inlineStr">
+        <is>
+          <t>Data Manager / Sean</t>
+        </is>
+      </c>
+      <c r="G87" s="18" t="inlineStr">
+        <is>
+          <t>w35,w38</t>
+        </is>
+      </c>
+      <c r="H87" s="18" t="inlineStr">
+        <is>
+          <t>w40</t>
+        </is>
+      </c>
+      <c r="I87" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J87" s="18" t="n"/>
+      <c r="K87" s="18" t="n"/>
+      <c r="L87" s="18" t="inlineStr"/>
+      <c r="M87" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="18" t="n">
+        <v>40</v>
+      </c>
+      <c r="B88" s="18" t="inlineStr">
+        <is>
+          <t>w40</t>
+        </is>
+      </c>
+      <c r="C88" s="18" t="inlineStr">
+        <is>
+          <t>Full-text readiness and screening</t>
+        </is>
+      </c>
+      <c r="D88" s="18" t="inlineStr">
+        <is>
+          <t>Full-text adjudication</t>
+        </is>
+      </c>
+      <c r="E88" s="18" t="inlineStr">
+        <is>
+          <t>Adjudication panel after full-text screening</t>
+        </is>
+      </c>
+      <c r="F88" s="18" t="inlineStr">
+        <is>
+          <t>Sean and Adjudication Panel</t>
+        </is>
+      </c>
+      <c r="G88" s="18" t="inlineStr">
+        <is>
+          <t>w39</t>
+        </is>
+      </c>
+      <c r="H88" s="18" t="inlineStr">
+        <is>
+          <t>w42,w43,w45</t>
+        </is>
+      </c>
+      <c r="I88" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J88" s="18" t="n"/>
+      <c r="K88" s="18" t="n"/>
+      <c r="L88" s="18" t="inlineStr"/>
+      <c r="M88" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="18" t="n">
+        <v>41</v>
+      </c>
+      <c r="B89" s="18" t="inlineStr">
+        <is>
+          <t>w41</t>
+        </is>
+      </c>
+      <c r="C89" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D89" s="18" t="inlineStr">
+        <is>
+          <t>Platform ready</t>
+        </is>
+      </c>
+      <c r="E89" s="18" t="inlineStr">
+        <is>
+          <t>Finalisation of Laser AI platform/server setup, if applicable</t>
+        </is>
+      </c>
+      <c r="F89" s="18" t="inlineStr">
+        <is>
+          <t>Core Team / Laser AI</t>
+        </is>
+      </c>
+      <c r="G89" s="18" t="inlineStr">
+        <is>
+          <t>w04,w07</t>
+        </is>
+      </c>
+      <c r="H89" s="18" t="inlineStr">
+        <is>
+          <t>w45</t>
+        </is>
+      </c>
+      <c r="I89" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J89" s="18" t="n"/>
+      <c r="K89" s="18" t="n"/>
+      <c r="L89" s="18" t="inlineStr"/>
+      <c r="M89" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="28" customHeight="1" s="29">
+      <c r="A90" s="18" t="n">
+        <v>42</v>
+      </c>
+      <c r="B90" s="18" t="inlineStr">
+        <is>
+          <t>w42</t>
+        </is>
+      </c>
+      <c r="C90" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D90" s="18" t="inlineStr">
+        <is>
+          <t>DE check-in</t>
+        </is>
+      </c>
+      <c r="E90" s="18" t="inlineStr">
+        <is>
+          <t>Meeting with Gerald and optional review team members before data extraction</t>
+        </is>
+      </c>
+      <c r="F90" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G90" s="18" t="inlineStr">
+        <is>
+          <t>w40</t>
+        </is>
+      </c>
+      <c r="H90" s="18" t="inlineStr">
+        <is>
+          <t>w43</t>
+        </is>
+      </c>
+      <c r="I90" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J90" s="18" t="n"/>
+      <c r="K90" s="18" t="n"/>
+      <c r="L90" s="18" t="inlineStr"/>
+      <c r="M90" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="18" t="n">
+        <v>43</v>
+      </c>
+      <c r="B91" s="18" t="inlineStr">
+        <is>
+          <t>w43</t>
+        </is>
+      </c>
+      <c r="C91" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D91" s="18" t="inlineStr">
+        <is>
+          <t>DE items confirmed</t>
+        </is>
+      </c>
+      <c r="E91" s="18" t="inlineStr">
+        <is>
+          <t>Confirm final data extraction items and definitions</t>
+        </is>
+      </c>
+      <c r="F91" s="18" t="inlineStr">
+        <is>
+          <t>Review Team / Sean</t>
+        </is>
+      </c>
+      <c r="G91" s="18" t="inlineStr">
+        <is>
+          <t>w12,w14,w40,w42</t>
+        </is>
+      </c>
+      <c r="H91" s="18" t="inlineStr">
+        <is>
+          <t>w44</t>
+        </is>
+      </c>
+      <c r="I91" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J91" s="18" t="n"/>
+      <c r="K91" s="18" t="n"/>
+      <c r="L91" s="18" t="inlineStr"/>
+      <c r="M91" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="18" t="n">
+        <v>44</v>
+      </c>
+      <c r="B92" s="18" t="inlineStr">
+        <is>
+          <t>w44</t>
+        </is>
+      </c>
+      <c r="C92" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D92" s="18" t="inlineStr">
+        <is>
+          <t>Form approved</t>
+        </is>
+      </c>
+      <c r="E92" s="18" t="inlineStr">
+        <is>
+          <t>Confirm extraction form/template is approved by Sean</t>
+        </is>
+      </c>
+      <c r="F92" s="18" t="inlineStr">
+        <is>
+          <t>Sean</t>
+        </is>
+      </c>
+      <c r="G92" s="18" t="inlineStr">
+        <is>
+          <t>w13,w14,w43</t>
+        </is>
+      </c>
+      <c r="H92" s="18" t="inlineStr">
+        <is>
+          <t>w45</t>
+        </is>
+      </c>
+      <c r="I92" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J92" s="18" t="n"/>
+      <c r="K92" s="18" t="n"/>
+      <c r="L92" s="18" t="inlineStr"/>
+      <c r="M92" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="28" customHeight="1" s="29">
+      <c r="A93" s="18" t="n">
+        <v>45</v>
+      </c>
+      <c r="B93" s="18" t="inlineStr">
+        <is>
+          <t>w45</t>
+        </is>
+      </c>
+      <c r="C93" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D93" s="18" t="inlineStr">
+        <is>
+          <t>Tool setup</t>
+        </is>
+      </c>
+      <c r="E93" s="18" t="inlineStr">
+        <is>
+          <t>Tool setup - allocated AI tool for data extraction</t>
+        </is>
+      </c>
+      <c r="F93" s="18" t="inlineStr">
+        <is>
+          <t>Response Team / Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G93" s="18" t="inlineStr">
+        <is>
+          <t>w41,w44</t>
+        </is>
+      </c>
+      <c r="H93" s="18" t="inlineStr">
+        <is>
+          <t>w46</t>
+        </is>
+      </c>
+      <c r="I93" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J93" s="18" t="n"/>
+      <c r="K93" s="18" t="n"/>
+      <c r="L93" s="18" t="inlineStr"/>
+      <c r="M93" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="28" customHeight="1" s="29">
+      <c r="A94" s="18" t="n">
+        <v>46</v>
+      </c>
+      <c r="B94" s="18" t="inlineStr">
+        <is>
+          <t>w46</t>
+        </is>
+      </c>
+      <c r="C94" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D94" s="18" t="inlineStr">
+        <is>
+          <t>Setup validated</t>
+        </is>
+      </c>
+      <c r="E94" s="18" t="inlineStr">
+        <is>
+          <t>Review team validates data extraction setup before starting</t>
+        </is>
+      </c>
+      <c r="F94" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G94" s="18" t="inlineStr">
+        <is>
+          <t>w45</t>
+        </is>
+      </c>
+      <c r="H94" s="18" t="inlineStr">
+        <is>
+          <t>w47,w48</t>
+        </is>
+      </c>
+      <c r="I94" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J94" s="18" t="n"/>
+      <c r="K94" s="18" t="n"/>
+      <c r="L94" s="18" t="inlineStr"/>
+      <c r="M94" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="18" t="n">
+        <v>47</v>
+      </c>
+      <c r="B95" s="18" t="inlineStr">
+        <is>
+          <t>w47</t>
+        </is>
+      </c>
+      <c r="C95" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D95" s="18" t="inlineStr">
+        <is>
+          <t>Human extraction</t>
+        </is>
+      </c>
+      <c r="E95" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction - Human workflow</t>
+        </is>
+      </c>
+      <c r="F95" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G95" s="18" t="inlineStr">
+        <is>
+          <t>w05,w08,w09,w46</t>
+        </is>
+      </c>
+      <c r="H95" s="18" t="inlineStr">
+        <is>
+          <t>w51,w54,w55</t>
+        </is>
+      </c>
+      <c r="I95" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J95" s="18" t="n"/>
+      <c r="K95" s="18" t="n"/>
+      <c r="L95" s="18" t="inlineStr"/>
+      <c r="M95" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="18" t="n">
+        <v>48</v>
+      </c>
+      <c r="B96" s="18" t="inlineStr">
+        <is>
+          <t>w48</t>
+        </is>
+      </c>
+      <c r="C96" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D96" s="18" t="inlineStr">
+        <is>
+          <t>AI extraction</t>
+        </is>
+      </c>
+      <c r="E96" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction - allocated AI tool</t>
+        </is>
+      </c>
+      <c r="F96" s="18" t="inlineStr">
+        <is>
+          <t>Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G96" s="18" t="inlineStr">
+        <is>
+          <t>w07,w08,w09,w46</t>
+        </is>
+      </c>
+      <c r="H96" s="18" t="inlineStr">
+        <is>
+          <t>w49,w51,w54,w55</t>
+        </is>
+      </c>
+      <c r="I96" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J96" s="18" t="n"/>
+      <c r="K96" s="18" t="n"/>
+      <c r="L96" s="18" t="inlineStr"/>
+      <c r="M96" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="18" t="n">
+        <v>49</v>
+      </c>
+      <c r="B97" s="18" t="inlineStr">
+        <is>
+          <t>w49</t>
+        </is>
+      </c>
+      <c r="C97" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D97" s="18" t="inlineStr">
+        <is>
+          <t>Export AI output</t>
+        </is>
+      </c>
+      <c r="E97" s="18" t="inlineStr">
+        <is>
+          <t>Export data extraction output from allocated AI tool</t>
+        </is>
+      </c>
+      <c r="F97" s="18" t="inlineStr">
+        <is>
+          <t>Allocated Tool Team</t>
+        </is>
+      </c>
+      <c r="G97" s="18" t="inlineStr">
+        <is>
+          <t>w48</t>
+        </is>
+      </c>
+      <c r="H97" s="18" t="inlineStr">
+        <is>
+          <t>w50</t>
+        </is>
+      </c>
+      <c r="I97" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J97" s="18" t="n"/>
+      <c r="K97" s="18" t="n"/>
+      <c r="L97" s="18" t="inlineStr"/>
+      <c r="M97" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="18" t="n">
+        <v>50</v>
+      </c>
+      <c r="B98" s="18" t="inlineStr">
+        <is>
+          <t>w50</t>
+        </is>
+      </c>
+      <c r="C98" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D98" s="18" t="inlineStr">
+        <is>
+          <t>Share output</t>
+        </is>
+      </c>
+      <c r="E98" s="18" t="inlineStr">
+        <is>
+          <t>Share data extraction output with Sean / data manager</t>
+        </is>
+      </c>
+      <c r="F98" s="18" t="inlineStr">
+        <is>
+          <t>Krishna / Data Manager</t>
+        </is>
+      </c>
+      <c r="G98" s="18" t="inlineStr">
+        <is>
+          <t>w49</t>
+        </is>
+      </c>
+      <c r="H98" s="18" t="inlineStr">
+        <is>
+          <t>w54,w55</t>
+        </is>
+      </c>
+      <c r="I98" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J98" s="18" t="n"/>
+      <c r="K98" s="18" t="n"/>
+      <c r="L98" s="18" t="inlineStr"/>
+      <c r="M98" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="18" t="n">
+        <v>51</v>
+      </c>
+      <c r="B99" s="18" t="inlineStr">
+        <is>
+          <t>w51</t>
+        </is>
+      </c>
+      <c r="C99" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D99" s="18" t="inlineStr">
+        <is>
+          <t>Survey sent</t>
+        </is>
+      </c>
+      <c r="E99" s="18" t="inlineStr">
+        <is>
+          <t>Share usability survey on data extraction workflow</t>
+        </is>
+      </c>
+      <c r="F99" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G99" s="18" t="inlineStr">
+        <is>
+          <t>w47,w48</t>
+        </is>
+      </c>
+      <c r="H99" s="18" t="inlineStr">
+        <is>
+          <t>w52</t>
+        </is>
+      </c>
+      <c r="I99" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J99" s="18" t="n"/>
+      <c r="K99" s="18" t="n"/>
+      <c r="L99" s="18" t="inlineStr"/>
+      <c r="M99" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="18" t="n">
+        <v>52</v>
+      </c>
+      <c r="B100" s="18" t="inlineStr">
+        <is>
+          <t>w52</t>
+        </is>
+      </c>
+      <c r="C100" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D100" s="18" t="inlineStr">
+        <is>
+          <t>Survey submitted</t>
+        </is>
+      </c>
+      <c r="E100" s="18" t="inlineStr">
+        <is>
+          <t>Submit usability survey on data extraction workflow</t>
+        </is>
+      </c>
+      <c r="F100" s="18" t="inlineStr">
+        <is>
+          <t>Review Team</t>
+        </is>
+      </c>
+      <c r="G100" s="18" t="inlineStr">
+        <is>
+          <t>w51</t>
+        </is>
+      </c>
+      <c r="H100" s="18" t="inlineStr">
+        <is>
+          <t>w53</t>
+        </is>
+      </c>
+      <c r="I100" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J100" s="18" t="n"/>
+      <c r="K100" s="18" t="n"/>
+      <c r="L100" s="18" t="inlineStr"/>
+      <c r="M100" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="28" customHeight="1" s="29">
+      <c r="A101" s="18" t="n">
+        <v>53</v>
+      </c>
+      <c r="B101" s="18" t="inlineStr">
+        <is>
+          <t>w53</t>
+        </is>
+      </c>
+      <c r="C101" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D101" s="18" t="inlineStr">
+        <is>
+          <t>Survey received</t>
+        </is>
+      </c>
+      <c r="E101" s="18" t="inlineStr">
+        <is>
+          <t>Confirm usability survey responses received for data extraction</t>
+        </is>
+      </c>
+      <c r="F101" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G101" s="18" t="inlineStr">
+        <is>
+          <t>w52</t>
+        </is>
+      </c>
+      <c r="H101" s="18" t="inlineStr">
+        <is>
+          <t>w54</t>
+        </is>
+      </c>
+      <c r="I101" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J101" s="18" t="n"/>
+      <c r="K101" s="18" t="n"/>
+      <c r="L101" s="18" t="inlineStr"/>
+      <c r="M101" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="28" customHeight="1" s="29">
+      <c r="A102" s="18" t="n">
+        <v>54</v>
+      </c>
+      <c r="B102" s="18" t="inlineStr">
+        <is>
+          <t>w54</t>
+        </is>
+      </c>
+      <c r="C102" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D102" s="18" t="inlineStr">
+        <is>
+          <t>Quality check</t>
+        </is>
+      </c>
+      <c r="E102" s="18" t="inlineStr">
+        <is>
+          <t>Data completeness and quality check before data extraction adjudication</t>
+        </is>
+      </c>
+      <c r="F102" s="18" t="inlineStr">
+        <is>
+          <t>Data Manager / Sean</t>
+        </is>
+      </c>
+      <c r="G102" s="18" t="inlineStr">
+        <is>
+          <t>w50,w53</t>
+        </is>
+      </c>
+      <c r="H102" s="18" t="inlineStr">
+        <is>
+          <t>w55</t>
+        </is>
+      </c>
+      <c r="I102" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J102" s="18" t="n"/>
+      <c r="K102" s="18" t="n"/>
+      <c r="L102" s="18" t="inlineStr"/>
+      <c r="M102" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="18" t="n">
+        <v>55</v>
+      </c>
+      <c r="B103" s="18" t="inlineStr">
+        <is>
+          <t>w55</t>
+        </is>
+      </c>
+      <c r="C103" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D103" s="18" t="inlineStr">
+        <is>
+          <t>Adjudication dataset</t>
+        </is>
+      </c>
+      <c r="E103" s="18" t="inlineStr">
+        <is>
+          <t>Prepare adjudication-ready dataset</t>
+        </is>
+      </c>
+      <c r="F103" s="18" t="inlineStr">
+        <is>
+          <t>Data Manager / Sean</t>
+        </is>
+      </c>
+      <c r="G103" s="18" t="inlineStr">
+        <is>
+          <t>w54</t>
+        </is>
+      </c>
+      <c r="H103" s="18" t="inlineStr">
+        <is>
+          <t>w56,w57,w58,w61,w62,w63</t>
+        </is>
+      </c>
+      <c r="I103" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J103" s="18" t="n"/>
+      <c r="K103" s="18" t="n"/>
+      <c r="L103" s="18" t="inlineStr"/>
+      <c r="M103" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="18" t="n">
+        <v>56</v>
+      </c>
+      <c r="B104" s="18" t="inlineStr">
+        <is>
+          <t>w56</t>
+        </is>
+      </c>
+      <c r="C104" s="18" t="inlineStr">
+        <is>
+          <t>Data extraction</t>
+        </is>
+      </c>
+      <c r="D104" s="18" t="inlineStr">
+        <is>
+          <t>DE adjudication</t>
+        </is>
+      </c>
+      <c r="E104" s="18" t="inlineStr">
+        <is>
+          <t>Adjudication panel after data extraction</t>
+        </is>
+      </c>
+      <c r="F104" s="18" t="inlineStr">
+        <is>
+          <t>Sean and Adjudication Panel</t>
+        </is>
+      </c>
+      <c r="G104" s="18" t="inlineStr">
+        <is>
+          <t>w55</t>
+        </is>
+      </c>
+      <c r="H104" s="18" t="inlineStr">
+        <is>
+          <t>w57,w60,w61,w62,w63</t>
+        </is>
+      </c>
+      <c r="I104" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J104" s="18" t="n"/>
+      <c r="K104" s="18" t="n"/>
+      <c r="L104" s="18" t="inlineStr"/>
+      <c r="M104" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="18" t="n">
+        <v>57</v>
+      </c>
+      <c r="B105" s="18" t="inlineStr">
+        <is>
+          <t>w57</t>
+        </is>
+      </c>
+      <c r="C105" s="18" t="inlineStr">
+        <is>
+          <t>Analysis and downstream work</t>
+        </is>
+      </c>
+      <c r="D105" s="18" t="inlineStr">
+        <is>
+          <t>Gerald closeout</t>
+        </is>
+      </c>
+      <c r="E105" s="18" t="inlineStr">
+        <is>
+          <t>Meeting with Gerald before analysis closeout</t>
+        </is>
+      </c>
+      <c r="F105" s="18" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="G105" s="18" t="inlineStr">
+        <is>
+          <t>w56</t>
+        </is>
+      </c>
+      <c r="H105" s="18" t="inlineStr">
+        <is>
+          <t>w59,w63</t>
+        </is>
+      </c>
+      <c r="I105" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J105" s="18" t="n"/>
+      <c r="K105" s="18" t="n"/>
+      <c r="L105" s="18" t="inlineStr"/>
+      <c r="M105" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="18" t="n">
+        <v>58</v>
+      </c>
+      <c r="B106" s="18" t="inlineStr">
+        <is>
+          <t>w58</t>
+        </is>
+      </c>
+      <c r="C106" s="18" t="inlineStr">
+        <is>
+          <t>Analysis and downstream work</t>
+        </is>
+      </c>
+      <c r="D106" s="18" t="inlineStr">
+        <is>
+          <t>Stability study</t>
+        </is>
+      </c>
+      <c r="E106" s="18" t="inlineStr">
+        <is>
+          <t>Fully automated and stability study - Pawel and Noosheen</t>
+        </is>
+      </c>
+      <c r="F106" s="18" t="inlineStr">
+        <is>
+          <t>Pawel / Noosheen</t>
+        </is>
+      </c>
+      <c r="G106" s="18" t="inlineStr">
+        <is>
+          <t>w55</t>
+        </is>
+      </c>
+      <c r="H106" s="18" t="inlineStr">
+        <is>
+          <t>w63</t>
+        </is>
+      </c>
+      <c r="I106" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J106" s="18" t="n"/>
+      <c r="K106" s="18" t="n"/>
+      <c r="L106" s="18" t="inlineStr"/>
+      <c r="M106" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="18" t="n">
+        <v>59</v>
+      </c>
+      <c r="B107" s="18" t="inlineStr">
+        <is>
+          <t>w59</t>
+        </is>
+      </c>
+      <c r="C107" s="18" t="inlineStr">
+        <is>
+          <t>Analysis and downstream work</t>
+        </is>
+      </c>
+      <c r="D107" s="18" t="inlineStr">
+        <is>
+          <t>Follow-up</t>
+        </is>
+      </c>
+      <c r="E107" s="18" t="inlineStr">
+        <is>
+          <t>Follow-up and review</t>
+        </is>
+      </c>
+      <c r="F107" s="18" t="inlineStr">
+        <is>
+          <t>Core Team</t>
+        </is>
+      </c>
+      <c r="G107" s="18" t="inlineStr">
+        <is>
+          <t>w57</t>
+        </is>
+      </c>
+      <c r="H107" s="18" t="inlineStr">
+        <is>
+          <t>w63</t>
+        </is>
+      </c>
+      <c r="I107" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J107" s="18" t="n"/>
+      <c r="K107" s="18" t="n"/>
+      <c r="L107" s="18" t="inlineStr"/>
+      <c r="M107" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="18" t="n">
+        <v>60</v>
+      </c>
+      <c r="B108" s="18" t="inlineStr">
+        <is>
+          <t>w60</t>
+        </is>
+      </c>
+      <c r="C108" s="18" t="inlineStr">
+        <is>
+          <t>Analysis and downstream work</t>
+        </is>
+      </c>
+      <c r="D108" s="18" t="inlineStr">
+        <is>
+          <t>Adjudication work</t>
+        </is>
+      </c>
+      <c r="E108" s="18" t="inlineStr">
+        <is>
+          <t>Adjudication panel parallel work</t>
+        </is>
+      </c>
+      <c r="F108" s="18" t="inlineStr">
+        <is>
+          <t>Adjudication Panel</t>
+        </is>
+      </c>
+      <c r="G108" s="18" t="inlineStr">
+        <is>
+          <t>w25,w40,w56</t>
+        </is>
+      </c>
+      <c r="H108" s="18" t="inlineStr">
+        <is>
+          <t>w63</t>
+        </is>
+      </c>
+      <c r="I108" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J108" s="18" t="n"/>
+      <c r="K108" s="18" t="n"/>
+      <c r="L108" s="18" t="inlineStr"/>
+      <c r="M108" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="18" t="n">
+        <v>61</v>
+      </c>
+      <c r="B109" s="18" t="inlineStr">
+        <is>
+          <t>w61</t>
+        </is>
+      </c>
+      <c r="C109" s="18" t="inlineStr">
+        <is>
+          <t>Analysis and downstream work</t>
+        </is>
+      </c>
+      <c r="D109" s="18" t="inlineStr">
+        <is>
+          <t>Afroditi analysis</t>
+        </is>
+      </c>
+      <c r="E109" s="18" t="inlineStr">
+        <is>
+          <t>Afroditi analysis</t>
+        </is>
+      </c>
+      <c r="F109" s="18" t="inlineStr">
+        <is>
+          <t>Afroditi</t>
+        </is>
+      </c>
+      <c r="G109" s="18" t="inlineStr">
+        <is>
+          <t>w55,w56</t>
+        </is>
+      </c>
+      <c r="H109" s="18" t="inlineStr">
+        <is>
+          <t>w63</t>
+        </is>
+      </c>
+      <c r="I109" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J109" s="18" t="n"/>
+      <c r="K109" s="18" t="n"/>
+      <c r="L109" s="18" t="inlineStr"/>
+      <c r="M109" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="18" t="n">
+        <v>62</v>
+      </c>
+      <c r="B110" s="18" t="inlineStr">
+        <is>
+          <t>w62</t>
+        </is>
+      </c>
+      <c r="C110" s="18" t="inlineStr">
+        <is>
+          <t>Analysis and downstream work</t>
+        </is>
+      </c>
+      <c r="D110" s="18" t="inlineStr">
+        <is>
+          <t>Downstream errors</t>
+        </is>
+      </c>
+      <c r="E110" s="18" t="inlineStr">
+        <is>
+          <t>Downstream impact of errors research - Max and Joanna</t>
+        </is>
+      </c>
+      <c r="F110" s="18" t="inlineStr">
+        <is>
+          <t>Max / Joanna</t>
+        </is>
+      </c>
+      <c r="G110" s="18" t="inlineStr">
+        <is>
+          <t>w55,w56</t>
+        </is>
+      </c>
+      <c r="H110" s="18" t="inlineStr">
+        <is>
+          <t>w63</t>
+        </is>
+      </c>
+      <c r="I110" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J110" s="18" t="n"/>
+      <c r="K110" s="18" t="n"/>
+      <c r="L110" s="18" t="inlineStr"/>
+      <c r="M110" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="18" t="n">
+        <v>63</v>
+      </c>
+      <c r="B111" s="18" t="inlineStr">
+        <is>
+          <t>w63</t>
+        </is>
+      </c>
+      <c r="C111" s="18" t="inlineStr">
+        <is>
+          <t>Analysis and downstream work</t>
+        </is>
+      </c>
+      <c r="D111" s="18" t="inlineStr">
+        <is>
+          <t>Final analysis</t>
+        </is>
+      </c>
+      <c r="E111" s="18" t="inlineStr">
+        <is>
+          <t>Final analysis</t>
+        </is>
+      </c>
+      <c r="F111" s="18" t="inlineStr">
+        <is>
+          <t>Analysis Team</t>
+        </is>
+      </c>
+      <c r="G111" s="18" t="inlineStr">
+        <is>
+          <t>w57,w58,w59,w60,w61,w62</t>
+        </is>
+      </c>
+      <c r="H111" s="18" t="n"/>
+      <c r="I111" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J111" s="18" t="n"/>
+      <c r="K111" s="18" t="n"/>
+      <c r="L111" s="18" t="inlineStr"/>
+      <c r="M111" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="5" t="inlineStr">
+        <is>
+          <t>Review Tasks Displayed in Dashboard</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="n"/>
+      <c r="C113" s="5" t="n"/>
+      <c r="D113" s="5" t="n"/>
+      <c r="E113" s="5" t="n"/>
+      <c r="F113" s="5" t="n"/>
+      <c r="G113" s="5" t="n"/>
+      <c r="H113" s="5" t="n"/>
+      <c r="I113" s="5" t="n"/>
+      <c r="J113" s="5" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="1" t="inlineStr">
+        <is>
+          <t>TaskID</t>
+        </is>
+      </c>
+      <c r="B114" s="1" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C114" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D114" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E114" s="1" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="F114" s="1" t="inlineStr">
+        <is>
+          <t>DueDate</t>
+        </is>
+      </c>
+      <c r="G114" s="1" t="inlineStr">
+        <is>
+          <t>Dependency</t>
+        </is>
+      </c>
+      <c r="H114" s="1" t="inlineStr">
+        <is>
+          <t>Communication</t>
+        </is>
+      </c>
+      <c r="I114" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="J114" s="1" t="inlineStr">
+        <is>
+          <t>SourceDate</t>
+        </is>
+      </c>
+      <c r="K114" s="1" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>task-phase1-09-001</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Confirm crossed reviewer allocation and complete review team split</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Gerald / Krishna / Review Team</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>December 2026</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Reviewer-allocation confirmation</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Initial onboarding completed; crossed reviewer allocation awaits Gerald's confirmation</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Project tracking</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120">
+      <c r="A120" s="5" t="inlineStr">
+        <is>
+          <t>Recent Mail / Communication Log Displayed in Dashboard</t>
+        </is>
+      </c>
+      <c r="B120" s="5" t="n"/>
+      <c r="C120" s="5" t="n"/>
+      <c r="D120" s="5" t="n"/>
+      <c r="E120" s="5" t="n"/>
+      <c r="F120" s="5" t="n"/>
+      <c r="G120" s="5" t="n"/>
+      <c r="H120" s="5" t="n"/>
+      <c r="I120" s="5" t="n"/>
+      <c r="J120" s="5" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="1" t="inlineStr">
+        <is>
+          <t>CommunicationID</t>
+        </is>
+      </c>
+      <c r="B121" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C121" s="1" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="D121" s="1" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+      <c r="E121" s="1" t="inlineStr">
+        <is>
+          <t>Responsible</t>
+        </is>
+      </c>
+      <c r="F121" s="1" t="inlineStr">
+        <is>
+          <t>DueDate</t>
+        </is>
+      </c>
+      <c r="G121" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H121" s="1" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="I121" s="1" t="inlineStr">
+        <is>
+          <t>LinkedTaskID</t>
+        </is>
+      </c>
+      <c r="J121" s="1" t="inlineStr">
+        <is>
+          <t>LinkedAction</t>
+        </is>
+      </c>
+      <c r="K121" s="1" t="inlineStr">
+        <is>
+          <t>SourceType</t>
+        </is>
+      </c>
+      <c r="L121" s="1" t="inlineStr">
+        <is>
+          <t>SourceLink</t>
+        </is>
+      </c>
+      <c r="M121" s="1" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>comm-phase1-09-001</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Orthodontic Retention added as eighth review</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Álvaro Limones / Concepción Martín Álvaro / Gerald / Krishna</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Gerald / Krishna</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>December 2026</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Initial onboarding completed; Gerald to confirm crossed reviewer allocation before setup proceeds</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>task-phase1-09-001</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Confirm crossed reviewer allocation and complete review team split</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>Project tracking</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="123"/>
+    <row r="124">
+      <c r="A124" s="5" t="inlineStr">
+        <is>
+          <t>Critical Items Displayed in Dashboard</t>
+        </is>
+      </c>
+      <c r="B124" s="5" t="n"/>
+      <c r="C124" s="5" t="n"/>
+      <c r="D124" s="5" t="n"/>
+      <c r="E124" s="5" t="n"/>
+      <c r="F124" s="5" t="n"/>
+      <c r="G124" s="5" t="n"/>
+      <c r="H124" s="5" t="n"/>
+      <c r="I124" s="5" t="n"/>
+      <c r="J124" s="5" t="n"/>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="1" t="inlineStr">
+        <is>
+          <t>CriticalItem</t>
+        </is>
+      </c>
+      <c r="B125" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C125" s="1" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="D125" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E125" s="1" t="inlineStr">
+        <is>
+          <t>DueDate</t>
+        </is>
+      </c>
+      <c r="F125" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G125" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>SourceDate</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Reviewer-allocation confirmation needed before setup</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Reviewer allocation is not yet confirmed.</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Gerald / Krishna</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>December 2026</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Finalize crossed reviewer allocation, team split and tool assignment before setup.</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Setup cannot proceed until allocation and tool plan are confirmed.</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Project tracking</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="18" customWidth="1" style="29" min="1" max="2"/>
@@ -42655,6 +47375,78 @@
       <c r="N12" t="inlineStr">
         <is>
           <t>phase1-08 LNS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>phase1-09</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Orthodontic Retention</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Retention procedures for stabilising tooth position after treatment with orthodontic braces</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Initial onboarding completed; reviewer-allocation model awaiting confirmation</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Álvaro Limones / Concepción Martín Álvaro</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Approximately 300–500 references expected; searches planned for November</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Gerald to confirm the crossed reviewer allocation; then finalize team split, tool assignment and setup</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>December 2026</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>phase1-09 Orthodontic Retention</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboard through October 4
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -12690,7 +12690,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Repository for finalized exports and protocols; working RIS and PDF sets remain in the relevant platform until consolidation.</t>
+          <t>Current review-specific folders contain RIS files and protocols; Sean will add full-text PDFs after each review’s adjudication</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -12733,7 +12733,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -22332,7 +22332,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Converted to phase1-07; abstract screening complete and the 77-reference full-text set approved</t>
+          <t>Converted to phase1-07; follow-up call requested after reviewer withdrawal and screening-record differences</t>
         </is>
       </c>
       <c r="E12" s="17" t="inlineStr">
@@ -22347,12 +22347,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Full-text screening ready; target 31 October</t>
+          <t>Full-text plan under review; target remains 31 October</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Both arms will use 77 references; at least two conventional reviewers are required following Michelle’s withdrawal</t>
+          <t>Seventy-seven-reference set approved; Michelle withdrew; Murali is the sole conventional reviewer; follow-up pending</t>
         </is>
       </c>
       <c r="I12" s="17" t="inlineStr">
@@ -22854,7 +22854,7 @@
       </c>
       <c r="D28" s="17" t="inlineStr">
         <is>
-          <t>Converted to phase1-06; both full-text arms aligned and cleared to proceed</t>
+          <t>Converted to phase1-06; full-text screening underway and NK extraction form prepared</t>
         </is>
       </c>
       <c r="E28" s="17" t="inlineStr">
@@ -22869,12 +22869,12 @@
       </c>
       <c r="G28" s="17" t="inlineStr">
         <is>
-          <t>Full-text screening underway; missing PDFs still required</t>
+          <t>Full-text screening underway; review and approve the NK extraction form before extraction</t>
         </is>
       </c>
       <c r="H28" s="17" t="inlineStr">
         <is>
-          <t>Meghan confirmed alignment of both arms; missing PDFs remain</t>
+          <t>Both arms aligned; missing PDFs remain; Meghan built and tested the NK extraction form</t>
         </is>
       </c>
       <c r="I28" s="17" t="inlineStr">
@@ -23177,7 +23177,7 @@
       </c>
       <c r="D35" s="17" t="inlineStr">
         <is>
-          <t>Converted to phase1-09; initial onboarding completed and reviewer allocation awaiting confirmation</t>
+          <t>Converted to phase1-09; separate reviewer groups required and updated searches being arranged</t>
         </is>
       </c>
       <c r="E35" s="17" t="inlineStr">
@@ -23192,12 +23192,12 @@
       </c>
       <c r="G35" s="17" t="inlineStr">
         <is>
-          <t>Onboarding completed; searches expected in November and screening/data extraction planned for December</t>
+          <t>Search updates being arranged; Irma will update Embase from April 2022 onward</t>
         </is>
       </c>
       <c r="H35" s="17" t="inlineStr">
         <is>
-          <t>Final eighth review; crossed reviewer allocation proposed and awaiting Gerald's confirmation</t>
+          <t>Crossed allocation rejected; both groups must receive the same records; finalize separate reviewer groups before setup</t>
         </is>
       </c>
       <c r="I35" s="17" t="inlineStr">
@@ -26901,7 +26901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="14" customWidth="1" style="29" min="1" max="2"/>
@@ -27512,7 +27512,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Recurring Thursday adjudication meetings through December; first review completed</t>
+          <t>BP adjudication complete; further adjudication awaits finalized review datasets</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -27538,6 +27538,58 @@
       <c r="M11" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>mtg-11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>10:00–11:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>3:00–4:00 PM BST</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>CESAR – Screening Accuracy Review</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Discuss Psoriasis accuracy data and reconciliation</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Gerald / Sean / Afroditi / Krishna</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
         </is>
       </c>
     </row>
@@ -27706,7 +27758,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abstract outputs reconciled; both full-text arms cleared to proceed; missing PDFs remain</t>
+          <t>Full-text screening underway; missing PDFs remain; NK extraction form prepared</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -27774,7 +27826,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Full-text screening underway</t>
+          <t>Both full-text arms progressing; NK extraction form built and tested</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -27791,7 +27843,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>NK updated with 16 Covidence-only citations; 14 AI-only citations were identified; both arms are aligned</t>
+          <t>NK form built from the 22 June Excel template; Jeremy asked to review and adjust it</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -27808,7 +27860,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Retrieve missing PDFs, complete both full-text arms and record time</t>
+          <t>Retrieve missing PDFs, finish both full-text arms, review the NK extraction form and record time</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -27898,7 +27950,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -28354,7 +28406,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Preparation underway</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Meghan built and tested the NK extraction form; review-team confirmation remains pending</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -30745,12 +30802,16 @@
       </c>
       <c r="I91" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J91" s="18" t="n"/>
       <c r="K91" s="18" t="n"/>
-      <c r="L91" s="18" t="n"/>
+      <c r="L91" s="18" t="inlineStr">
+        <is>
+          <t>NK extraction form built from the 22 June template; review-team confirmation pending</t>
+        </is>
+      </c>
       <c r="M91" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -30798,12 +30859,16 @@
       </c>
       <c r="I92" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J92" s="18" t="n"/>
       <c r="K92" s="18" t="n"/>
-      <c r="L92" s="18" t="n"/>
+      <c r="L92" s="18" t="inlineStr">
+        <is>
+          <t>Jeremy/review team to review and adjust the form; Sean approval remains pending</t>
+        </is>
+      </c>
       <c r="M92" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -30851,12 +30916,16 @@
       </c>
       <c r="I93" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete / Under Review</t>
         </is>
       </c>
       <c r="J93" s="18" t="n"/>
       <c r="K93" s="18" t="n"/>
-      <c r="L93" s="18" t="n"/>
+      <c r="L93" s="18" t="inlineStr">
+        <is>
+          <t>Meghan built and tested the form on several full-text articles</t>
+        </is>
+      </c>
       <c r="M93" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -30904,12 +30973,16 @@
       </c>
       <c r="I94" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J94" s="18" t="n"/>
       <c r="K94" s="18" t="n"/>
-      <c r="L94" s="18" t="n"/>
+      <c r="L94" s="18" t="inlineStr">
+        <is>
+          <t>Initial testing was successful; final review and adjustments remain</t>
+        </is>
+      </c>
       <c r="M94" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -32380,7 +32453,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abstract screening complete; reconciled 77-reference full-text set approved</t>
+          <t>Abstract screening complete; full-text plan under review following reviewer withdrawal and record-set differences</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -32465,7 +32538,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Meghan cleared both arms to use the 77-reference set and will update Nested Knowledge</t>
+          <t>Michelle withdrew; Murali will be the sole conventional reviewer; follow-up call requested to resolve record differences and next steps</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -32482,7 +32555,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Send the abstract survey, confirm at least two conventional reviewers and complete both full-text arms</t>
+          <t>Hold the follow-up call, confirm the one-reviewer arrangement and resolve record differences before screening continues</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -32516,7 +32589,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Full-text set finalized; NK update and conventional-reviewer coverage pending</t>
+          <t>Seventy-seven-reference set approved; reviewer structure and screening-record differences remain under review</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -32572,7 +32645,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -33016,7 +33089,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Ready / Under Review</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -33026,7 +33099,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Conventional arm can proceed; NK update pending for the AI arm; at least two conventional reviewers required</t>
+          <t>Follow-up call requested; confirm record differences and the one-reviewer exception before both arms proceed</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -33384,12 +33457,16 @@
       </c>
       <c r="I53" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J53" s="18" t="n"/>
       <c r="K53" s="18" t="n"/>
-      <c r="L53" s="18" t="n"/>
+      <c r="L53" s="18" t="inlineStr">
+        <is>
+          <t>Michelle withdrew; Murali remains the sole conventional reviewer under the exception communicated on 1 October</t>
+        </is>
+      </c>
       <c r="M53" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -34879,14 +34956,14 @@
       </c>
       <c r="I80" s="18" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J80" s="18" t="n"/>
       <c r="K80" s="18" t="n"/>
       <c r="L80" s="18" t="inlineStr">
         <is>
-          <t>Conventional screening cleared for 77 references; confirm at least two reviewers</t>
+          <t>Murali is the sole conventional reviewer; confirm the arrangement and strict blinding during the follow-up</t>
         </is>
       </c>
       <c r="M80" s="18" t="inlineStr">
@@ -36871,12 +36948,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Human Milk 77-reference full-text set approved</t>
+          <t>Human Milk follow-up call requested</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -36891,12 +36968,12 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Both arms will use 77 references; Michelle cannot continue screening and conventional-reviewer coverage must be confirmed</t>
+          <t>Call requested with Murali, Mohan, Gerald and the study team to resolve record differences and next steps</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -36906,7 +36983,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>Send the survey, confirm two conventional reviewers and complete full-text screening</t>
+          <t>Confirm the reviewer arrangement and record set before full-text screening continues</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -36952,7 +37029,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Complete full-text screening on the 77-reference set</t>
+          <t>Resolve reviewer structure and screening-record differences</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -36972,12 +37049,12 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Use the approved 77-reference set; confirm two conventional reviewers and document the source-set discrepancies</t>
+          <t>Follow-up call pending; confirm the one-reviewer exception, strict blinding and the final record set</t>
         </is>
       </c>
     </row>
@@ -41800,7 +41877,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M130"/>
+  <dimension ref="A1:M126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="14" customWidth="1" style="29" min="1" max="1"/>
@@ -41822,11 +41899,6 @@
           <t>phase1-08 LNS | Dashboard Content Sheet</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>phase1-09 Orthodontic Retention | Dashboard Content Sheet</t>
-        </is>
-      </c>
       <c r="K1" s="18" t="n"/>
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
@@ -41945,7 +42017,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Initial onboarding completed; reviewer-allocation model awaiting confirmation</t>
+          <t>Onboarding in progress; non-overlapping reviewer groups required and updated searches being arranged</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -41979,7 +42051,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Laser AI</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -42013,7 +42085,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Approximately 300–500 references expected; searches planned for November</t>
+          <t>About 300–500 references expected; separate reviewer groups required; Irma will update Embase from April 2022 onward</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -42030,7 +42102,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Initial onboarding completed; crossed reviewer-allocation model proposed and awaiting Gerald's confirmation</t>
+          <t>Gerald rejected crossed allocation; Conchita agreed to follow the protocol; both groups must receive identical records</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -42047,7 +42119,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Gerald to confirm the crossed reviewer allocation; then finalize team split, tool assignment and setup</t>
+          <t>Finalize two non-overlapping groups, complete searches, share RIS files and configure Laser AI</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -42081,7 +42153,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Final eighth review; onboarding completed and setup depends on reviewer-allocation confirmation</t>
+          <t>Final eighth review; reviewer model resolved, but team names and updated searches remain pending</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -42137,7 +42209,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -42930,7 +43002,7 @@
       </c>
       <c r="I52" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J52" s="18" t="n"/>
@@ -43258,7 +43330,7 @@
       <c r="K58" s="18" t="n"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>All available search results received; seven databases were inaccessible</t>
+          <t>Previous searches cover through 27 April 2022; updated search results are not yet available</t>
         </is>
       </c>
       <c r="M58" s="18" t="inlineStr">
@@ -43308,14 +43380,14 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J59" s="18" t="n"/>
       <c r="K59" s="18" t="n"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>Kanza approved the decision flow on 29 September</t>
+          <t>Previous review and Embase strategy shared; updated Embase search will run from April 2022 onward</t>
         </is>
       </c>
       <c r="M59" s="18" t="inlineStr">
@@ -43528,7 +43600,7 @@
       <c r="K63" s="18" t="n"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>All accessible searches uploaded; 16,891 citations after deduplication</t>
+          <t>Awaiting completed searches and finalized separate reviewer groups</t>
         </is>
       </c>
       <c r="M63" s="18" t="inlineStr">
@@ -43585,7 +43657,7 @@
       <c r="K64" s="18" t="n"/>
       <c r="L64" s="18" t="inlineStr">
         <is>
-          <t>Decision flow approved; access provided and citations can be distributed</t>
+          <t>Not yet validated; two non-overlapping reviewer groups must be finalized first</t>
         </is>
       </c>
       <c r="M64" s="18" t="inlineStr">
@@ -46211,10 +46283,6 @@
         </is>
       </c>
     </row>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
@@ -46360,7 +46428,6 @@
         </is>
       </c>
     </row>
-    <row r="123"/>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
@@ -46447,12 +46514,12 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Reviewer-allocation confirmation needed before setup</t>
+          <t>Separate reviewer groups and updated searches required before setup</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Reviewer allocation is not yet confirmed.</t>
+          <t>Crossed allocation was rejected; distinct reviewer groups must now be named and confirmed</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -46462,37 +46529,37 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Gerald / Krishna</t>
+          <t>Review Team / Irma / Krishna</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>December 2026</t>
+          <t>Before setup</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>Finalize crossed reviewer allocation, team split and tool assignment before setup.</t>
+          <t>Finalize two separate groups, complete the database searches and share the resulting RIS files</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>Setup cannot proceed until allocation and tool plan are confirmed.</t>
+          <t>Laser AI setup cannot proceed until the team split and complete search set are available</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Project tracking</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -46501,10 +46568,6 @@
         </is>
       </c>
     </row>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -46778,12 +46841,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Pilot 2 completed, including conflict resolution; Bi 2025 omission remains documented</t>
+          <t>Pilot 2 and conflict resolution complete; James’s senior-reviewer responses are pending and downstream-impact work has started</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Complete the time-on-task, fully automated and downstream-impact analyses</t>
+          <t>Obtain James’s responses, reschedule the automated-analysis meeting around 20 October and continue downstream-impact analysis</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
@@ -46830,7 +46893,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Analysis underway; corrective validation and final reconciliation in progress</t>
+          <t>Analysis and final reconciliation underway; report-to-trial mapping is being clarified</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -46850,17 +46913,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Updated decisions received for all 139 conventional records; 25 full texts are ready in NK; time-on-task data are available</t>
+          <t>All 139 decisions received; DOI mapping added; ICONIC Advance 1/2 must be separate trials and ICONIC Lead is excluded</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Complete the 25-record NK screening, rerun the comparison and save the finalized export</t>
+          <t>Complete the 25-record NK screening, finalize report-to-trial mapping and rerun the comparison</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Overdue / confirmation required</t>
+          <t>2026-10-07 — accuracy meeting</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -47185,7 +47248,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Abstract outputs reconciled; both full-text arms cleared to proceed; missing PDFs remain</t>
+          <t>Full-text screening underway; missing PDFs remain; NK extraction form prepared for review</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -47205,12 +47268,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>NK updated with Covidence-only citations; Meghan confirmed both arms are aligned</t>
+          <t>Both arms aligned; NK extraction form built from the 22 June template and tested on several articles</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Retrieve missing PDFs, complete both full-text arms and record time</t>
+          <t>Retrieve missing PDFs, complete both full-text arms and review/approve the NK extraction form</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -47257,7 +47320,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Abstract screening complete; reconciled 77-reference full-text set approved</t>
+          <t>Abstract screening complete; full-text plan under review following reviewer withdrawal and record-set differences</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -47277,12 +47340,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Both arms will use the 77-reference set; the NK update and conventional-reviewer coverage remain pending</t>
+          <t>Michelle withdrew; Murali remains the sole conventional reviewer under the exception communicated on 1 October; follow-up call requested</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Send the abstract survey, confirm at least two conventional reviewers and complete full-text screening</t>
+          <t>Hold the follow-up call, confirm the reviewer arrangement and resolve record-set differences before full-text screening continues</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -47401,7 +47464,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Initial onboarding completed; reviewer-allocation model awaiting confirmation</t>
+          <t>Onboarding in progress; non-overlapping reviewer groups required and updated searches being arranged</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -47411,7 +47474,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Laser AI</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -47421,12 +47484,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Approximately 300–500 references expected; searches planned for November</t>
+          <t>Crossed allocation rejected; both groups must receive the same records; Irma will update Embase from April 2022 onward</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Gerald to confirm the crossed reviewer allocation; then finalize team split, tool assignment and setup</t>
+          <t>Finalize two non-overlapping reviewer groups, complete searches and configure Laser AI</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -51028,12 +51091,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Mid April to End June</t>
+          <t>Mid April to mid-December 2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Focus on completing active reviews while onboarding the final Orthodontic Retention review</t>
+          <t>Complete active reviews and onboard Orthodontic Retention; project-management support confirmed at 20% FTE through mid-December</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -51060,7 +51123,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>BP adjudication complete; time-on-task, automated and downstream-impact analyses underway; no interim report or mid-term review is planned</t>
+          <t>BP adjudication complete; time-on-task and downstream-impact analyses underway; automated-analysis meeting to be rescheduled around 20 October; Psoriasis accuracy review scheduled for 7 October</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -51197,7 +51260,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Krishna / Core Team</t>
+          <t>Current source of truth; review folders were re-shared with Noosheen and full-text PDFs will be added as each adjudication completes</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -61222,7 +61285,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Panel completed the first adjudication review, including conflict resolution; Bi 2025 remains documented</t>
+          <t>Adjudication complete; questions sent to James on 1 October; Doreen connected with Jo-Ana and Max on 4 October</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -61239,7 +61302,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete the time-on-task, fully automated and downstream-impact analyses</t>
+          <t>Obtain James’s responses, reschedule the automated-analysis meeting around 20 October and continue downstream-impact work</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -61273,7 +61336,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Bi 2025 remains documented; a direct invitation and Teams link were sent for the automated-analysis meeting</t>
+          <t>Automated meeting postponed at Paweł’s request; target around 20 October; James’s response remains pending</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -61329,7 +61392,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -64973,14 +65036,14 @@
       </c>
       <c r="I106" s="18" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Rescheduling</t>
         </is>
       </c>
       <c r="J106" s="18" t="n"/>
       <c r="K106" s="18" t="n"/>
       <c r="L106" s="18" t="inlineStr">
         <is>
-          <t>Fully automated analysis meeting scheduled for 1 October; direct invitation and Teams link sent</t>
+          <t>Meeting canceled; Paweł requested 15–16 or preferably 20–21 October; plan around 20 October</t>
         </is>
       </c>
       <c r="M106" s="18" t="inlineStr">
@@ -65197,14 +65260,14 @@
       </c>
       <c r="I110" s="18" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J110" s="18" t="n"/>
       <c r="K110" s="18" t="n"/>
       <c r="L110" s="18" t="inlineStr">
         <is>
-          <t>Downstream-impact analysis meeting scheduled for 2 October</t>
+          <t>Downstream work started; Doreen was connected with Jo-Ana and Max on 4 October to discuss meta-analysis status and plans</t>
         </is>
       </c>
       <c r="M110" s="18" t="inlineStr">
@@ -66551,7 +66614,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Analysis underway; corrective validation and final reconciliation in progress</t>
+          <t>Analysis and final reconciliation underway; report-to-trial mapping being clarified</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -66619,7 +66682,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Analysis: corrective validation in progress</t>
+          <t>Conventional corrective screening complete; 25-record NK screening remains pending; accuracy meeting scheduled</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -66636,7 +66699,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Psoriasis is currently the complete PDF package available to the extension team</t>
+          <t>Sivem added DOI mapping; ICONIC Advance 1/2 are separate trials and ICONIC Lead is excluded</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -66653,7 +66716,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete the NK corrective screening, rerun the comparison and save the finalized export</t>
+          <t>Complete the 25-record NK screening, finalize report-to-trial mapping and rerun the comparison</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -66670,7 +66733,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Overdue / confirmation required</t>
+          <t>2026-10-07 — accuracy meeting</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -66743,7 +66806,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -66990,7 +67053,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Consolidated full-text package available directly from NK; duplicate records remain documented</t>
+          <t>Decisions received; 25 NK full texts ready; DOI mapping added; ICONIC Advance 1/2 separate; ICONIC Lead excluded</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -67248,7 +67311,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Nested Knowledge data-extraction setup and repeated-run validation analysis are underway.</t>
+          <t>Sean is reconciling conventional report IDs with the search set; accuracy meeting scheduled for 7 October</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -70191,7 +70254,11 @@
       </c>
       <c r="J102" s="18" t="n"/>
       <c r="K102" s="18" t="n"/>
-      <c r="L102" s="18" t="n"/>
+      <c r="L102" s="18" t="inlineStr">
+        <is>
+          <t>Validation blocked by the 25-record NK screening; conventional report mapping is being reconciled</t>
+        </is>
+      </c>
       <c r="M102" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -70244,7 +70311,11 @@
       </c>
       <c r="J103" s="18" t="n"/>
       <c r="K103" s="18" t="n"/>
-      <c r="L103" s="18" t="n"/>
+      <c r="L103" s="18" t="inlineStr">
+        <is>
+          <t>Prepare after the NK screening and report-to-trial reconciliation are finalized</t>
+        </is>
+      </c>
       <c r="M103" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -70564,7 +70635,7 @@
       <c r="K109" s="18" t="n"/>
       <c r="L109" s="18" t="inlineStr">
         <is>
-          <t>Psoriasis time-on-task data received; analysis underway</t>
+          <t>Time-on-task data received; screening-accuracy discussion scheduled for 7 October</t>
         </is>
       </c>
       <c r="M109" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Update dashboard through October 9
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2402,7 +2402,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Full-text screening underway; six oversized-PDF exceptions identified</t>
+          <t>Full-text screening underway; extraction setup started; final data-item list pending</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2470,7 +2470,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Full-text screening underway</t>
+          <t>Full-text screening underway; Laser AI extraction setup is being prepared</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Kate successfully distributed all 138 records; six oversized PDFs cannot receive model suggestions</t>
+          <t>Six PDFs are being screened without model suggestions; Sean requested the latest data-item list</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete both full-text arms and document the six exceptions in the comparison</t>
+          <t>Complete full-text screening, provide the final data items and finish extraction setup</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2538,7 +2538,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Screening underway; six records will be evaluated without AI model suggestions</t>
+          <t>Screening continues; extraction setup is waiting for the final data-item list</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2594,7 +2594,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3084,7 +3084,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Preparation underway</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Meghan is setting up extraction in Laser AI; Kate and Bec were asked for the latest data items</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -3801,7 +3806,11 @@
       </c>
       <c r="J60" s="18" t="n"/>
       <c r="K60" s="18" t="n"/>
-      <c r="L60" s="18" t="n"/>
+      <c r="L60" s="18" t="inlineStr">
+        <is>
+          <t>Sean requested the latest data-item list on 8 October</t>
+        </is>
+      </c>
       <c r="M60" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3854,7 +3863,11 @@
       </c>
       <c r="J61" s="18" t="n"/>
       <c r="K61" s="18" t="n"/>
-      <c r="L61" s="18" t="n"/>
+      <c r="L61" s="18" t="inlineStr">
+        <is>
+          <t>Field-for-field comparability requires confirmation against the final list</t>
+        </is>
+      </c>
       <c r="M61" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3907,7 +3920,11 @@
       </c>
       <c r="J62" s="18" t="n"/>
       <c r="K62" s="18" t="n"/>
-      <c r="L62" s="18" t="n"/>
+      <c r="L62" s="18" t="inlineStr">
+        <is>
+          <t>Final approval follows receipt of the updated data items</t>
+        </is>
+      </c>
       <c r="M62" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -5487,12 +5504,16 @@
       </c>
       <c r="I91" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J91" s="18" t="n"/>
       <c r="K91" s="18" t="n"/>
-      <c r="L91" s="18" t="n"/>
+      <c r="L91" s="18" t="inlineStr">
+        <is>
+          <t>Latest extraction items requested from Kate and Bec</t>
+        </is>
+      </c>
       <c r="M91" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -5593,12 +5614,16 @@
       </c>
       <c r="I93" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J93" s="18" t="n"/>
       <c r="K93" s="18" t="n"/>
-      <c r="L93" s="18" t="n"/>
+      <c r="L93" s="18" t="inlineStr">
+        <is>
+          <t>Meghan has started configuring the Laser AI extraction form</t>
+        </is>
+      </c>
       <c r="M93" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -12690,7 +12715,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Current review-specific folders contain RIS files and protocols; Sean will add full-text PDFs after each review’s adjudication</t>
+          <t>Noosheen’s NK and Laser AI access is working; folder organization continues and finalized PDFs will be added after adjudication</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -12733,7 +12758,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -22332,7 +22357,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Converted to phase1-07; follow-up call requested after reviewer withdrawal and screening-record differences</t>
+          <t>Converted to phase1-07; supplemental abstract screening underway after master-file harmonization</t>
         </is>
       </c>
       <c r="E12" s="17" t="inlineStr">
@@ -22347,12 +22372,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Full-text plan under review; target remains 31 October</t>
+          <t>508 Covidence and one NK citation require screening before full-text harmonization</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Seventy-seven-reference set approved; Michelle withdrew; Murali is the sole conventional reviewer; follow-up pending</t>
+          <t>Master RIS contains 4,173 citations; final full-text set will be established after supplemental screening</t>
         </is>
       </c>
       <c r="I12" s="17" t="inlineStr">
@@ -22854,7 +22879,7 @@
       </c>
       <c r="D28" s="17" t="inlineStr">
         <is>
-          <t>Converted to phase1-06; full-text screening underway and NK extraction form prepared</t>
+          <t>Converted to phase1-06; full-text screening underway and extraction form reviewed/revised</t>
         </is>
       </c>
       <c r="E28" s="17" t="inlineStr">
@@ -22869,12 +22894,12 @@
       </c>
       <c r="G28" s="17" t="inlineStr">
         <is>
-          <t>Full-text screening underway; review and approve the NK extraction form before extraction</t>
+          <t>Full-text screening and extraction calibration can proceed; missing PDFs remain</t>
         </is>
       </c>
       <c r="H28" s="17" t="inlineStr">
         <is>
-          <t>Both arms aligned; missing PDFs remain; Meghan built and tested the NK extraction form</t>
+          <t>Jeremy reviewed and revised the form and received instructions for running the AI extraction</t>
         </is>
       </c>
       <c r="I28" s="17" t="inlineStr">
@@ -23177,7 +23202,7 @@
       </c>
       <c r="D35" s="17" t="inlineStr">
         <is>
-          <t>Converted to phase1-09; separate reviewer groups required and updated searches being arranged</t>
+          <t>Converted to phase1-09; searches received, consolidation underway and NK training scheduled</t>
         </is>
       </c>
       <c r="E35" s="17" t="inlineStr">
@@ -23192,12 +23217,12 @@
       </c>
       <c r="G35" s="17" t="inlineStr">
         <is>
-          <t>Search updates being arranged; Irma will update Embase from April 2022 onward</t>
+          <t>Consolidate/deduplicate the search files; NK training scheduled for 12 October</t>
         </is>
       </c>
       <c r="H35" s="17" t="inlineStr">
         <is>
-          <t>Crossed allocation rejected; both groups must receive the same records; finalize separate reviewer groups before setup</t>
+          <t>Embase and ClinicalTrials.gov RIS files received; other searches completed; final groups and deduplicated RIS pending</t>
         </is>
       </c>
       <c r="I35" s="17" t="inlineStr">
@@ -26901,7 +26926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="14" customWidth="1" style="29" min="1" max="2"/>
@@ -27590,6 +27615,68 @@
       <c r="J12" t="inlineStr">
         <is>
           <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>mtg-12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>11:00 AM–12:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>4:00–5:00 PM BST</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Nested Knowledge Training – Orthodontic Retention</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>NK training and initial project-setup guidance; 10:00–11:00 AM Central / 5:00–6:00 PM Madrid</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Ranita Tarchand / Orthodontic review team / Krishna</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>phase1-09</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -27758,7 +27845,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Full-text screening underway; missing PDFs remain; NK extraction form prepared</t>
+          <t>Full-text screening underway; missing PDFs remain; extraction form reviewed and revised</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -27826,7 +27913,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Both full-text arms progressing; NK extraction form built and tested</t>
+          <t>Both full-text arms progressing; extraction form reviewed and ready for calibration</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -27843,7 +27930,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>NK form built from the 22 June Excel template; Jeremy asked to review and adjust it</t>
+          <t>Jeremy reviewed the form, made minor revisions and received instructions for running and revising the AI output</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -27860,7 +27947,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Retrieve missing PDFs, finish both full-text arms, review the NK extraction form and record time</t>
+          <t>Retrieve missing PDFs, complete full-text screening and undertake calibration/AI extraction</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -27894,7 +27981,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Meghan confirmed both arms are aligned and cleared to proceed; missing PDFs remain</t>
+          <t>Both arms remain active; extraction can be calibrated while missing PDFs are retrieved</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -27950,7 +28037,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -28231,7 +28318,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Received</t>
+          <t>Form reviewed and revised; ready for calibration</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -28411,7 +28498,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Meghan built and tested the NK extraction form; review-team confirmation remains pending</t>
+          <t>Jeremy reviewed and revised the form; AI-extraction instructions were provided</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -30802,14 +30889,14 @@
       </c>
       <c r="I91" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Complete / Under Review</t>
         </is>
       </c>
       <c r="J91" s="18" t="n"/>
       <c r="K91" s="18" t="n"/>
       <c r="L91" s="18" t="inlineStr">
         <is>
-          <t>NK extraction form built from the 22 June template; review-team confirmation pending</t>
+          <t>Jeremy reviewed and revised the form; calibration may identify further adjustments</t>
         </is>
       </c>
       <c r="M91" s="18" t="inlineStr">
@@ -30866,7 +30953,7 @@
       <c r="K92" s="18" t="n"/>
       <c r="L92" s="18" t="inlineStr">
         <is>
-          <t>Jeremy/review team to review and adjust the form; Sean approval remains pending</t>
+          <t>Review-team revisions completed; final Sean approval remains pending</t>
         </is>
       </c>
       <c r="M92" s="18" t="inlineStr">
@@ -30923,7 +31010,7 @@
       <c r="K93" s="18" t="n"/>
       <c r="L93" s="18" t="inlineStr">
         <is>
-          <t>Meghan built and tested the form on several full-text articles</t>
+          <t>Form tested, reviewed and revised; instructions for running the AI were provided</t>
         </is>
       </c>
       <c r="M93" s="18" t="inlineStr">
@@ -30980,7 +31067,7 @@
       <c r="K94" s="18" t="n"/>
       <c r="L94" s="18" t="inlineStr">
         <is>
-          <t>Initial testing was successful; final review and adjustments remain</t>
+          <t>Ready for calibration; the AI must be rerun if the form changes</t>
         </is>
       </c>
       <c r="M94" s="18" t="inlineStr">
@@ -31083,12 +31170,16 @@
       </c>
       <c r="I96" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="J96" s="18" t="n"/>
       <c r="K96" s="18" t="n"/>
-      <c r="L96" s="18" t="n"/>
+      <c r="L96" s="18" t="inlineStr">
+        <is>
+          <t>Jeremy received instructions for running and manually revising the AI extraction</t>
+        </is>
+      </c>
       <c r="M96" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -32453,7 +32544,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abstract screening complete; full-text plan under review following reviewer withdrawal and record-set differences</t>
+          <t>Supplemental abstract screening underway after master-file harmonization; full-text baseline pending</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -32521,7 +32612,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Both abstract arms complete; reconciled full-text set expanded to 77 references</t>
+          <t>Master file created with 4,173 citations; 508 Covidence and one NK citation require screening</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -32538,7 +32629,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Michelle withdrew; Murali will be the sole conventional reviewer; follow-up call requested to resolve record differences and next steps</t>
+          <t>Covidence deduplicated the master file to 2,138 records and NK to 2,028; the earlier 77-record set is no longer final</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -32555,7 +32646,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Hold the follow-up call, confirm the one-reviewer arrangement and resolve record differences before screening continues</t>
+          <t>Complete the supplemental screening and establish a harmonized full-text baseline</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -32589,7 +32680,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Seventy-seven-reference set approved; reviewer structure and screening-record differences remain under review</t>
+          <t>Platform-specific deduplication produced different sets; full-text screening is blocked pending harmonization</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -32645,7 +32736,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -32761,7 +32852,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Ready / Under Review</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -32860,7 +32951,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Deduplicated RIS/search file received - 2,053 records.</t>
+          <t>Master RIS containing 4,173 undeduplicated citations uploaded to SharePoint</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -32882,7 +32973,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Seventy-seven full-text references approved; PDF collection and NK updating remain</t>
+          <t>Final full-text/PDF set pending supplemental screening and harmonization</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -33067,12 +33158,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Both abstract arms complete; Mohan screened all 2,024 NK records</t>
+          <t>Murali must screen 508 additional Covidence records and Mohan one additional NK record</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -33089,7 +33180,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -33099,7 +33190,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Follow-up call requested; confirm record differences and the one-reviewer exception before both arms proceed</t>
+          <t>Nicholas/Meghan will establish the harmonized full-text baseline after supplemental screening</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -34129,14 +34220,14 @@
       </c>
       <c r="I65" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J65" s="18" t="n"/>
       <c r="K65" s="18" t="n"/>
       <c r="L65" s="18" t="inlineStr">
         <is>
-          <t>Conventional abstract screening complete; 59 records advanced</t>
+          <t>Murali to screen 508 additional Covidence citations; Covidence AI decisions are disabled</t>
         </is>
       </c>
       <c r="M65" s="18" t="inlineStr">
@@ -34186,14 +34277,14 @@
       </c>
       <c r="I66" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J66" s="18" t="n"/>
       <c r="K66" s="18" t="n"/>
       <c r="L66" s="18" t="inlineStr">
         <is>
-          <t>AI-assisted abstract screening complete; 42 records advanced</t>
+          <t>Mohan to screen one additional Nested Knowledge citation</t>
         </is>
       </c>
       <c r="M66" s="18" t="inlineStr">
@@ -34243,14 +34334,14 @@
       </c>
       <c r="I67" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J67" s="18" t="n"/>
       <c r="K67" s="18" t="n"/>
       <c r="L67" s="18" t="inlineStr">
         <is>
-          <t>AI-arm output exported; 16 records were unique to the AI arm</t>
+          <t>Re-export the final NK output after the additional citation is screened</t>
         </is>
       </c>
       <c r="M67" s="18" t="inlineStr">
@@ -34300,14 +34391,14 @@
       </c>
       <c r="I68" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J68" s="18" t="n"/>
       <c r="K68" s="18" t="n"/>
       <c r="L68" s="18" t="inlineStr">
         <is>
-          <t>RIS and Excel files sent to Michelle and copied to the project team</t>
+          <t>Share the harmonized output after supplemental screening</t>
         </is>
       </c>
       <c r="M68" s="18" t="inlineStr">
@@ -34626,14 +34717,14 @@
       </c>
       <c r="I74" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J74" s="18" t="n"/>
       <c r="K74" s="18" t="n"/>
       <c r="L74" s="18" t="inlineStr">
         <is>
-          <t>Reconciled 77-reference full-text set approved</t>
+          <t>Final full-text set will be established after the two abstract outputs are compared</t>
         </is>
       </c>
       <c r="M74" s="18" t="inlineStr">
@@ -34842,14 +34933,14 @@
       </c>
       <c r="I78" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="J78" s="18" t="n"/>
       <c r="K78" s="18" t="n"/>
       <c r="L78" s="18" t="inlineStr">
         <is>
-          <t>Meghan will update Nested Knowledge to the 77-reference set</t>
+          <t>Await the harmonized full-text baseline</t>
         </is>
       </c>
       <c r="M78" s="18" t="inlineStr">
@@ -34899,14 +34990,14 @@
       </c>
       <c r="I79" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="J79" s="18" t="n"/>
       <c r="K79" s="18" t="n"/>
       <c r="L79" s="18" t="inlineStr">
         <is>
-          <t>Validate the 77-reference set after the NK update</t>
+          <t>Validate the harmonized set after supplemental screening</t>
         </is>
       </c>
       <c r="M79" s="18" t="inlineStr">
@@ -34956,14 +35047,14 @@
       </c>
       <c r="I80" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="J80" s="18" t="n"/>
       <c r="K80" s="18" t="n"/>
       <c r="L80" s="18" t="inlineStr">
         <is>
-          <t>Murali is the sole conventional reviewer; confirm the arrangement and strict blinding during the follow-up</t>
+          <t>Conventional full-text screening waits for the harmonized baseline</t>
         </is>
       </c>
       <c r="M80" s="18" t="inlineStr">
@@ -35013,14 +35104,14 @@
       </c>
       <c r="I81" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="J81" s="18" t="n"/>
       <c r="K81" s="18" t="n"/>
       <c r="L81" s="18" t="inlineStr">
         <is>
-          <t>Update NK to the approved 77-reference set before AI full-text screening</t>
+          <t>NK full-text screening waits for the harmonized baseline</t>
         </is>
       </c>
       <c r="M81" s="18" t="inlineStr">
@@ -36810,7 +36901,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Complete full-text screening using the 77-reference set</t>
+          <t>Complete supplemental abstract screening and establish the harmonized full-text set</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Murali / Mohan / Nicholas Henschke / Meghan</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -36830,12 +36926,12 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>Full-text screening</t>
+          <t>Supplemental abstract screening and reconciliation</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Both arms cleared to use 77 references; send the survey and confirm conventional-reviewer coverage</t>
+          <t>Murali screens 508 records and Mohan one record; notify Nicholas and Meghan when complete</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -36845,7 +36941,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -36948,32 +37044,37 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Human Milk follow-up call requested</t>
+          <t>Human Milk master-file recalibration</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Murali / Mohan / Meghan / Nicholas Henschke / Sean / Krishna</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Meghan / Murali / Mohan / Krishna</t>
+          <t>Murali / Mohan / Nicholas Henschke / Meghan</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>2026-10-31</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Call requested with Murali, Mohan, Gerald and the study team to resolve record differences and next steps</t>
+          <t>Master file contains 4,173 citations; Covidence requires 508 additional decisions and NK requires one</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -36983,7 +37084,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>Confirm the reviewer arrangement and record set before full-text screening continues</t>
+          <t>Complete supplemental screening and establish the harmonized full-text set</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -37029,7 +37130,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Resolve reviewer structure and screening-record differences</t>
+          <t>Complete supplemental abstract screening and harmonize the full-text baseline</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -37039,7 +37140,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Murali / Mohan / Meghan / Krishna</t>
+          <t>Murali / Mohan / Nicholas Henschke / Meghan</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -37049,12 +37150,12 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Follow-up call pending; confirm the one-reviewer exception, strict blinding and the final record set</t>
+          <t>Full-text screening cannot proceed until the 508 Covidence and one NK citation are screened and compared</t>
         </is>
       </c>
     </row>
@@ -41896,7 +41997,7 @@
     <row r="1" ht="18" customHeight="1" s="29">
       <c r="A1" s="28" t="inlineStr">
         <is>
-          <t>phase1-08 LNS | Dashboard Content Sheet</t>
+          <t>phase1-09 Orthodontic Retention | Dashboard Content Sheet</t>
         </is>
       </c>
       <c r="K1" s="18" t="n"/>
@@ -42017,7 +42118,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Onboarding in progress; non-overlapping reviewer groups required and updated searches being arranged</t>
+          <t>Search files received and consolidation underway; NK training scheduled for 12 October</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -42051,7 +42152,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Laser AI</t>
+          <t>Nested Knowledge</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -42085,7 +42186,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>About 300–500 references expected; separate reviewer groups required; Irma will update Embase from April 2022 onward</t>
+          <t>Embase and ClinicalTrials.gov RIS files received; other database searches completed; consolidation/deduplication underway</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -42102,7 +42203,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Gerald rejected crossed allocation; Conchita agreed to follow the protocol; both groups must receive identical records</t>
+          <t>Crossed allocation rejected and protocol accepted; Irma supplied the updated search files</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -42119,7 +42220,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Finalize two non-overlapping groups, complete searches, share RIS files and configure Laser AI</t>
+          <t>Finalize the two groups, consolidate/deduplicate the searches, attend NK training and configure the project</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -42136,7 +42237,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>December 2026</t>
+          <t>2026-10-12 — NK training</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -42153,7 +42254,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Final eighth review; reviewer model resolved, but team names and updated searches remain pending</t>
+          <t>Search files received and training scheduled; reviewer-group names and final deduplicated RIS remain pending</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -42209,7 +42310,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -42284,7 +42385,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Initial onboarding completed; reviewer allocation awaiting Gerald confirmation</t>
+          <t>Reviewer-allocation method resolved; search consolidation and training underway</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -42311,7 +42412,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Tool assignment and setup pending reviewer allocation</t>
+          <t>Nested Knowledge selected; training scheduled and final RIS pending</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -42429,17 +42530,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Searches planned for November</t>
+          <t>Embase and ClinicalTrials.gov RIS files received; remaining searches completed; consolidation underway</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Approximately 300-500 references expected</t>
+          <t>Final reference count will be available after consolidation and deduplication</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -42640,7 +42741,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Initial onboarding completed; reviewer allocation awaiting Gerald confirmation</t>
+          <t>Reviewer model resolved; searches received; NK training scheduled for 12 October</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -42668,7 +42769,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Searches expected in November</t>
+          <t>Search consolidation and deduplication underway</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -43009,7 +43110,7 @@
       <c r="K52" s="18" t="n"/>
       <c r="L52" s="18" t="inlineStr">
         <is>
-          <t>Tool allocation to be confirmed after onboarding.</t>
+          <t>Nested Knowledge allocated</t>
         </is>
       </c>
       <c r="M52" s="18" t="inlineStr">
@@ -43064,7 +43165,11 @@
       </c>
       <c r="J53" s="18" t="n"/>
       <c r="K53" s="18" t="n"/>
-      <c r="L53" s="18" t="inlineStr"/>
+      <c r="L53" s="18" t="inlineStr">
+        <is>
+          <t>Two non-overlapping groups must be named before screening setup</t>
+        </is>
+      </c>
       <c r="M53" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -43323,14 +43428,14 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J58" s="18" t="n"/>
       <c r="K58" s="18" t="n"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>Previous searches cover through 27 April 2022; updated search results are not yet available</t>
+          <t>Updated Embase and ClinicalTrials.gov RIS files received; consolidated RIS remains pending</t>
         </is>
       </c>
       <c r="M58" s="18" t="inlineStr">
@@ -43593,14 +43698,14 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J63" s="18" t="n"/>
       <c r="K63" s="18" t="n"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Awaiting completed searches and finalized separate reviewer groups</t>
+          <t>NK training scheduled; setup awaits the consolidated RIS and reviewer groups</t>
         </is>
       </c>
       <c r="M63" s="18" t="inlineStr">
@@ -43650,14 +43755,14 @@
       </c>
       <c r="I64" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J64" s="18" t="n"/>
       <c r="K64" s="18" t="n"/>
       <c r="L64" s="18" t="inlineStr">
         <is>
-          <t>Not yet validated; two non-overlapping reviewer groups must be finalized first</t>
+          <t>Validate after NK training, final RIS import and group confirmation</t>
         </is>
       </c>
       <c r="M64" s="18" t="inlineStr">
@@ -46234,7 +46339,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Confirm crossed reviewer allocation and complete review team split</t>
+          <t>Finalize non-overlapping reviewer groups and consolidate search results</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -46244,7 +46349,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -46259,12 +46364,12 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Reviewer-allocation confirmation</t>
+          <t>Reviewer names and final deduplicated RIS</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Initial onboarding completed; crossed reviewer allocation awaits Gerald's confirmation</t>
+          <t>Crossed allocation rejected; searches received; NK training scheduled for 12 October</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -46274,7 +46379,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -46374,12 +46479,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Orthodontic Retention added as eighth review</t>
+          <t>Orthodontic searches received and NK training scheduled</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -46399,12 +46504,12 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Initial onboarding completed; Gerald to confirm crossed reviewer allocation before setup proceeds</t>
+          <t>Embase/ClinicalTrials.gov files received; consolidation underway; NK training scheduled for 12 October</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -46414,7 +46519,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>Confirm crossed reviewer allocation and complete review team split</t>
+          <t>Finalize groups, consolidate searches and configure Nested Knowledge</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -46841,12 +46946,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Pilot 2 and conflict resolution complete; James’s senior-reviewer responses are pending and downstream-impact work has started</t>
+          <t>Adjudication complete; James’s responses remain pending; downstream-impact work continues and analysis-support requests were sent</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Obtain James’s responses, reschedule the automated-analysis meeting around 20 October and continue downstream-impact analysis</t>
+          <t>Obtain James’s responses, schedule the adjudication-analysis discussion and confirm automated-analysis statistical support</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
@@ -46893,7 +46998,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Analysis and final reconciliation underway; report-to-trial mapping is being clarified</t>
+          <t>Analysis and reconciliation underway; 25-record NK screening and five-report timing clarification remain</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -46913,17 +47018,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>All 139 decisions received; DOI mapping added; ICONIC Advance 1/2 must be separate trials and ICONIC Lead is excluded</t>
+          <t>Sean confirmed that the platform-study unit is the study report and combined the two ICONIC reports; five reports were not found in the 30 April search</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Complete the 25-record NK screening, finalize report-to-trial mapping and rerun the comparison</t>
+          <t>Complete the 25-record NK screening, clarify when the five missing reports were identified and rerun the comparison</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-10-07 — accuracy meeting</t>
+          <t>Immediate — awaiting review-team clarification</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -46965,7 +47070,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Full-text screening underway; six oversized-PDF exceptions identified</t>
+          <t>Full-text screening underway; extraction setup started; final data-item list pending</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -46985,12 +47090,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Kate distributed all 138 records; six oversized PDFs will be screened without model suggestions</t>
+          <t>Both full-text arms are underway; six PDFs are being screened without model suggestions; Meghan has started extraction setup</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Complete full-text screening and document the six model-suggestion exceptions</t>
+          <t>Complete full-text screening, provide the latest data-item list and finish extraction setup</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -47248,7 +47353,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Full-text screening underway; missing PDFs remain; NK extraction form prepared for review</t>
+          <t>Full-text screening underway; missing PDFs remain; NK extraction form reviewed and revised</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -47268,12 +47373,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Both arms aligned; NK extraction form built from the 22 June template and tested on several articles</t>
+          <t>Jeremy reviewed and revised the extraction form; instructions for running and revising the AI extraction were provided</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Retrieve missing PDFs, complete both full-text arms and review/approve the NK extraction form</t>
+          <t>Retrieve missing PDFs, complete full-text screening and undertake the calibration/AI-extraction exercise</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -47320,7 +47425,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Abstract screening complete; full-text plan under review following reviewer withdrawal and record-set differences</t>
+          <t>Supplemental abstract screening underway following master-file harmonization; full-text baseline pending</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -47340,12 +47445,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Michelle withdrew; Murali remains the sole conventional reviewer under the exception communicated on 1 October; follow-up call requested</t>
+          <t>A 4,173-citation master file produced 2,138 Covidence and 2,028 NK records; 508 Covidence and one NK citation require screening</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Hold the follow-up call, confirm the reviewer arrangement and resolve record-set differences before full-text screening continues</t>
+          <t>Murali to screen 508 records and Mohan one record; then notify Nicholas/Meghan to establish the harmonized full-text set</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -47464,7 +47569,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Onboarding in progress; non-overlapping reviewer groups required and updated searches being arranged</t>
+          <t>Searches received and consolidation underway; Nested Knowledge training scheduled</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -47474,7 +47579,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Laser AI</t>
+          <t>Nested Knowledge</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -47484,17 +47589,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Crossed allocation rejected; both groups must receive the same records; Irma will update Embase from April 2022 onward</t>
+          <t>Embase and ClinicalTrials.gov RIS files received; other searches completed; consolidation/deduplication underway</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Finalize two non-overlapping reviewer groups, complete searches and configure Laser AI</t>
+          <t>Finalize reviewer groups, consolidate and deduplicate searches, attend NK training and configure the project</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>December 2026</t>
+          <t>2026-10-12 — NK training</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -51096,7 +51201,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Complete active reviews and onboard Orthodontic Retention; project-management support confirmed at 20% FTE through mid-December</t>
+          <t>Complete active reviews; Orthodontic search files received and NK training scheduled for 12 October; 20% FTE support continues through mid-December</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -51123,7 +51228,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>BP adjudication complete; time-on-task and downstream-impact analyses underway; automated-analysis meeting to be rescheduled around 20 October; Psoriasis accuracy review scheduled for 7 October</t>
+          <t>BP analysis-support requests sent; Psoriasis reconciliation continues with five report-timing questions; usability and automated-analysis support inquiries sent</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -51177,7 +51282,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Colloquium special session shortlisted; time slot pending; final reporting and project closeout due in December</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -51260,7 +51365,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Current source of truth; review folders were re-shared with Noosheen and full-text PDFs will be added as each adjudication completes</t>
+          <t>Noosheen confirmed access to three NK projects and the Laser AI directory; a fourth NK project is expected Monday; finalized PDFs will follow adjudication</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -51388,7 +51493,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Fruit &amp; Vegetable full-text screening underway; six oversized PDFs will be screened without model suggestions</t>
+          <t>Fruit &amp; Vegetable full-text screening continues; six PDFs lack model suggestions; extraction setup awaits the latest data-item list</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -61285,7 +61390,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Adjudication complete; questions sent to James on 1 October; Doreen connected with Jo-Ana and Max on 4 October</t>
+          <t>Adjudication complete; James’s responses pending; analysis-support and scheduling requests sent on 8 October</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -61302,7 +61407,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Obtain James’s responses, reschedule the automated-analysis meeting around 20 October and continue downstream-impact work</t>
+          <t>Obtain James’s responses, schedule the adjudication-analysis discussion and confirm automated-analysis support</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -61336,7 +61441,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Automated meeting postponed at Paweł’s request; target around 20 October; James’s response remains pending</t>
+          <t>James’s response and analysis scheduling remain pending; automated-analysis target remains around 20 October</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -61392,7 +61497,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -65036,14 +65141,14 @@
       </c>
       <c r="I106" s="18" t="inlineStr">
         <is>
-          <t>Rescheduling</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J106" s="18" t="n"/>
       <c r="K106" s="18" t="n"/>
       <c r="L106" s="18" t="inlineStr">
         <is>
-          <t>Meeting canceled; Paweł requested 15–16 or preferably 20–21 October; plan around 20 October</t>
+          <t>Statistical-support request sent to Paweł and Noosheen; target remains around 20 October</t>
         </is>
       </c>
       <c r="M106" s="18" t="inlineStr">
@@ -65210,7 +65315,7 @@
       <c r="K109" s="18" t="n"/>
       <c r="L109" s="18" t="inlineStr">
         <is>
-          <t>Time-on-task meeting held on 28 September; BP and Psoriasis data received</t>
+          <t>Availability requested from the analysis team for an adjudication-data analysis discussion</t>
         </is>
       </c>
       <c r="M109" s="18" t="inlineStr">
@@ -66614,7 +66719,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Analysis and final reconciliation underway; report-to-trial mapping being clarified</t>
+          <t>Analysis and reconciliation underway; 25-record NK screening and five-report timing clarification pending</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -66682,7 +66787,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Conventional corrective screening complete; 25-record NK screening remains pending; accuracy meeting scheduled</t>
+          <t>Conventional corrective screening complete; 25-record NK screening and final report-level reconciliation remain</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -66699,7 +66804,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Sivem added DOI mapping; ICONIC Advance 1/2 are separate trials and ICONIC Lead is excluded</t>
+          <t>Sean confirmed report-level analysis and combined the two ICONIC reports; five reports require search-timing clarification</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -66716,7 +66821,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete the 25-record NK screening, finalize report-to-trial mapping and rerun the comparison</t>
+          <t>Complete the 25-record NK screening, clarify the five reports and rerun the comparison</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -66733,7 +66838,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-10-07 — accuracy meeting</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -66750,7 +66855,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Analysis active, but final outputs remain dependent on corrective NK screening and reconciliation</t>
+          <t>Final outputs remain blocked by the 25-record screening and five-report clarification</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -66806,7 +66911,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -67053,7 +67158,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Decisions received; 25 NK full texts ready; DOI mapping added; ICONIC Advance 1/2 separate; ICONIC Lead excluded</t>
+          <t>All 139 conventional decisions received; 25 NK full texts ready; Sean combined the ICONIC reports and requested clarification for five reports</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -67311,7 +67416,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Sean is reconciling conventional report IDs with the search set; accuracy meeting scheduled for 7 October</t>
+          <t>Sean confirmed report-level analysis and requested identification timing for five reports absent from the 30 April search</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -70256,7 +70361,7 @@
       <c r="K102" s="18" t="n"/>
       <c r="L102" s="18" t="inlineStr">
         <is>
-          <t>Validation blocked by the 25-record NK screening; conventional report mapping is being reconciled</t>
+          <t>Validation blocked by the 25-record NK screening and five-report timing clarification</t>
         </is>
       </c>
       <c r="M102" s="18" t="inlineStr">
@@ -70313,7 +70418,7 @@
       <c r="K103" s="18" t="n"/>
       <c r="L103" s="18" t="inlineStr">
         <is>
-          <t>Prepare after the NK screening and report-to-trial reconciliation are finalized</t>
+          <t>Prepare after the NK screening and report-level reconciliation are finalized</t>
         </is>
       </c>
       <c r="M103" s="18" t="inlineStr">
@@ -70635,7 +70740,7 @@
       <c r="K109" s="18" t="n"/>
       <c r="L109" s="18" t="inlineStr">
         <is>
-          <t>Time-on-task data received; screening-accuracy discussion scheduled for 7 October</t>
+          <t>Reconciliation continues; review-team clarification is required for five reports</t>
         </is>
       </c>
       <c r="M109" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Refresh dashboard through October 14
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2402,7 +2402,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Full-text screening underway; extraction setup started; final data-item list pending</t>
+          <t>Laser AI full-text screening complete; conventional full-text screening pending</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2470,7 +2470,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Full-text screening underway; Laser AI extraction setup is being prepared</t>
+          <t>Laser AI full-text screening complete; conventional arm not yet complete</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Six PDFs are being screened without model suggestions; Sean requested the latest data-item list</t>
+          <t>Kate completed Laser AI screening; the six oversized PDFs were handled without model suggestions</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete full-text screening, provide the final data items and finish extraction setup</t>
+          <t>Complete the conventional arm, consolidate results and confirm which reports proceed to extraction</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2521,7 +2521,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TBD - after full-text set reconciliation</t>
+          <t>Pending conventional-team completion</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2538,7 +2538,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Screening continues; extraction setup is waiting for the final data-item list</t>
+          <t>AI arm complete; conventional arm pending; fewer than 10 studies may qualify for extraction</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2594,7 +2594,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2875,7 +2875,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Updated extraction form submitted to Sean on 14 October; approval pending</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2919,7 +2919,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Full-text time-on-task data requested; not yet received</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3052,7 +3052,7 @@
         <v>0</v>
       </c>
       <c r="C44" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -3061,7 +3061,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Kate distributed the 138 records; both full-text workflows are underway</t>
+          <t>Laser AI screening complete; Kate has prompted the conventional team to finish</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -3089,7 +3089,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Meghan is setting up extraction in Laser AI; Kate and Bec were asked for the latest data items</t>
+          <t>Updated extraction form submitted; study-selection guidance requested because fewer than 10 studies may qualify</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -4920,7 +4920,7 @@
       <c r="K80" s="18" t="n"/>
       <c r="L80" s="18" t="inlineStr">
         <is>
-          <t>Conventional full-text screening underway; the six oversized records were already screened conventionally</t>
+          <t>Conventional screening remains incomplete; Kate has prompted the team</t>
         </is>
       </c>
       <c r="M80" s="18" t="inlineStr">
@@ -4970,14 +4970,14 @@
       </c>
       <c r="I81" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J81" s="18" t="n"/>
       <c r="K81" s="18" t="n"/>
       <c r="L81" s="18" t="inlineStr">
         <is>
-          <t>Laser AI screening underway; six PDFs will be screened without model suggestions</t>
+          <t>Laser AI full-text screening complete; six oversized PDFs were screened without model suggestions</t>
         </is>
       </c>
       <c r="M81" s="18" t="inlineStr">
@@ -5133,12 +5133,16 @@
       </c>
       <c r="I84" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J84" s="18" t="n"/>
       <c r="K84" s="18" t="n"/>
-      <c r="L84" s="18" t="n"/>
+      <c r="L84" s="18" t="inlineStr">
+        <is>
+          <t>Full-text usability survey sent to Kate on 13 October</t>
+        </is>
+      </c>
       <c r="M84" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -5186,12 +5190,16 @@
       </c>
       <c r="I85" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J85" s="18" t="n"/>
       <c r="K85" s="18" t="n"/>
-      <c r="L85" s="18" t="n"/>
+      <c r="L85" s="18" t="inlineStr">
+        <is>
+          <t>Kate indicated that she would complete the survey</t>
+        </is>
+      </c>
       <c r="M85" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -5504,14 +5512,14 @@
       </c>
       <c r="I91" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J91" s="18" t="n"/>
       <c r="K91" s="18" t="n"/>
       <c r="L91" s="18" t="inlineStr">
         <is>
-          <t>Latest extraction items requested from Kate and Bec</t>
+          <t>Updated extraction form sent to Sean on 14 October</t>
         </is>
       </c>
       <c r="M91" s="18" t="inlineStr">
@@ -5561,12 +5569,16 @@
       </c>
       <c r="I92" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="J92" s="18" t="n"/>
       <c r="K92" s="18" t="n"/>
-      <c r="L92" s="18" t="n"/>
+      <c r="L92" s="18" t="inlineStr">
+        <is>
+          <t>Sean's final approval and extraction-study selection guidance are pending</t>
+        </is>
+      </c>
       <c r="M92" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -23202,7 +23214,7 @@
       </c>
       <c r="D35" s="17" t="inlineStr">
         <is>
-          <t>Converted to phase1-09; searches received, consolidation underway and NK training scheduled</t>
+          <t>Converted to phase1-09; NK training complete and five RIS files received</t>
         </is>
       </c>
       <c r="E35" s="17" t="inlineStr">
@@ -23217,12 +23229,12 @@
       </c>
       <c r="G35" s="17" t="inlineStr">
         <is>
-          <t>Consolidate/deduplicate the search files; NK training scheduled for 12 October</t>
+          <t>RIS import, deduplication and workflow configuration pending</t>
         </is>
       </c>
       <c r="H35" s="17" t="inlineStr">
         <is>
-          <t>Embase and ClinicalTrials.gov RIS files received; other searches completed; final groups and deduplicated RIS pending</t>
+          <t>Conchita and Álvaro completed NK training; Nest created; conventional-screening access remains unresolved</t>
         </is>
       </c>
       <c r="I35" s="17" t="inlineStr">
@@ -26926,7 +26938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="14" customWidth="1" style="29" min="1" max="2"/>
@@ -27631,27 +27643,27 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>11:00 AM–12:00 PM EDT</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>4:00–5:00 PM BST</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Nested Knowledge Training – Orthodontic Retention</t>
+          <t>Orthodontic NK training</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>NK training and initial project-setup guidance; 10:00–11:00 AM Central / 5:00–6:00 PM Madrid</t>
+          <t>Nested Knowledge training for Orthodontic Retention</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Ranita Tarchand / Orthodontic review team / Krishna</t>
+          <t>Conchita / Álvaro / Krishna / Nested Knowledge</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -27666,15 +27678,186 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>phase1-09</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>mtg-13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>10:00–11:00 AM CT</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>CESAR Adjudication Data Analysis</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Review data and statistical-analysis requirements</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Gerald / Afroditi / Sean / Andreea / Krishna</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Project coordination</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
           <t>Scheduled</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>phase1-09</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>mtg-14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>9:00–10:00 AM CT</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>CESAR Usability Survey Analysis</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Review usability-analysis status</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Gerald / Ursula / Susan / Afroditi / Krishna</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Project coordination</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>mtg-15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>11:00 AM–12:00 PM CT</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>CESAR Automated Analysis</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Confirm automated-analysis status and requirements</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Paweł / Noosheen / Gerald / Afroditi / Sean / Krishna</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Project coordination</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -27930,7 +28113,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Jeremy reviewed the form, made minor revisions and received instructions for running and revising the AI output</t>
+          <t>Jeremy reviewed the form, made minor revisions and requested instructions for running/reviewing AI extraction</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -27947,7 +28130,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Retrieve missing PDFs, complete full-text screening and undertake calibration/AI extraction</t>
+          <t>Confirm the screening timeline, retrieve missing PDFs, complete both full-text arms and finalize extraction instructions</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -27981,7 +28164,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Both arms remain active; extraction can be calibrated while missing PDFs are retrieved</t>
+          <t>Both arms remain active; Bradley will confirm the screening timeline; missing PDFs remain</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -28037,7 +28220,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -28498,7 +28681,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Jeremy reviewed and revised the form; AI-extraction instructions were provided</t>
+          <t>Jeremy reviewed and revised the form; final instructions and approval remain pending</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -30896,7 +31079,7 @@
       <c r="K91" s="18" t="n"/>
       <c r="L91" s="18" t="inlineStr">
         <is>
-          <t>Jeremy reviewed and revised the form; calibration may identify further adjustments</t>
+          <t>Jeremy reviewed the form and added minor revisions/details</t>
         </is>
       </c>
       <c r="M91" s="18" t="inlineStr">
@@ -30953,7 +31136,7 @@
       <c r="K92" s="18" t="n"/>
       <c r="L92" s="18" t="inlineStr">
         <is>
-          <t>Review-team revisions completed; final Sean approval remains pending</t>
+          <t>Review completed; final approval and NK extraction instructions remain pending</t>
         </is>
       </c>
       <c r="M92" s="18" t="inlineStr">
@@ -32544,7 +32727,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Supplemental abstract screening underway after master-file harmonization; full-text baseline pending</t>
+          <t>Conventional full-text screening complete; NK full-text screening awaits PDFs</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -32612,7 +32795,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Master file created with 4,173 citations; 508 Covidence and one NK citation require screening</t>
+          <t>Conventional full-text screening complete; NK shows 74 records advanced</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -32629,7 +32812,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Covidence deduplicated the master file to 2,138 records and NK to 2,028; the earlier 77-record set is no longer final</t>
+          <t>Murali completed conventional screening and uploaded PDFs to Covidence; Mohan is waiting for NK PDFs</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -32646,7 +32829,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete the supplemental screening and establish a harmonized full-text baseline</t>
+          <t>Confirm the shared-drive PDF upload, load PDFs into NK and begin AI-assisted full-text screening</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -32680,7 +32863,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Platform-specific deduplication produced different sets; full-text screening is blocked pending harmonization</t>
+          <t>Conventional arm complete; AI arm has 74 records and is blocked pending PDF availability</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -32736,7 +32919,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -32973,7 +33156,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Final full-text/PDF set pending supplemental screening and harmonization</t>
+          <t>Murali uploaded full texts to Covidence; shared-drive and NK PDF availability remain to be confirmed</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -33180,7 +33363,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -33190,7 +33373,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Nicholas/Meghan will establish the harmonized full-text baseline after supplemental screening</t>
+          <t>Conventional full-text screening complete; NK full-text screening is waiting for PDFs</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -35047,14 +35230,14 @@
       </c>
       <c r="I80" s="18" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J80" s="18" t="n"/>
       <c r="K80" s="18" t="n"/>
       <c r="L80" s="18" t="inlineStr">
         <is>
-          <t>Conventional full-text screening waits for the harmonized baseline</t>
+          <t>Murali completed conventional full-text screening</t>
         </is>
       </c>
       <c r="M80" s="18" t="inlineStr">
@@ -35104,14 +35287,14 @@
       </c>
       <c r="I81" s="18" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J81" s="18" t="n"/>
       <c r="K81" s="18" t="n"/>
       <c r="L81" s="18" t="inlineStr">
         <is>
-          <t>NK full-text screening waits for the harmonized baseline</t>
+          <t>NK shows 74 records advanced; Mohan is waiting for the full texts</t>
         </is>
       </c>
       <c r="M81" s="18" t="inlineStr">
@@ -36931,7 +37114,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Murali screens 508 records and Mohan one record; notify Nicholas and Meghan when complete</t>
+          <t>Conventional screening complete; confirm PDF handoff and begin the 74-record NK full-text stage</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -37044,12 +37227,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Human Milk master-file recalibration</t>
+          <t>Human Milk conventional full-text screening completed</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -37074,7 +37257,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Master file contains 4,173 citations; Covidence requires 508 additional decisions and NK requires one</t>
+          <t>Murali completed screening; Mohan is waiting for PDFs for the 74 NK records</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -37084,7 +37267,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>Complete supplemental screening and establish the harmonized full-text set</t>
+          <t>Confirm shared-drive/NK PDF upload and start AI-assisted full-text screening</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -37130,7 +37313,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Complete supplemental abstract screening and harmonize the full-text baseline</t>
+          <t>Complete PDF handoff and begin NK full-text screening</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -37155,7 +37338,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Full-text screening cannot proceed until the 508 Covidence and one NK citation are screened and compared</t>
+          <t>Conventional screening complete; AI screening cannot start until PDFs are available in NK</t>
         </is>
       </c>
     </row>
@@ -42118,7 +42301,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Search files received and consolidation underway; NK training scheduled for 12 October</t>
+          <t>NK training complete; Nest created; five RIS files received; setup guidance pending</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -42186,7 +42369,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Embase and ClinicalTrials.gov RIS files received; other database searches completed; consolidation/deduplication underway</t>
+          <t>Five search files received; NK import/deduplication and workflow configuration pending</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -42203,7 +42386,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Crossed allocation rejected and protocol accepted; Irma supplied the updated search files</t>
+          <t>Conchita and Álvaro completed NK training; Conchita will perform screening; conventional-platform access remains unresolved</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -42220,7 +42403,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Finalize the two groups, consolidate/deduplicate the searches, attend NK training and configure the project</t>
+          <t>Import and deduplicate the RIS files, finalize reviewer groups and NK settings, and resolve conventional screening access</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -42254,7 +42437,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Search files received and training scheduled; reviewer-group names and final deduplicated RIS remain pending</t>
+          <t>Training and searches received; reviewer allocation, NK settings and conventional workflow remain pending</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -42271,7 +42454,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Onboarding</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -42310,7 +42493,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -42375,7 +42558,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -42385,7 +42568,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Reviewer-allocation method resolved; search consolidation and training underway</t>
+          <t>Initial onboarding and NK introductory training completed</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -42402,7 +42585,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -42412,7 +42595,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Nested Knowledge selected; training scheduled and final RIS pending</t>
+          <t>Nest created; RIS import and workflow configuration pending</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -42530,12 +42713,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Embase and ClinicalTrials.gov RIS files received; remaining searches completed; consolidation underway</t>
+          <t>Five RIS files received: ICTRP, MEDLINE, ClinicalTrials.gov, Embase and CENTRAL</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -42584,7 +42767,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Pending reviewer allocation</t>
+          <t>PICO-based eligibility prompts awaiting configuration guidance</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -42731,7 +42914,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Onboarding</t>
+          <t>Setup In Progress</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -42741,7 +42924,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Reviewer model resolved; searches received; NK training scheduled for 12 October</t>
+          <t>NK training complete and Nest created; import/settings work remains</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -43269,12 +43452,16 @@
       </c>
       <c r="I55" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J55" s="18" t="n"/>
       <c r="K55" s="18" t="n"/>
-      <c r="L55" s="18" t="inlineStr"/>
+      <c r="L55" s="18" t="inlineStr">
+        <is>
+          <t>NK access confirmed; team created its Nest</t>
+        </is>
+      </c>
       <c r="M55" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -43428,14 +43615,14 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J58" s="18" t="n"/>
       <c r="K58" s="18" t="n"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>Updated Embase and ClinicalTrials.gov RIS files received; consolidated RIS remains pending</t>
+          <t>Five completed-search RIS files received on 12 October</t>
         </is>
       </c>
       <c r="M58" s="18" t="inlineStr">
@@ -43698,14 +43885,14 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J63" s="18" t="n"/>
       <c r="K63" s="18" t="n"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>NK training scheduled; setup awaits the consolidated RIS and reviewer groups</t>
+          <t>Nest created; RIS import, deduplication and workflow settings pending</t>
         </is>
       </c>
       <c r="M63" s="18" t="inlineStr">
@@ -46369,7 +46556,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Crossed allocation rejected; searches received; NK training scheduled for 12 October</t>
+          <t>NK training complete; reviewer allocation and conventional-platform arrangement remain pending</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -46479,12 +46666,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Orthodontic searches received and NK training scheduled</t>
+          <t>Orthodontic NK training and search-file handoff completed</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -46509,7 +46696,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Embase/ClinicalTrials.gov files received; consolidation underway; NK training scheduled for 12 October</t>
+          <t>Conchita and Álvaro completed training; five RIS files received; setup questions sent</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -46619,7 +46806,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Separate reviewer groups and updated searches required before setup</t>
+          <t>Finalize reviewer groups, NK settings and conventional screening access</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -46649,12 +46836,12 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>Finalize two separate groups, complete the database searches and share the resulting RIS files</t>
+          <t>Import the five RIS files, finalize groups/settings and resolve Covidence or alternative manual-screening access</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>Laser AI setup cannot proceed until the team split and complete search set are available</t>
+          <t>NK setup can proceed, but parallel conventional screening access remains unresolved</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -46946,17 +47133,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Adjudication complete; James’s responses remain pending; downstream-impact work continues and analysis-support requests were sent</t>
+          <t>Questions sent directly to James on 14 October; automated-analysis meeting scheduled for 21 October; downstream-impact work awaits BP RevMan/meta-analysis progress</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Obtain James’s responses, schedule the adjudication-analysis discussion and confirm automated-analysis statistical support</t>
+          <t>Obtain James's responses; hold the 21 October automated-analysis meeting; reconnect with Doreen when RevMan analysis begins</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
         <is>
-          <t>December 2026</t>
+          <t>2026-10-21 — automated-analysis meeting</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -47018,7 +47205,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Sean confirmed that the platform-study unit is the study report and combined the two ICONIC reports; five reports were not found in the 30 April search</t>
+          <t>Sivem clarified source records for CLEAR-1, Khan, STRIDE, VESPUCCI and Zhang; final mapping and 25-record NK screening remain pending</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -47028,7 +47215,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Immediate — awaiting review-team clarification</t>
+          <t>TBD — after corrective NK screening and reconciliation</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -47070,7 +47257,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Full-text screening underway; extraction setup started; final data-item list pending</t>
+          <t>Laser AI full-text screening complete; conventional full-text screening pending</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -47090,17 +47277,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Both full-text arms are underway; six PDFs are being screened without model suggestions; Meghan has started extraction setup</t>
+          <t>Kate completed Laser AI full-text screening; survey sent; updated extraction form submitted to Sean</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Complete full-text screening, provide the latest data-item list and finish extraction setup</t>
+          <t>Complete conventional full-text screening, consolidate both arms and obtain Sean's extraction-form/selection guidance</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>TBD - after full-text set reconciliation</t>
+          <t>Pending conventional full-text completion</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -47373,17 +47560,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Jeremy reviewed and revised the extraction form; instructions for running and revising the AI extraction were provided</t>
+          <t>Jeremy reviewed and revised the NK extraction form; Bradley will confirm the full-text screening timeline</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Retrieve missing PDFs, complete full-text screening and undertake the calibration/AI-extraction exercise</t>
+          <t>Confirm the screening timeline, retrieve missing PDFs, complete both arms and obtain final form approval</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Awaiting review-team timeline</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -47425,7 +47612,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Supplemental abstract screening underway following master-file harmonization; full-text baseline pending</t>
+          <t>Conventional full-text screening complete; 74 records advanced in NK; AI full-text screening awaits PDFs</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -47445,12 +47632,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>A 4,173-citation master file produced 2,138 Covidence and 2,028 NK records; 508 Covidence and one NK citation require screening</t>
+          <t>Murali completed conventional full-text screening and uploaded PDFs to Covidence; Mohan is waiting for the PDFs for 74 NK records</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Murali to screen 508 records and Mohan one record; then notify Nicholas/Meghan to establish the harmonized full-text set</t>
+          <t>Confirm the shared-drive PDF upload, add PDFs to NK and begin AI-assisted full-text screening</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -47569,7 +47756,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Searches received and consolidation underway; Nested Knowledge training scheduled</t>
+          <t>NK training complete; Nest created; five RIS search files received; setup guidance pending</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -47589,12 +47776,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Embase and ClinicalTrials.gov RIS files received; other searches completed; consolidation/deduplication underway</t>
+          <t>Conchita and Álvaro completed NK training; five RIS files were supplied; Covidence access and workflow settings require confirmation</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Finalize reviewer groups, consolidate and deduplicate searches, attend NK training and configure the project</t>
+          <t>Import and deduplicate the five RIS files, finalize reviewer groups and NK settings, and resolve conventional-platform access</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -51098,7 +51285,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="18" customWidth="1" style="29" min="1" max="1"/>
@@ -51201,7 +51388,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Complete active reviews; Orthodontic search files received and NK training scheduled for 12 October; 20% FTE support continues through mid-December</t>
+          <t>Complete active reviews; Orthodontic NK training is complete and setup is underway; project-management support continues through mid-December</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -51228,7 +51415,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>BP analysis-support requests sent; Psoriasis reconciliation continues with five report-timing questions; usability and automated-analysis support inquiries sent</t>
+          <t>BP adjudication complete; time-on-task clarified; analysis meetings scheduled for 14, 15 and 21 October; downstream-impact work awaits BP RevMan/meta-analysis progress</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -51493,7 +51680,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Fruit &amp; Vegetable full-text screening continues; six PDFs lack model suggestions; extraction setup awaits the latest data-item list</t>
+          <t>Laser AI full-text screening complete; conventional screening remains; six PDFs were screened without model suggestions</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -51735,6 +51922,132 @@
         </is>
       </c>
       <c r="H28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>meet-012</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>CESAR – Adjudication Data Analysis</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Gerald / Afroditi / Sean / Andreea / Krishna</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Review data and statistical-analysis requirements</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>10:00–11:00 AM CT</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>meet-013</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>CESAR – Usability Survey Analysis</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Gerald / Ursula / Susan / Afroditi / Krishna</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Review usability-analysis status</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>9:00–10:00 AM CT</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>meet-014</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>CESAR – Automated Analysis</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Paweł / Noosheen / Gerald / Afroditi / Sean / Krishna</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Confirm automated-analysis status and requirements</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>11:00 AM–12:00 PM CT</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -61390,7 +61703,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Adjudication complete; James’s responses pending; analysis-support and scheduling requests sent on 8 October</t>
+          <t>Questions sent directly to James on 14 October; automated-analysis meeting scheduled for 21 October</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -61407,7 +61720,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Obtain James’s responses, schedule the adjudication-analysis discussion and confirm automated-analysis support</t>
+          <t>Obtain James's responses, hold the 21 October meeting and reconnect with Doreen after RevMan analysis begins</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -61441,7 +61754,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>James’s response and analysis scheduling remain pending; automated-analysis target remains around 20 October</t>
+          <t>Automated meeting scheduled for 21 October; James's response remains pending; BP meta-analysis has not started</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -61497,7 +61810,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -61832,7 +62145,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Time reports received; time-on-task analysis underway</t>
+          <t>2,459 minutes cover extraction of 31 primary studies/associated reports; RevMan conversion and entry time were excluded</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -65141,14 +65454,14 @@
       </c>
       <c r="I106" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Scheduled</t>
         </is>
       </c>
       <c r="J106" s="18" t="n"/>
       <c r="K106" s="18" t="n"/>
       <c r="L106" s="18" t="inlineStr">
         <is>
-          <t>Statistical-support request sent to Paweł and Noosheen; target remains around 20 October</t>
+          <t>Automated-analysis meeting scheduled for 21 October, 11:00 AM–12:00 PM CT</t>
         </is>
       </c>
       <c r="M106" s="18" t="inlineStr">
@@ -65315,7 +65628,7 @@
       <c r="K109" s="18" t="n"/>
       <c r="L109" s="18" t="inlineStr">
         <is>
-          <t>Availability requested from the analysis team for an adjudication-data analysis discussion</t>
+          <t>Doreen clarified that 2,459 minutes cover extraction only across 31 reports; RevMan work was excluded</t>
         </is>
       </c>
       <c r="M109" s="18" t="inlineStr">
@@ -65365,14 +65678,14 @@
       </c>
       <c r="I110" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Waiting on Review Team</t>
         </is>
       </c>
       <c r="J110" s="18" t="n"/>
       <c r="K110" s="18" t="n"/>
       <c r="L110" s="18" t="inlineStr">
         <is>
-          <t>Downstream work started; Doreen was connected with Jo-Ana and Max on 4 October to discuss meta-analysis status and plans</t>
+          <t>BP team is finalizing included/ongoing/awaiting-classification lists and risk-of-bias assessments; RevMan entry and meta-analysis have not started</t>
         </is>
       </c>
       <c r="M110" s="18" t="inlineStr">
@@ -66804,7 +67117,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Sean confirmed report-level analysis and combined the two ICONIC reports; five reports require search-timing clarification</t>
+          <t>Sivem additionally clarified the source records for CLEAR-1, Khan, STRIDE, VESPUCCI and Zhang</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -66838,7 +67151,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Immediate</t>
+          <t>TBD — after corrective screening and reconciliation</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -66911,7 +67224,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -67416,7 +67729,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Sean confirmed report-level analysis and requested identification timing for five reports absent from the 30 April search</t>
+          <t>Sean is reconciling report-to-trial mapping using Sivem's additional source-record clarifications</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -70361,7 +70674,7 @@
       <c r="K102" s="18" t="n"/>
       <c r="L102" s="18" t="inlineStr">
         <is>
-          <t>Validation blocked by the 25-record NK screening and five-report timing clarification</t>
+          <t>Validation remains blocked by the 25-record NK screening and final report-to-trial mapping</t>
         </is>
       </c>
       <c r="M102" s="18" t="inlineStr">

</xml_diff>